<commit_message>
Convert match times to CDMX in template
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_Final_vacia.xlsx
+++ b/Quiniela_Mundial_2026_Final_vacia.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-3840" yWindow="-19785" windowWidth="28800" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,12 +81,6 @@
     <font>
       <name val="Arial"/>
       <family val="2"/>
-      <color rgb="FF31333F"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
       <i val="1"/>
       <color rgb="FF31333F"/>
       <sz val="12"/>
@@ -121,32 +115,39 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Segoe UI"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="000F4C43"/>
+      <color rgb="FF0F4C43"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00333333"/>
+      <family val="2"/>
+      <color rgb="FF333333"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -179,32 +180,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F4C43"/>
-        <bgColor rgb="000F4C43"/>
+        <fgColor rgb="FF0F4C43"/>
+        <bgColor rgb="FF0F4C43"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D4EDDA"/>
-        <bgColor rgb="00D4EDDA"/>
+        <fgColor rgb="FFD4EDDA"/>
+        <bgColor rgb="FFD4EDDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7FAF9"/>
-        <bgColor rgb="00F7FAF9"/>
+        <fgColor rgb="FFF7FAF9"/>
+        <bgColor rgb="FFF7FAF9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
-        <bgColor rgb="00F8D7DA"/>
+        <fgColor rgb="FFF8D7DA"/>
+        <bgColor rgb="FFF8D7DA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEEEEE"/>
-        <bgColor rgb="00EEEEEE"/>
+        <fgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFEEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -255,38 +262,40 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -312,91 +321,170 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="12">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00D4EDDA"/>
-          <bgColor rgb="00D4EDDA"/>
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD4EDDA"/>
+          <bgColor rgb="FFD4EDDA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -763,89 +851,96 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G44"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="148" customWidth="1" style="16" min="1" max="1"/>
-    <col width="75.42578125" customWidth="1" style="16" min="7" max="7"/>
+    <col width="148" customWidth="1" style="28" min="1" max="1"/>
+    <col width="75.42578125" customWidth="1" style="28" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.75" customHeight="1" s="16">
-      <c r="A1" s="18" t="inlineStr">
+    <row r="1" ht="33.75" customHeight="1" s="28">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>QUINIELA MUNDIAL DE FÚTBOL 2026 - 100% AUTOMATIZADA</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="16">
+    <row r="3" ht="16.5" customHeight="1" s="28">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>La Copa Mundial de la FIFA 26™ tendrá 48 equipos divididos en doce grupos con cuatro equipos cada uno.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="16">
+    <row r="4" ht="16.5" customHeight="1" s="28">
       <c r="A4" s="1" t="n"/>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="16">
+    <row r="5" ht="16.5" customHeight="1" s="28">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Los dos primeros de cada grupo y los ocho mejores terceros avanzarán a los dieciseisavos de final.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="16">
+    <row r="6" ht="16.5" customHeight="1" s="28">
       <c r="A6" s="1" t="n"/>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="16">
+    <row r="7" ht="16.5" customHeight="1" s="28">
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Los equipos que lleguen a la final del 19 de julio habrán disputado ocho partidos, uno más que en Catar 2022.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="16">
+    <row r="8" ht="16.5" customHeight="1" s="28">
       <c r="A8" s="1" t="n"/>
     </row>
-    <row r="9" ht="33" customHeight="1" s="16">
-      <c r="A9" s="20" t="inlineStr">
+    <row r="9" ht="33" customHeight="1" s="28">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>El nuevo esquema establece que los equipos que lleguen a la final, a jugarse el domingo 19 de julio, tendrán que haber atravesado ocho partidos, uno más de los disputados en la última Copa Mundial de la FIFA 2022™, en Catar.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="16">
+    <row r="10" ht="16.5" customHeight="1" s="28">
       <c r="A10" s="1" t="n"/>
     </row>
-    <row r="11" ht="26.25" customHeight="1" s="16">
-      <c r="A11" s="18" t="inlineStr">
+    <row r="11" ht="26.25" customHeight="1" s="28">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>CÓMO FUNCIONA:</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="16">
+    <row r="13" ht="16.5" customHeight="1" s="28">
       <c r="A13" s="1" t="inlineStr">
         <is>
           <t>1. Pestaña 'Grupos': Ingresa los resultados. Las tablas se calculan en tiempo real.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="16">
+    <row r="14" ht="16.5" customHeight="1" s="28">
       <c r="A14" s="1" t="inlineStr">
         <is>
           <t>2. Pestaña 'Eliminatorias': Al ir llenando, verás cómo los nombres se auto-completan gracias a la corrección del motor.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="16">
+    <row r="15" ht="16.5" customHeight="1" s="28">
       <c r="A15" s="1" t="inlineStr">
         <is>
           <t>3. Puedes empezar a llenar y los líderes de cada grupo aparecerán de inmediato.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="26.25" customHeight="1" s="16">
-      <c r="A17" s="18" t="inlineStr">
+    <row r="16" ht="16.5" customHeight="1" s="28">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>4. Guarda tu quiniela con tu nombre y apellido. Ejemplo: Quiniela_Cristiano_Ronaldo.xlsx, Quiniela_Lionel_Messi.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26.25" customHeight="1" s="28">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Sistema de Puntuación</t>
         </is>
@@ -854,8 +949,8 @@
     <row r="18">
       <c r="A18" s="7" t="n"/>
     </row>
-    <row r="19" ht="15.75" customHeight="1" s="16">
-      <c r="A19" s="21" t="inlineStr">
+    <row r="19" ht="15.75" customHeight="1" s="28">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Fase de Grupos:</t>
         </is>
@@ -878,8 +973,8 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="16">
-      <c r="A24" s="21" t="inlineStr">
+    <row r="24" ht="15.75" customHeight="1" s="28">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Fase Eliminatoria:</t>
         </is>
@@ -944,8 +1039,8 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1" s="16">
-      <c r="A35" s="21" t="inlineStr">
+    <row r="35" ht="15.75" customHeight="1" s="28">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Podio (Predicciones Finales):</t>
         </is>
@@ -1012,7 +1107,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H212"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8242,64 +8337,64 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:T99"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="16" min="1" max="1"/>
-    <col width="16" customWidth="1" style="16" min="3" max="3"/>
-    <col width="16" customWidth="1" style="16" min="7" max="7"/>
-    <col width="16" customWidth="1" style="16" min="11" max="11"/>
+    <col width="8" customWidth="1" style="28" min="1" max="1"/>
+    <col width="16" customWidth="1" style="28" min="3" max="3"/>
+    <col width="16" customWidth="1" style="28" min="7" max="7"/>
+    <col width="16" customWidth="1" style="28" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>PARTIDOS DE GRUPOS</t>
         </is>
       </c>
-      <c r="J1" s="26" t="inlineStr">
+      <c r="J1" s="27" t="inlineStr">
         <is>
           <t>TABLAS DE POSICIONES (AUTOMÁTICAS)</t>
         </is>
       </c>
     </row>
     <row r="2"/>
-    <row r="4" ht="16.5" customHeight="1" s="16">
-      <c r="A4" s="14" t="inlineStr">
+    <row r="4" ht="16.5" customHeight="1" s="28">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Equipo 1</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="G4" s="14" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Equipo 2</t>
         </is>
       </c>
-      <c r="H4" s="14" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -8360,13 +8455,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18.75" customHeight="1" s="16">
-      <c r="A5" s="27" t="inlineStr">
+    <row r="5" ht="18.75" customHeight="1" s="28">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>GRUPO A</t>
         </is>
       </c>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO A</t>
         </is>
@@ -8671,7 +8766,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="18.75" customHeight="1" s="16">
+    <row r="11" ht="18.75" customHeight="1" s="28">
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Sudáfrica</t>
@@ -8693,7 +8788,7 @@
         <f>IF(AND(ISNUMBER(D11),ISNUMBER(F11)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J11" s="27" t="inlineStr">
+      <c r="J11" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO B</t>
         </is>
@@ -8747,8 +8842,8 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="18.75" customHeight="1" s="16">
-      <c r="A13" s="27" t="inlineStr">
+    <row r="13" ht="18.75" customHeight="1" s="28">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>GRUPO B</t>
         </is>
@@ -8961,7 +9056,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="18.75" customHeight="1" s="16">
+    <row r="17" ht="18.75" customHeight="1" s="28">
       <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Bosnia y Herze.</t>
@@ -8983,7 +9078,7 @@
         <f>IF(AND(ISNUMBER(D17),ISNUMBER(F17)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J17" s="27" t="inlineStr">
+      <c r="J17" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO C</t>
         </is>
@@ -9175,8 +9270,8 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="18.75" customHeight="1" s="16">
-      <c r="A21" s="27" t="inlineStr">
+    <row r="21" ht="18.75" customHeight="1" s="28">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>GRUPO C</t>
         </is>
@@ -9251,7 +9346,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="18.75" customHeight="1" s="16">
+    <row r="23" ht="18.75" customHeight="1" s="28">
       <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Haití</t>
@@ -9273,7 +9368,7 @@
         <f>IF(AND(ISNUMBER(D23),ISNUMBER(F23)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J23" s="27" t="inlineStr">
+      <c r="J23" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO D</t>
         </is>
@@ -9555,13 +9650,13 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="18.75" customHeight="1" s="16">
-      <c r="A29" s="27" t="inlineStr">
+    <row r="29" ht="18.75" customHeight="1" s="28">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>GRUPO D</t>
         </is>
       </c>
-      <c r="J29" s="27" t="inlineStr">
+      <c r="J29" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO E</t>
         </is>
@@ -9866,7 +9961,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="18.75" customHeight="1" s="16">
+    <row r="35" ht="18.75" customHeight="1" s="28">
       <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Paraguay</t>
@@ -9888,7 +9983,7 @@
         <f>IF(AND(ISNUMBER(D35),ISNUMBER(F35)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J35" s="27" t="inlineStr">
+      <c r="J35" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO F</t>
         </is>
@@ -9942,8 +10037,8 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="18.75" customHeight="1" s="16">
-      <c r="A37" s="27" t="inlineStr">
+    <row r="37" ht="18.75" customHeight="1" s="28">
+      <c r="A37" s="29" t="inlineStr">
         <is>
           <t>GRUPO E</t>
         </is>
@@ -10156,7 +10251,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="18.75" customHeight="1" s="16">
+    <row r="41" ht="18.75" customHeight="1" s="28">
       <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Curaçao</t>
@@ -10178,7 +10273,7 @@
         <f>IF(AND(ISNUMBER(D41),ISNUMBER(F41)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J41" s="27" t="inlineStr">
+      <c r="J41" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO G</t>
         </is>
@@ -10370,8 +10465,8 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="18.75" customHeight="1" s="16">
-      <c r="A45" s="27" t="inlineStr">
+    <row r="45" ht="18.75" customHeight="1" s="28">
+      <c r="A45" s="29" t="inlineStr">
         <is>
           <t>GRUPO F</t>
         </is>
@@ -10446,7 +10541,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="18.75" customHeight="1" s="16">
+    <row r="47" ht="18.75" customHeight="1" s="28">
       <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Suecia</t>
@@ -10468,7 +10563,7 @@
         <f>IF(AND(ISNUMBER(D47),ISNUMBER(F47)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J47" s="27" t="inlineStr">
+      <c r="J47" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO H</t>
         </is>
@@ -10750,13 +10845,13 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="18.75" customHeight="1" s="16">
-      <c r="A53" s="27" t="inlineStr">
+    <row r="53" ht="18.75" customHeight="1" s="28">
+      <c r="A53" s="29" t="inlineStr">
         <is>
           <t>GRUPO G</t>
         </is>
       </c>
-      <c r="J53" s="27" t="inlineStr">
+      <c r="J53" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO I</t>
         </is>
@@ -11061,7 +11156,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" ht="18.75" customHeight="1" s="16">
+    <row r="59" ht="18.75" customHeight="1" s="28">
       <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Egipto</t>
@@ -11083,7 +11178,7 @@
         <f>IF(AND(ISNUMBER(D59),ISNUMBER(F59)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J59" s="27" t="inlineStr">
+      <c r="J59" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO J</t>
         </is>
@@ -11137,8 +11232,8 @@
         <v/>
       </c>
     </row>
-    <row r="61" ht="18.75" customHeight="1" s="16">
-      <c r="A61" s="27" t="inlineStr">
+    <row r="61" ht="18.75" customHeight="1" s="28">
+      <c r="A61" s="29" t="inlineStr">
         <is>
           <t>GRUPO H</t>
         </is>
@@ -11351,7 +11446,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" ht="18.75" customHeight="1" s="16">
+    <row r="65" ht="18.75" customHeight="1" s="28">
       <c r="C65" s="4" t="inlineStr">
         <is>
           <t>Cabo Verde</t>
@@ -11373,7 +11468,7 @@
         <f>IF(AND(ISNUMBER(D65),ISNUMBER(F65)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J65" s="27" t="inlineStr">
+      <c r="J65" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO K</t>
         </is>
@@ -11565,8 +11660,8 @@
         <v/>
       </c>
     </row>
-    <row r="69" ht="18.75" customHeight="1" s="16">
-      <c r="A69" s="27" t="inlineStr">
+    <row r="69" ht="18.75" customHeight="1" s="28">
+      <c r="A69" s="29" t="inlineStr">
         <is>
           <t>GRUPO I</t>
         </is>
@@ -11641,7 +11736,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" ht="18.75" customHeight="1" s="16">
+    <row r="71" ht="18.75" customHeight="1" s="28">
       <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Irak</t>
@@ -11663,7 +11758,7 @@
         <f>IF(AND(ISNUMBER(D71),ISNUMBER(F71)),"Ok","")</f>
         <v/>
       </c>
-      <c r="J71" s="27" t="inlineStr">
+      <c r="J71" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO L</t>
         </is>
@@ -11945,8 +12040,8 @@
         <v/>
       </c>
     </row>
-    <row r="77" ht="18.75" customHeight="1" s="16">
-      <c r="A77" s="27" t="inlineStr">
+    <row r="77" ht="18.75" customHeight="1" s="28">
+      <c r="A77" s="29" t="inlineStr">
         <is>
           <t>GRUPO J</t>
         </is>
@@ -12090,8 +12185,8 @@
         <v/>
       </c>
     </row>
-    <row r="85" ht="18.75" customHeight="1" s="16">
-      <c r="A85" s="27" t="inlineStr">
+    <row r="85" ht="18.75" customHeight="1" s="28">
+      <c r="A85" s="29" t="inlineStr">
         <is>
           <t>GRUPO K</t>
         </is>
@@ -12235,8 +12330,8 @@
         <v/>
       </c>
     </row>
-    <row r="93" ht="18.75" customHeight="1" s="16">
-      <c r="A93" s="27" t="inlineStr">
+    <row r="93" ht="18.75" customHeight="1" s="28">
+      <c r="A93" s="29" t="inlineStr">
         <is>
           <t>GRUPO L</t>
         </is>
@@ -12409,66 +12504,6 @@
     <mergeCell ref="J71:T71"/>
     <mergeCell ref="A93:H93"/>
   </mergeCells>
-  <conditionalFormatting sqref="J6:S9">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T6&gt;=LARGE($T$6:$T$9,2), AND($T6=LARGE($T$6:$T$9,3), $T6&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J12:S15">
-    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T12&gt;=LARGE($T$12:$T$15,2), AND($T12=LARGE($T$12:$T$15,3), $T12&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J18:S21">
-    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T18&gt;=LARGE($T$18:$T$21,2), AND($T18=LARGE($T$18:$T$21,3), $T18&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J24:S27">
-    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T24&gt;=LARGE($T$24:$T$27,2), AND($T24=LARGE($T$24:$T$27,3), $T24&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J30:S33">
-    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T30&gt;=LARGE($T$30:$T$33,2), AND($T30=LARGE($T$30:$T$33,3), $T30&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J36:S39">
-    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T36&gt;=LARGE($T$36:$T$39,2), AND($T36=LARGE($T$36:$T$39,3), $T36&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J42:S45">
-    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T42&gt;=LARGE($T$42:$T$45,2), AND($T42=LARGE($T$42:$T$45,3), $T42&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J48:S51">
-    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T48&gt;=LARGE($T$48:$T$51,2), AND($T48=LARGE($T$48:$T$51,3), $T48&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J54:S57">
-    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T54&gt;=LARGE($T$54:$T$57,2), AND($T54=LARGE($T$54:$T$57,3), $T54&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J60:S63">
-    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T60&gt;=LARGE($T$60:$T$63,2), AND($T60=LARGE($T$60:$T$63,3), $T60&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J66:S69">
-    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T66&gt;=LARGE($T$66:$T$69,2), AND($T66=LARGE($T$66:$T$69,3), $T66&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J72:S75">
-    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
-      <formula>=OR($T72&gt;=LARGE($T$72:$T$75,2), AND($T72=LARGE($T$72:$T$75,3), $T72&gt;=LARGE(Backend!$E$2:$E$13,8)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12480,353 +12515,351 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" style="16" min="1" max="1"/>
-    <col width="12" customWidth="1" style="16" min="2" max="2"/>
-    <col width="12" customWidth="1" style="16" min="3" max="3"/>
-    <col width="25" customWidth="1" style="16" min="4" max="4"/>
-    <col width="10" customWidth="1" style="16" min="5" max="5"/>
-    <col width="10" customWidth="1" style="16" min="6" max="6"/>
-    <col width="25" customWidth="1" style="16" min="7" max="7"/>
+    <col width="3" customWidth="1" style="28" min="1" max="1"/>
+    <col width="12" customWidth="1" style="28" min="2" max="3"/>
+    <col width="25" customWidth="1" style="28" min="4" max="4"/>
+    <col width="10" customWidth="1" style="28" min="5" max="6"/>
+    <col width="25" customWidth="1" style="28" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="30" t="inlineStr">
+      <c r="B2" s="35" t="inlineStr">
         <is>
           <t>RANKING DE MEJORES TERCEROS LUGARES</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="5">
-      <c r="B5" s="31" t="inlineStr">
+    <row r="5" ht="16.5" customHeight="1" s="28">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Posición</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>PTS</t>
         </is>
       </c>
-      <c r="F5" s="31" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>DIF</t>
         </is>
       </c>
-      <c r="G5" s="31" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>Clasifica a 16avos</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="32" t="n">
+    <row r="6" ht="16.5" customHeight="1" s="28">
+      <c r="B6" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="20">
         <f>Backend!B16</f>
         <v/>
       </c>
-      <c r="D6" s="33">
+      <c r="D6" s="21">
         <f>Backend!C16</f>
         <v/>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="20">
         <f>IF(D6="","",VLOOKUP(D6, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="20">
         <f>IF(D6="","",VLOOKUP(D6, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="22">
         <f>IF(Backend!C16="","",IF(1&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="35" t="n">
+    <row r="7" ht="16.5" customHeight="1" s="28">
+      <c r="B7" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="35">
+      <c r="C7" s="23">
         <f>Backend!B17</f>
         <v/>
       </c>
-      <c r="D7" s="36">
+      <c r="D7" s="24">
         <f>Backend!C17</f>
         <v/>
       </c>
-      <c r="E7" s="35">
+      <c r="E7" s="23">
         <f>IF(D7="","",VLOOKUP(D7, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F7" s="35">
+      <c r="F7" s="23">
         <f>IF(D7="","",VLOOKUP(D7, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G7" s="34">
+      <c r="G7" s="22">
         <f>IF(Backend!C17="","",IF(2&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="B8" s="32" t="n">
+    <row r="8" ht="16.5" customHeight="1" s="28">
+      <c r="B8" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="20">
         <f>Backend!B18</f>
         <v/>
       </c>
-      <c r="D8" s="33">
+      <c r="D8" s="21">
         <f>Backend!C18</f>
         <v/>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="20">
         <f>IF(D8="","",VLOOKUP(D8, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="20">
         <f>IF(D8="","",VLOOKUP(D8, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G8" s="34">
+      <c r="G8" s="22">
         <f>IF(Backend!C18="","",IF(3&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="35" t="n">
+    <row r="9" ht="16.5" customHeight="1" s="28">
+      <c r="B9" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="35">
+      <c r="C9" s="23">
         <f>Backend!B19</f>
         <v/>
       </c>
-      <c r="D9" s="36">
+      <c r="D9" s="24">
         <f>Backend!C19</f>
         <v/>
       </c>
-      <c r="E9" s="35">
+      <c r="E9" s="23">
         <f>IF(D9="","",VLOOKUP(D9, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F9" s="35">
+      <c r="F9" s="23">
         <f>IF(D9="","",VLOOKUP(D9, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="22">
         <f>IF(Backend!C19="","",IF(4&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="32" t="n">
+    <row r="10" ht="16.5" customHeight="1" s="28">
+      <c r="B10" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="32">
+      <c r="C10" s="20">
         <f>Backend!B20</f>
         <v/>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="21">
         <f>Backend!C20</f>
         <v/>
       </c>
-      <c r="E10" s="32">
+      <c r="E10" s="20">
         <f>IF(D10="","",VLOOKUP(D10, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F10" s="32">
+      <c r="F10" s="20">
         <f>IF(D10="","",VLOOKUP(D10, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G10" s="34">
+      <c r="G10" s="22">
         <f>IF(Backend!C20="","",IF(5&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="35" t="n">
+    <row r="11" ht="16.5" customHeight="1" s="28">
+      <c r="B11" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="C11" s="35">
+      <c r="C11" s="23">
         <f>Backend!B21</f>
         <v/>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="24">
         <f>Backend!C21</f>
         <v/>
       </c>
-      <c r="E11" s="35">
+      <c r="E11" s="23">
         <f>IF(D11="","",VLOOKUP(D11, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F11" s="35">
+      <c r="F11" s="23">
         <f>IF(D11="","",VLOOKUP(D11, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G11" s="34">
+      <c r="G11" s="22">
         <f>IF(Backend!C21="","",IF(6&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="32" t="n">
+    <row r="12" ht="16.5" customHeight="1" s="28">
+      <c r="B12" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="20">
         <f>Backend!B22</f>
         <v/>
       </c>
-      <c r="D12" s="33">
+      <c r="D12" s="21">
         <f>Backend!C22</f>
         <v/>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="20">
         <f>IF(D12="","",VLOOKUP(D12, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F12" s="32">
+      <c r="F12" s="20">
         <f>IF(D12="","",VLOOKUP(D12, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G12" s="34">
+      <c r="G12" s="22">
         <f>IF(Backend!C22="","",IF(7&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="35" t="n">
+    <row r="13" ht="16.5" customHeight="1" s="28">
+      <c r="B13" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="C13" s="35">
+      <c r="C13" s="23">
         <f>Backend!B23</f>
         <v/>
       </c>
-      <c r="D13" s="36">
+      <c r="D13" s="24">
         <f>Backend!C23</f>
         <v/>
       </c>
-      <c r="E13" s="35">
+      <c r="E13" s="23">
         <f>IF(D13="","",VLOOKUP(D13, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F13" s="35">
+      <c r="F13" s="23">
         <f>IF(D13="","",VLOOKUP(D13, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G13" s="34">
+      <c r="G13" s="22">
         <f>IF(Backend!C23="","",IF(8&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="32" t="n">
+    <row r="14" ht="16.5" customHeight="1" s="28">
+      <c r="B14" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="20">
         <f>Backend!B24</f>
         <v/>
       </c>
-      <c r="D14" s="33">
+      <c r="D14" s="21">
         <f>Backend!C24</f>
         <v/>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="20">
         <f>IF(D14="","",VLOOKUP(D14, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F14" s="32">
+      <c r="F14" s="20">
         <f>IF(D14="","",VLOOKUP(D14, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G14" s="37">
+      <c r="G14" s="25">
         <f>IF(Backend!C24="","",IF(9&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="35" t="n">
+    <row r="15" ht="16.5" customHeight="1" s="28">
+      <c r="B15" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="C15" s="35">
+      <c r="C15" s="23">
         <f>Backend!B25</f>
         <v/>
       </c>
-      <c r="D15" s="36">
+      <c r="D15" s="24">
         <f>Backend!C25</f>
         <v/>
       </c>
-      <c r="E15" s="35">
+      <c r="E15" s="23">
         <f>IF(D15="","",VLOOKUP(D15, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="23">
         <f>IF(D15="","",VLOOKUP(D15, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G15" s="37">
+      <c r="G15" s="25">
         <f>IF(Backend!C25="","",IF(10&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="32" t="n">
+    <row r="16" ht="16.5" customHeight="1" s="28">
+      <c r="B16" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="20">
         <f>Backend!B26</f>
         <v/>
       </c>
-      <c r="D16" s="33">
+      <c r="D16" s="21">
         <f>Backend!C26</f>
         <v/>
       </c>
-      <c r="E16" s="32">
+      <c r="E16" s="20">
         <f>IF(D16="","",VLOOKUP(D16, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F16" s="32">
+      <c r="F16" s="20">
         <f>IF(D16="","",VLOOKUP(D16, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G16" s="37">
+      <c r="G16" s="25">
         <f>IF(Backend!C26="","",IF(11&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="35" t="n">
+    <row r="17" ht="16.5" customHeight="1" s="28">
+      <c r="B17" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="C17" s="35">
+      <c r="C17" s="23">
         <f>Backend!B27</f>
         <v/>
       </c>
-      <c r="D17" s="36">
+      <c r="D17" s="24">
         <f>Backend!C27</f>
         <v/>
       </c>
-      <c r="E17" s="35">
+      <c r="E17" s="23">
         <f>IF(D17="","",VLOOKUP(D17, Grupos!$K$6:$S$77, 9, FALSE))</f>
         <v/>
       </c>
-      <c r="F17" s="35">
+      <c r="F17" s="23">
         <f>IF(D17="","",VLOOKUP(D17, Grupos!$K$6:$R$77, 8, FALSE))</f>
         <v/>
       </c>
-      <c r="G17" s="37">
+      <c r="G17" s="25">
         <f>IF(Backend!C27="","",IF(12&lt;=8, "✅ Avanza", "❌ Eliminado"))</f>
         <v/>
       </c>
@@ -12846,7 +12879,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E29"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -13383,45 +13416,42 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I62"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="16" min="2" max="2"/>
-    <col width="6" customWidth="1" style="16" min="3" max="3"/>
-    <col width="6" customWidth="1" style="16" min="4" max="4"/>
-    <col width="3" customWidth="1" style="16" min="5" max="5"/>
-    <col width="6" customWidth="1" style="16" min="6" max="7"/>
-    <col width="6" customWidth="1" style="16" min="7" max="7"/>
-    <col width="18" customWidth="1" style="16" min="8" max="8"/>
-    <col width="18" customWidth="1" style="16" min="9" max="9"/>
+    <col width="20" customWidth="1" style="28" min="2" max="2"/>
+    <col width="6" customWidth="1" style="28" min="3" max="4"/>
+    <col width="3" customWidth="1" style="28" min="5" max="5"/>
+    <col width="6" customWidth="1" style="28" min="6" max="7"/>
+    <col width="18" customWidth="1" style="28" min="8" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>FASE FINAL (ELIMINACIÓN DIRECTA)</t>
         </is>
       </c>
     </row>
     <row r="2"/>
-    <row r="4" ht="18.75" customHeight="1" s="16">
-      <c r="A4" s="27" t="inlineStr">
+    <row r="4" ht="18.75" customHeight="1" s="28">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>DIECISEISAVOS DE FINAL (Ronda de 32)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="16">
-      <c r="A5" s="14" t="inlineStr">
+    <row r="5" ht="16.5" customHeight="1" s="28">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Equipo A</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
@@ -13431,7 +13461,7 @@
           <t>Pen.</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
@@ -13441,17 +13471,17 @@
           <t>Pen.</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="I5" s="14" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
         </is>
@@ -13468,13 +13498,13 @@
         <v/>
       </c>
       <c r="C6" s="5" t="n"/>
-      <c r="D6" s="38" t="n"/>
+      <c r="D6" s="26" t="n"/>
       <c r="E6" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F6" s="38" t="n"/>
+      <c r="F6" s="26" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6">
         <f>Backend!C3</f>
@@ -13496,13 +13526,13 @@
         <v/>
       </c>
       <c r="C7" s="5" t="n"/>
-      <c r="D7" s="38" t="n"/>
+      <c r="D7" s="26" t="n"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="38" t="n"/>
+      <c r="F7" s="26" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7">
         <f>Backend!C4</f>
@@ -13524,13 +13554,13 @@
         <v/>
       </c>
       <c r="C8" s="5" t="n"/>
-      <c r="D8" s="38" t="n"/>
+      <c r="D8" s="26" t="n"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="38" t="n"/>
+      <c r="F8" s="26" t="n"/>
       <c r="G8" s="5" t="n"/>
       <c r="H8">
         <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 5, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
@@ -13552,13 +13582,13 @@
         <v/>
       </c>
       <c r="C9" s="5" t="n"/>
-      <c r="D9" s="38" t="n"/>
+      <c r="D9" s="26" t="n"/>
       <c r="E9" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="38" t="n"/>
+      <c r="F9" s="26" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9">
         <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 7, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
@@ -13580,13 +13610,13 @@
         <v/>
       </c>
       <c r="C10" s="5" t="n"/>
-      <c r="D10" s="38" t="n"/>
+      <c r="D10" s="26" t="n"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="38" t="n"/>
+      <c r="F10" s="26" t="n"/>
       <c r="G10" s="5" t="n"/>
       <c r="H10">
         <f>Backend!C7</f>
@@ -13608,13 +13638,13 @@
         <v/>
       </c>
       <c r="C11" s="5" t="n"/>
-      <c r="D11" s="38" t="n"/>
+      <c r="D11" s="26" t="n"/>
       <c r="E11" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F11" s="38" t="n"/>
+      <c r="F11" s="26" t="n"/>
       <c r="G11" s="5" t="n"/>
       <c r="H11">
         <f>Backend!C10</f>
@@ -13636,13 +13666,13 @@
         <v/>
       </c>
       <c r="C12" s="5" t="n"/>
-      <c r="D12" s="38" t="n"/>
+      <c r="D12" s="26" t="n"/>
       <c r="E12" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F12" s="38" t="n"/>
+      <c r="F12" s="26" t="n"/>
       <c r="G12" s="5" t="n"/>
       <c r="H12">
         <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 2, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
@@ -13664,13 +13694,13 @@
         <v/>
       </c>
       <c r="C13" s="5" t="n"/>
-      <c r="D13" s="38" t="n"/>
+      <c r="D13" s="26" t="n"/>
       <c r="E13" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F13" s="38" t="n"/>
+      <c r="F13" s="26" t="n"/>
       <c r="G13" s="5" t="n"/>
       <c r="H13">
         <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 9, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
@@ -13692,13 +13722,13 @@
         <v/>
       </c>
       <c r="C14" s="5" t="n"/>
-      <c r="D14" s="38" t="n"/>
+      <c r="D14" s="26" t="n"/>
       <c r="E14" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F14" s="38" t="n"/>
+      <c r="F14" s="26" t="n"/>
       <c r="G14" s="5" t="n"/>
       <c r="H14">
         <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 4, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
@@ -13720,13 +13750,13 @@
         <v/>
       </c>
       <c r="C15" s="5" t="n"/>
-      <c r="D15" s="38" t="n"/>
+      <c r="D15" s="26" t="n"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F15" s="38" t="n"/>
+      <c r="F15" s="26" t="n"/>
       <c r="G15" s="5" t="n"/>
       <c r="H15">
         <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 6, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
@@ -13748,13 +13778,13 @@
         <v/>
       </c>
       <c r="C16" s="5" t="n"/>
-      <c r="D16" s="38" t="n"/>
+      <c r="D16" s="26" t="n"/>
       <c r="E16" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F16" s="38" t="n"/>
+      <c r="F16" s="26" t="n"/>
       <c r="G16" s="5" t="n"/>
       <c r="H16">
         <f>Backend!C13</f>
@@ -13776,13 +13806,13 @@
         <v/>
       </c>
       <c r="C17" s="5" t="n"/>
-      <c r="D17" s="38" t="n"/>
+      <c r="D17" s="26" t="n"/>
       <c r="E17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="38" t="n"/>
+      <c r="F17" s="26" t="n"/>
       <c r="G17" s="5" t="n"/>
       <c r="H17">
         <f>Backend!C11</f>
@@ -13804,13 +13834,13 @@
         <v/>
       </c>
       <c r="C18" s="5" t="n"/>
-      <c r="D18" s="38" t="n"/>
+      <c r="D18" s="26" t="n"/>
       <c r="E18" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F18" s="38" t="n"/>
+      <c r="F18" s="26" t="n"/>
       <c r="G18" s="5" t="n"/>
       <c r="H18">
         <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 3, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
@@ -13832,13 +13862,13 @@
         <v/>
       </c>
       <c r="C19" s="5" t="n"/>
-      <c r="D19" s="38" t="n"/>
+      <c r="D19" s="26" t="n"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F19" s="38" t="n"/>
+      <c r="F19" s="26" t="n"/>
       <c r="G19" s="5" t="n"/>
       <c r="H19">
         <f>IFERROR(INDEX(Backend!$C$16:$C$23, MATCH(VLOOKUP(Backend!$D$29, MatrizTerceros!$A$1:$I$495, 8, FALSE), Backend!$B$16:$B$23, 0)), "")</f>
@@ -13860,13 +13890,13 @@
         <v/>
       </c>
       <c r="C20" s="5" t="n"/>
-      <c r="D20" s="38" t="n"/>
+      <c r="D20" s="26" t="n"/>
       <c r="E20" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F20" s="38" t="n"/>
+      <c r="F20" s="26" t="n"/>
       <c r="G20" s="5" t="n"/>
       <c r="H20">
         <f>Backend!C9</f>
@@ -13888,13 +13918,13 @@
         <v/>
       </c>
       <c r="C21" s="5" t="n"/>
-      <c r="D21" s="38" t="n"/>
+      <c r="D21" s="26" t="n"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F21" s="38" t="n"/>
+      <c r="F21" s="26" t="n"/>
       <c r="G21" s="5" t="n"/>
       <c r="H21">
         <f>Backend!C8</f>
@@ -13905,8 +13935,8 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="18.75" customHeight="1" s="16">
-      <c r="A23" s="27" t="inlineStr">
+    <row r="23" ht="18.75" customHeight="1" s="28">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>OCTAVOS DE FINAL</t>
         </is>
@@ -13923,13 +13953,13 @@
         <v/>
       </c>
       <c r="C25" s="5" t="n"/>
-      <c r="D25" s="38" t="n"/>
+      <c r="D25" s="26" t="n"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F25" s="38" t="n"/>
+      <c r="F25" s="26" t="n"/>
       <c r="G25" s="5" t="n"/>
       <c r="H25">
         <f>I7</f>
@@ -13951,13 +13981,13 @@
         <v/>
       </c>
       <c r="C26" s="5" t="n"/>
-      <c r="D26" s="38" t="n"/>
+      <c r="D26" s="26" t="n"/>
       <c r="E26" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F26" s="38" t="n"/>
+      <c r="F26" s="26" t="n"/>
       <c r="G26" s="5" t="n"/>
       <c r="H26">
         <f>I9</f>
@@ -13979,13 +14009,13 @@
         <v/>
       </c>
       <c r="C27" s="5" t="n"/>
-      <c r="D27" s="38" t="n"/>
+      <c r="D27" s="26" t="n"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F27" s="38" t="n"/>
+      <c r="F27" s="26" t="n"/>
       <c r="G27" s="5" t="n"/>
       <c r="H27">
         <f>I11</f>
@@ -14007,13 +14037,13 @@
         <v/>
       </c>
       <c r="C28" s="5" t="n"/>
-      <c r="D28" s="38" t="n"/>
+      <c r="D28" s="26" t="n"/>
       <c r="E28" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F28" s="38" t="n"/>
+      <c r="F28" s="26" t="n"/>
       <c r="G28" s="5" t="n"/>
       <c r="H28">
         <f>I13</f>
@@ -14035,13 +14065,13 @@
         <v/>
       </c>
       <c r="C29" s="5" t="n"/>
-      <c r="D29" s="38" t="n"/>
+      <c r="D29" s="26" t="n"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F29" s="38" t="n"/>
+      <c r="F29" s="26" t="n"/>
       <c r="G29" s="5" t="n"/>
       <c r="H29">
         <f>I15</f>
@@ -14063,13 +14093,13 @@
         <v/>
       </c>
       <c r="C30" s="5" t="n"/>
-      <c r="D30" s="38" t="n"/>
+      <c r="D30" s="26" t="n"/>
       <c r="E30" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F30" s="38" t="n"/>
+      <c r="F30" s="26" t="n"/>
       <c r="G30" s="5" t="n"/>
       <c r="H30">
         <f>I17</f>
@@ -14091,13 +14121,13 @@
         <v/>
       </c>
       <c r="C31" s="5" t="n"/>
-      <c r="D31" s="38" t="n"/>
+      <c r="D31" s="26" t="n"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F31" s="38" t="n"/>
+      <c r="F31" s="26" t="n"/>
       <c r="G31" s="5" t="n"/>
       <c r="H31">
         <f>I19</f>
@@ -14119,13 +14149,13 @@
         <v/>
       </c>
       <c r="C32" s="5" t="n"/>
-      <c r="D32" s="38" t="n"/>
+      <c r="D32" s="26" t="n"/>
       <c r="E32" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F32" s="38" t="n"/>
+      <c r="F32" s="26" t="n"/>
       <c r="G32" s="5" t="n"/>
       <c r="H32">
         <f>I21</f>
@@ -14154,45 +14184,45 @@
       <c r="H34" s="8" t="n"/>
       <c r="I34" s="8" t="n"/>
     </row>
-    <row r="35" ht="18.75" customHeight="1" s="16">
-      <c r="A35" s="28" t="inlineStr">
+    <row r="35" ht="18.75" customHeight="1" s="28">
+      <c r="A35" s="32" t="inlineStr">
         <is>
           <t>CUARTOS DE FINAL</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="16">
-      <c r="A36" s="14" t="inlineStr">
+    <row r="36" ht="16.5" customHeight="1" s="28">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Equipo A</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="E36" s="14" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="H36" s="14" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="I36" s="14" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
         </is>
@@ -14209,13 +14239,13 @@
         <v/>
       </c>
       <c r="C37" s="5" t="n"/>
-      <c r="D37" s="38" t="n"/>
+      <c r="D37" s="26" t="n"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F37" s="38" t="n"/>
+      <c r="F37" s="26" t="n"/>
       <c r="G37" s="5" t="n"/>
       <c r="H37">
         <f>I26</f>
@@ -14237,13 +14267,13 @@
         <v/>
       </c>
       <c r="C38" s="5" t="n"/>
-      <c r="D38" s="38" t="n"/>
+      <c r="D38" s="26" t="n"/>
       <c r="E38" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F38" s="38" t="n"/>
+      <c r="F38" s="26" t="n"/>
       <c r="G38" s="5" t="n"/>
       <c r="H38">
         <f>I28</f>
@@ -14265,13 +14295,13 @@
         <v/>
       </c>
       <c r="C39" s="5" t="n"/>
-      <c r="D39" s="38" t="n"/>
+      <c r="D39" s="26" t="n"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F39" s="38" t="n"/>
+      <c r="F39" s="26" t="n"/>
       <c r="G39" s="5" t="n"/>
       <c r="H39">
         <f>I30</f>
@@ -14293,13 +14323,13 @@
         <v/>
       </c>
       <c r="C40" s="5" t="n"/>
-      <c r="D40" s="38" t="n"/>
+      <c r="D40" s="26" t="n"/>
       <c r="E40" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F40" s="38" t="n"/>
+      <c r="F40" s="26" t="n"/>
       <c r="G40" s="5" t="n"/>
       <c r="H40">
         <f>I32</f>
@@ -14328,45 +14358,45 @@
       <c r="H42" s="8" t="n"/>
       <c r="I42" s="8" t="n"/>
     </row>
-    <row r="43" ht="18.75" customHeight="1" s="16">
-      <c r="A43" s="28" t="inlineStr">
+    <row r="43" ht="18.75" customHeight="1" s="28">
+      <c r="A43" s="32" t="inlineStr">
         <is>
           <t>SEMIFINALES</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="16">
-      <c r="A44" s="14" t="inlineStr">
+    <row r="44" ht="16.5" customHeight="1" s="28">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Equipo A</t>
         </is>
       </c>
-      <c r="C44" s="14" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="G44" s="14" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="H44" s="14" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="I44" s="14" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
         </is>
@@ -14383,13 +14413,13 @@
         <v/>
       </c>
       <c r="C45" s="5" t="n"/>
-      <c r="D45" s="38" t="n"/>
+      <c r="D45" s="26" t="n"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F45" s="38" t="n"/>
+      <c r="F45" s="26" t="n"/>
       <c r="G45" s="5" t="n"/>
       <c r="H45">
         <f>I38</f>
@@ -14411,13 +14441,13 @@
         <v/>
       </c>
       <c r="C46" s="5" t="n"/>
-      <c r="D46" s="38" t="n"/>
+      <c r="D46" s="26" t="n"/>
       <c r="E46" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F46" s="38" t="n"/>
+      <c r="F46" s="26" t="n"/>
       <c r="G46" s="5" t="n"/>
       <c r="H46">
         <f>I40</f>
@@ -14446,45 +14476,45 @@
       <c r="H48" s="8" t="n"/>
       <c r="I48" s="8" t="n"/>
     </row>
-    <row r="49" ht="18.75" customHeight="1" s="16">
-      <c r="A49" s="28" t="inlineStr">
+    <row r="49" ht="18.75" customHeight="1" s="28">
+      <c r="A49" s="32" t="inlineStr">
         <is>
           <t>PARTIDO POR EL TERCER LUGAR</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="16">
-      <c r="A50" s="14" t="inlineStr">
+    <row r="50" ht="16.5" customHeight="1" s="28">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Equipo A</t>
         </is>
       </c>
-      <c r="C50" s="14" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="G50" s="14" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="H50" s="14" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="I50" s="14" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
         </is>
@@ -14501,13 +14531,13 @@
         <v/>
       </c>
       <c r="C51" s="5" t="n"/>
-      <c r="D51" s="38" t="n"/>
+      <c r="D51" s="26" t="n"/>
       <c r="E51" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F51" s="38" t="n"/>
+      <c r="F51" s="26" t="n"/>
       <c r="G51" s="5" t="n"/>
       <c r="H51">
         <f>IF(OR(C46="", G46=""), "", IF(C46&lt;G46, B46, IF(G46&lt;C46, H46, IF(D46&lt;F46, B46, IF(F46&lt;D46, H46, "")))))</f>
@@ -14536,45 +14566,45 @@
       <c r="H53" s="8" t="n"/>
       <c r="I53" s="8" t="n"/>
     </row>
-    <row r="54" ht="18.75" customHeight="1" s="16">
-      <c r="A54" s="28" t="inlineStr">
+    <row r="54" ht="18.75" customHeight="1" s="28">
+      <c r="A54" s="32" t="inlineStr">
         <is>
           <t>GRAN FINAL</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="16">
-      <c r="A55" s="14" t="inlineStr">
+    <row r="55" ht="16.5" customHeight="1" s="28">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
         </is>
       </c>
-      <c r="B55" s="14" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Equipo A</t>
         </is>
       </c>
-      <c r="C55" s="14" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="E55" s="14" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="G55" s="14" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>Goles</t>
         </is>
       </c>
-      <c r="H55" s="14" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>Equipo B</t>
         </is>
       </c>
-      <c r="I55" s="14" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
         </is>
@@ -14591,13 +14621,13 @@
         <v/>
       </c>
       <c r="C56" s="5" t="n"/>
-      <c r="D56" s="38" t="n"/>
+      <c r="D56" s="26" t="n"/>
       <c r="E56" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F56" s="38" t="n"/>
+      <c r="F56" s="26" t="n"/>
       <c r="G56" s="5" t="n"/>
       <c r="H56">
         <f>I46</f>
@@ -14626,16 +14656,16 @@
       <c r="H58" s="8" t="n"/>
       <c r="I58" s="8" t="n"/>
     </row>
-    <row r="59" ht="18.75" customHeight="1" s="16">
-      <c r="A59" s="28" t="inlineStr">
+    <row r="59" ht="18.75" customHeight="1" s="28">
+      <c r="A59" s="32" t="inlineStr">
         <is>
           <t>PODIO DE HONOR 🏆</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="16">
+    <row r="60" ht="16.5" customHeight="1" s="28">
       <c r="A60" s="8" t="n"/>
-      <c r="B60" s="29" t="inlineStr">
+      <c r="B60" s="33" t="inlineStr">
         <is>
           <t>CAMPEÓN MUNDIAL 🏆</t>
         </is>
@@ -14646,9 +14676,9 @@
       </c>
       <c r="I60" s="8" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="16">
+    <row r="61" ht="16.5" customHeight="1" s="28">
       <c r="A61" s="8" t="n"/>
-      <c r="B61" s="29" t="inlineStr">
+      <c r="B61" s="33" t="inlineStr">
         <is>
           <t>Subcampeón 🥈</t>
         </is>
@@ -14659,9 +14689,9 @@
       </c>
       <c r="I61" s="8" t="n"/>
     </row>
-    <row r="62" ht="16.5" customHeight="1" s="16">
+    <row r="62" ht="16.5" customHeight="1" s="28">
       <c r="A62" s="8" t="n"/>
-      <c r="B62" s="29" t="inlineStr">
+      <c r="B62" s="33" t="inlineStr">
         <is>
           <t>Tercer Lugar 🥉</t>
         </is>
@@ -14675,15 +14705,15 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A59:I59"/>
-    <mergeCell ref="B62:G62"/>
     <mergeCell ref="A43:I43"/>
     <mergeCell ref="A49:I49"/>
     <mergeCell ref="B60:G60"/>
+    <mergeCell ref="A4:I4"/>
     <mergeCell ref="B61:G61"/>
     <mergeCell ref="A23:I23"/>
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="B62:G62"/>
     <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14696,23 +14726,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B183"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B183"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="124.28515625" customWidth="1" style="16" min="2" max="2"/>
+    <col width="124.28515625" customWidth="1" style="28" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="2" ht="26.25" customHeight="1" s="16">
-      <c r="B2" s="18" t="inlineStr">
+    <row r="1"/>
+    <row r="2" ht="26.25" customHeight="1" s="28">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Fase de grupos: calendario y horarios de la Copa Mundial de la FIFA 2026™</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>Todos los horarios son del Este de Estados Unidos. Hay que restarle  2 horas para tener el horario de México.</t>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Todos los horarios son de la Ciudad de México.</t>
         </is>
       </c>
     </row>
@@ -14726,17 +14758,18 @@
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>15:00 - México v Sudáfrica – Grupo A - Estadio Ciudad de México</t>
+          <t>13:00 - México v Sudáfrica – Grupo A - Estadio Ciudad de México</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>22:00 - República de Corea v República Checa – Grupo A - Estadio Guadalajara</t>
-        </is>
-      </c>
-    </row>
+          <t>20:00 - República de Corea v República Checa – Grupo A - Estadio Guadalajara</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
@@ -14747,17 +14780,18 @@
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>15:00 - Canadá v Bosnia y Herzegovina – Grupo B - Estadio Toronto</t>
+          <t>13:00 - Canadá v Bosnia y Herzegovina – Grupo B - Estadio Toronto</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>21:00 - Estados Unidos v Paraguay – Grupo D - Estadio Los Ángeles</t>
-        </is>
-      </c>
-    </row>
+          <t>19:00 - Estados Unidos v Paraguay – Grupo D - Estadio Los Ángeles</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
@@ -14768,31 +14802,32 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>15:00 - Catar v Suiza – Grupo B - Estadio Bahía de San Francisco</t>
+          <t>13:00 - Catar v Suiza – Grupo B - Estadio Bahía de San Francisco</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>18:00 - Brasil v Marruecos – Grupo C - Estadio Nueva York Nueva Jersey</t>
+          <t>16:00 - Brasil v Marruecos – Grupo C - Estadio Nueva York Nueva Jersey</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>21:00 - Haití v Escocia – Grupo C - Estadio Boston</t>
+          <t>19:00 - Haití v Escocia – Grupo C - Estadio Boston</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>00:00 - Australia v Turquía – Grupo D - Estadio BC Place Vancouver</t>
-        </is>
-      </c>
-    </row>
+          <t>22:00 - Australia v Turquía – Grupo D - Estadio BC Place Vancouver</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
@@ -14803,31 +14838,32 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>13:00 - Alemania v Curazao – Grupo E - Estadio Houston</t>
+          <t>11:00 - Alemania v Curazao – Grupo E - Estadio Houston</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>16:00 - Países Bajos v Japón – Grupo F - Estadio Dallas</t>
+          <t>14:00 - Países Bajos v Japón – Grupo F - Estadio Dallas</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>19:00 - Costa de Marfil v Ecuador – Grupo E - Estadio Filadelfia</t>
+          <t>17:00 - Costa de Marfil v Ecuador – Grupo E - Estadio Filadelfia</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>22:00 - Suecia v Túnez – Grupo F - Estadio Monterrey</t>
-        </is>
-      </c>
-    </row>
+          <t>20:00 - Suecia v Túnez – Grupo F - Estadio Monterrey</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
@@ -14838,31 +14874,32 @@
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>12:00 - España v Cabo Verde – Grupo H - Estadio Atlanta</t>
+          <t>10:00 - España v Cabo Verde – Grupo H - Estadio Atlanta</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>15:00 - Bélgica v Egipto – Grupo G - Estadio Seattle</t>
+          <t>13:00 - Bélgica v Egipto – Grupo G - Estadio Seattle</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>18:00 - Arabia Saudí v Uruguay – Grupo H - Estadio Miami</t>
+          <t>16:00 - Arabia Saudí v Uruguay – Grupo H - Estadio Miami</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>21:00 - RI de Irán v Nueva Zelanda – Grupo G - Estadio Los Ángeles</t>
-        </is>
-      </c>
-    </row>
+          <t>19:00 - RI de Irán v Nueva Zelanda – Grupo G - Estadio Los Ángeles</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
@@ -14873,31 +14910,32 @@
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>15:00 - Francia v Senegal – Grupo I - Estadio Nueva York Nueva Jersey</t>
+          <t>13:00 - Francia v Senegal – Grupo I - Estadio Nueva York Nueva Jersey</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>18:00 - Irak v Noruega – Grupo I - Estadio Boston</t>
+          <t>16:00 - Irak v Noruega – Grupo I - Estadio Boston</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>21:00 - Argentina v Argelia – Grupo J - Estadio Kansas City</t>
+          <t>19:00 - Argentina v Argelia – Grupo J - Estadio Kansas City</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>00:00 - Austria v Jordania – Grupo J - Estadio Bahía de San Francisco</t>
-        </is>
-      </c>
-    </row>
+          <t>22:00 - Austria v Jordania – Grupo J - Estadio Bahía de San Francisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
@@ -14908,31 +14946,32 @@
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>13:00 - Portugal v RD Congo – Grupo K - Estadio Houston</t>
+          <t>11:00 - Portugal v RD Congo – Grupo K - Estadio Houston</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>16:00 - Inglaterra v Croacia – Grupo L - Estadio Dallas</t>
+          <t>14:00 - Inglaterra v Croacia – Grupo L - Estadio Dallas</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>19:00 - Ghana v Panamá – Grupo L - Estadio Toronto</t>
+          <t>17:00 - Ghana v Panamá – Grupo L - Estadio Toronto</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>22:00 - Uzbekistán v Colombia – Grupo K - Estadio Ciudad de México</t>
-        </is>
-      </c>
-    </row>
+          <t>20:00 - Uzbekistán v Colombia – Grupo K - Estadio Ciudad de México</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
@@ -14943,31 +14982,32 @@
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>12:00 - República Checa v Sudáfrica – Grupo A - Estadio Atlanta</t>
+          <t>10:00 - República Checa v Sudáfrica – Grupo A - Estadio Atlanta</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>15:00 - Suiza v Bosnia y Herzegovina – Grupo B - Estadio Los Ángeles</t>
+          <t>13:00 - Suiza v Bosnia y Herzegovina – Grupo B - Estadio Los Ángeles</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>18:00 - Canadá v Catar – Grupo B - Estadio BC Place Vancouver</t>
+          <t>16:00 - Canadá v Catar – Grupo B - Estadio BC Place Vancouver</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>21:00 - México v República de Corea – Grupo A - Estadio Guadalajara</t>
-        </is>
-      </c>
-    </row>
+          <t>19:00 - México v República de Corea – Grupo A - Estadio Guadalajara</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
@@ -14978,31 +15018,32 @@
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>15:00 - Estados Unidos v Australia – Grupo D - Estadio Seattle</t>
+          <t>13:00 - Estados Unidos v Australia – Grupo D - Estadio Seattle</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>18:00 - Escocia v Marruecos – Grupo C - Estadio Boston</t>
+          <t>16:00 - Escocia v Marruecos – Grupo C - Estadio Boston</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>21:00 - Brasil v Haití – Grupo C - Estadio Filadelfia</t>
+          <t>19:00 - Brasil v Haití – Grupo C - Estadio Filadelfia</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>00:00 - Turquía v Paraguay – Grupo D - Estadio Bahía de San Francisco</t>
-        </is>
-      </c>
-    </row>
+          <t>22:00 - Turquía v Paraguay – Grupo D - Estadio Bahía de San Francisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
@@ -15013,31 +15054,33 @@
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>13:00 - Países Bajos v Suecia – Grupo F - Estadio Houston</t>
+          <t>11:00 - Países Bajos v Suecia – Grupo F - Estadio Houston</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>16:00 - Alemania v Costa de Marfil – Grupo E - Estadio Toronto</t>
+          <t>14:00 - Alemania v Costa de Marfil – Grupo E - Estadio Toronto</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t>22:00 - Ecuador v Curazao – Grupo E - Estadio Kansas City</t>
+          <t>20:00 - Ecuador v Curazao – Grupo E - Estadio Kansas City</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>00:00 - Túnez v Japón – Grupo F - Estadio Monterrey</t>
-        </is>
-      </c>
-    </row>
+          <t>22:00 - Túnez v Japón – Grupo F - Estadio Monterrey</t>
+        </is>
+      </c>
+    </row>
+    <row r="60"/>
+    <row r="61"/>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
@@ -15048,31 +15091,32 @@
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>12:00 - España v Arabia Saudí – Grupo H - Estadio Atlanta</t>
+          <t>10:00 - España v Arabia Saudí – Grupo H - Estadio Atlanta</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>15:00 - Bélgica v Irán – Grupo G - Estadio Los Ángeles</t>
+          <t>13:00 - Bélgica v Irán – Grupo G - Estadio Los Ángeles</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t>18:00 - Uruguay v Cabo Verde – Grupo H - Estadio Miami</t>
+          <t>16:00 - Uruguay v Cabo Verde – Grupo H - Estadio Miami</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" t="inlineStr">
         <is>
-          <t>21:00 - Nueva Zelanda v Egipto – Grupo G - Estadio BC Place Vancouver</t>
-        </is>
-      </c>
-    </row>
+          <t>19:00 - Nueva Zelanda v Egipto – Grupo G - Estadio BC Place Vancouver</t>
+        </is>
+      </c>
+    </row>
+    <row r="67"/>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
@@ -15083,31 +15127,32 @@
     <row r="69">
       <c r="B69" t="inlineStr">
         <is>
-          <t>13:00 - Argentina v Austria – Grupo J - Estadio Dallas</t>
+          <t>11:00 - Argentina v Austria – Grupo J - Estadio Dallas</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t>17:00 - Francia v Irak – Grupo I - Estadio Filadelfia</t>
+          <t>15:00 - Francia v Irak – Grupo I - Estadio Filadelfia</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>20:00 - Noruega v Senegal – Grupo I - Estadio Nueva York Nueva Jersey</t>
+          <t>18:00 - Noruega v Senegal – Grupo I - Estadio Nueva York Nueva Jersey</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
-          <t>23:00 - Jordania v Argelia – Grupo J - Estadio Bahía de San Francisco Bay</t>
-        </is>
-      </c>
-    </row>
+          <t>21:00 - Jordania v Argelia – Grupo J - Estadio Bahía de San Francisco Bay</t>
+        </is>
+      </c>
+    </row>
+    <row r="73"/>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
@@ -15118,31 +15163,32 @@
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t>13:00 - Portugal v Uzbekistán – Grupo K - Estadio Houston</t>
+          <t>11:00 - Portugal v Uzbekistán – Grupo K - Estadio Houston</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" t="inlineStr">
         <is>
-          <t>16:00 - Inglaterra v Ghana – Grupo L - Estadio Boston</t>
+          <t>14:00 - Inglaterra v Ghana – Grupo L - Estadio Boston</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>19:00 - Panamá v Croacia – Grupo L - Estadio Toronto</t>
+          <t>17:00 - Panamá v Croacia – Grupo L - Estadio Toronto</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>22:00 - Colombia v RD Congo – Grupo K - Estadio Guadalajara</t>
-        </is>
-      </c>
-    </row>
+          <t>20:00 - Colombia v RD Congo – Grupo K - Estadio Guadalajara</t>
+        </is>
+      </c>
+    </row>
+    <row r="79"/>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
@@ -15153,45 +15199,46 @@
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>15:00 - Suiza v Canadá – Grupo B - Estadio BC Place Vancouver</t>
+          <t>13:00 - Suiza v Canadá – Grupo B - Estadio BC Place Vancouver</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>15:00 - Bosnia y Herzegovina v Catar – Grupo B - Estadio Seattle</t>
+          <t>13:00 - Bosnia y Herzegovina v Catar – Grupo B - Estadio Seattle</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>18:00 - Escocia v Brasil – Grupo C - Estadio Miami</t>
+          <t>16:00 - Escocia v Brasil – Grupo C - Estadio Miami</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>18:00 - Marruecos v Haití – Grupo C - Estadio Atlanta</t>
+          <t>16:00 - Marruecos v Haití – Grupo C - Estadio Atlanta</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>21:00 - República Checa v México – Grupo A - Estadio Ciudad de México</t>
+          <t>19:00 - República Checa v México – Grupo A - Estadio Ciudad de México</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>21:00 - Sudáfrica v República de Corea – Grupo A - Estadio Monterrey</t>
-        </is>
-      </c>
-    </row>
+          <t>19:00 - Sudáfrica v República de Corea – Grupo A - Estadio Monterrey</t>
+        </is>
+      </c>
+    </row>
+    <row r="87"/>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
@@ -15202,45 +15249,46 @@
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>16:00 - Curazao v Costa de Marfil – Grupo E - Estadio Filadelfia</t>
+          <t>14:00 - Curazao v Costa de Marfil – Grupo E - Estadio Filadelfia</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>16:00 - Ecuador v Alemania – Grupo E - Estadio Nueva York Nueva Jersey</t>
+          <t>14:00 - Ecuador v Alemania – Grupo E - Estadio Nueva York Nueva Jersey</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>19:00 - Japón v Suecia – Grupo F - Estadio Dallas</t>
+          <t>17:00 - Japón v Suecia – Grupo F - Estadio Dallas</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>19:00 - Túnez v Países Bajos – Grupo F - Estadio Kansas City</t>
+          <t>17:00 - Túnez v Países Bajos – Grupo F - Estadio Kansas City</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>22:00 - Turquía v Estados Unidos – Grupo D - Estadio Los Ángeles</t>
+          <t>20:00 - Turquía v Estados Unidos – Grupo D - Estadio Los Ángeles</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>22:00 - Paraguay v Australia – Grupo D - Estadio Bahía de San Francisco</t>
-        </is>
-      </c>
-    </row>
+          <t>20:00 - Paraguay v Australia – Grupo D - Estadio Bahía de San Francisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="95"/>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
@@ -15251,45 +15299,46 @@
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>15:00 - Noruega v Francia – Grupo I - Estadio Boston</t>
+          <t>13:00 - Noruega v Francia – Grupo I - Estadio Boston</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>15:00 - Senegal v Irak – Grupo I - Estadio Toronto</t>
+          <t>13:00 - Senegal v Irak – Grupo I - Estadio Toronto</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>20:00 - Cabo Verde v Arabia Saudí – Grupo H - Estadio Houston</t>
+          <t>18:00 - Cabo Verde v Arabia Saudí – Grupo H - Estadio Houston</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>20:00 - Uruguay v España – Grupo H - Estadio Guadalajara</t>
+          <t>18:00 - Uruguay v España – Grupo H - Estadio Guadalajara</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>23:00 - Egipto v Irán – Grupo G - Estadio Seattle</t>
+          <t>21:00 - Egipto v Irán – Grupo G - Estadio Seattle</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>23:00 - Nueva Zelanda v Bélgica – Grupo G - Estadio BC Place Vancouver</t>
-        </is>
-      </c>
-    </row>
+          <t>21:00 - Nueva Zelanda v Bélgica – Grupo G - Estadio BC Place Vancouver</t>
+        </is>
+      </c>
+    </row>
+    <row r="103"/>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
@@ -15300,45 +15349,46 @@
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>17:00 - Panamá v Inglaterra – Grupo L - Estadio Nueva York Nueva Jersey</t>
+          <t>15:00 - Panamá v Inglaterra – Grupo L - Estadio Nueva York Nueva Jersey</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>17:00 - Croacia v Ghana – Grupo L - Estadio Filadelfia</t>
+          <t>15:00 - Croacia v Ghana – Grupo L - Estadio Filadelfia</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>19:30 - Colombia v Portugal – Grupo K - Estadio Miami</t>
+          <t>17:30 - Colombia v Portugal – Grupo K - Estadio Miami</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>19:30 - RD Congo v Uzbekistán – Grupo K - Estadio Atlanta</t>
+          <t>17:30 - RD Congo v Uzbekistán – Grupo K - Estadio Atlanta</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>22:00 - Argelia v Austria – Grupo J - Estadio Kansas City</t>
+          <t>20:00 - Argelia v Austria – Grupo J - Estadio Kansas City</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>22:00 - Jordania v Argentina – Grupo J - Estadio Dallas</t>
-        </is>
-      </c>
-    </row>
+          <t>20:00 - Jordania v Argentina – Grupo J - Estadio Dallas</t>
+        </is>
+      </c>
+    </row>
+    <row r="111"/>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
@@ -15346,6 +15396,7 @@
         </is>
       </c>
     </row>
+    <row r="113"/>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
@@ -15360,6 +15411,7 @@
         </is>
       </c>
     </row>
+    <row r="116"/>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
@@ -15388,6 +15440,7 @@
         </is>
       </c>
     </row>
+    <row r="121"/>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
@@ -15416,6 +15469,7 @@
         </is>
       </c>
     </row>
+    <row r="126"/>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
@@ -15444,6 +15498,7 @@
         </is>
       </c>
     </row>
+    <row r="131"/>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
@@ -15472,6 +15527,7 @@
         </is>
       </c>
     </row>
+    <row r="136"/>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
@@ -15500,6 +15556,7 @@
         </is>
       </c>
     </row>
+    <row r="141"/>
     <row r="142">
       <c r="B142" t="inlineStr">
         <is>
@@ -15528,6 +15585,7 @@
         </is>
       </c>
     </row>
+    <row r="146"/>
     <row r="147">
       <c r="B147" t="inlineStr">
         <is>
@@ -15549,6 +15607,7 @@
         </is>
       </c>
     </row>
+    <row r="150"/>
     <row r="151">
       <c r="B151" t="inlineStr">
         <is>
@@ -15570,6 +15629,7 @@
         </is>
       </c>
     </row>
+    <row r="154"/>
     <row r="155">
       <c r="B155" t="inlineStr">
         <is>
@@ -15591,6 +15651,7 @@
         </is>
       </c>
     </row>
+    <row r="158"/>
     <row r="159">
       <c r="B159" t="inlineStr">
         <is>
@@ -15612,6 +15673,7 @@
         </is>
       </c>
     </row>
+    <row r="162"/>
     <row r="163">
       <c r="B163" t="inlineStr">
         <is>
@@ -15626,6 +15688,7 @@
         </is>
       </c>
     </row>
+    <row r="165"/>
     <row r="166">
       <c r="B166" t="inlineStr">
         <is>
@@ -15647,6 +15710,7 @@
         </is>
       </c>
     </row>
+    <row r="169"/>
     <row r="170">
       <c r="B170" t="inlineStr">
         <is>
@@ -15668,6 +15732,7 @@
         </is>
       </c>
     </row>
+    <row r="173"/>
     <row r="174">
       <c r="B174" t="inlineStr">
         <is>
@@ -15682,6 +15747,7 @@
         </is>
       </c>
     </row>
+    <row r="176"/>
     <row r="177">
       <c r="B177" t="inlineStr">
         <is>
@@ -15703,6 +15769,7 @@
         </is>
       </c>
     </row>
+    <row r="180"/>
     <row r="181">
       <c r="B181" t="inlineStr">
         <is>
@@ -15736,37 +15803,37 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="146" customWidth="1" style="16" min="2" max="2"/>
+    <col width="146" customWidth="1" style="28" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="2" ht="26.25" customHeight="1" s="16">
-      <c r="B2" s="18" t="inlineStr">
+    <row r="2" ht="26.25" customHeight="1" s="28">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Link para descargar archvivo ICS del  Calendario Mundial 2026 para Outlook o iPhone:</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1" s="16">
-      <c r="B3" s="22" t="inlineStr">
+    <row r="3" ht="45" customHeight="1" s="28">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>https://calendar.google.com/calendar/ical/611d68120c62daa60625df08296c3333f1416dbeb64241045a3c75dd62f175d8%40group.calendar.google.com/public/basic.ics</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="26.25" customHeight="1" s="16">
-      <c r="B6" s="18" t="inlineStr">
+    <row r="6" ht="26.25" customHeight="1" s="28">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Calendario para Google Calendar</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="23" t="n"/>
-    </row>
-    <row r="8" ht="60" customHeight="1" s="16">
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B7" s="17" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1" s="28">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>https://calendar.google.com/calendar/u/4?cid=NjExZDY4MTIwYzYyZGFhNjA2MjVkZjA4Mjk2YzMzMzNmMTQxNmRiZWI2NDI0MTA0NWEzYzc1ZGQ2MmYxNzVkOEBncm91cC5jYWxlbmRhci5nb29nbGUuY29t</t>
         </is>
@@ -15788,7 +15855,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -16282,7 +16349,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I495"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Insert separator column J in Grupos sheet
</commit_message>
<xml_diff>
--- a/Quiniela_Mundial_2026_Final_vacia.xlsx
+++ b/Quiniela_Mundial_2026_Final_vacia.xlsx
@@ -372,12 +372,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -389,14 +390,80 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -692,93 +759,93 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="148" customWidth="1" style="29" min="1" max="1"/>
-    <col width="75.42578125" customWidth="1" style="29" min="7" max="7"/>
+    <col width="148" customWidth="1" style="30" min="1" max="1"/>
+    <col width="75.42578125" customWidth="1" style="30" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.75" customHeight="1" s="29">
+    <row r="1" ht="33.75" customHeight="1" s="30">
       <c r="A1" s="10" t="inlineStr">
         <is>
           <t>QUINIELA MUNDIAL DE FÚTBOL 2026 - 100% AUTOMATIZADA</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="29">
+    <row r="3" ht="16.5" customHeight="1" s="30">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>La Copa Mundial de la FIFA 26™ tendrá 48 equipos divididos en doce grupos con cuatro equipos cada uno.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="29">
+    <row r="4" ht="16.5" customHeight="1" s="30">
       <c r="A4" s="1" t="n"/>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="29">
+    <row r="5" ht="16.5" customHeight="1" s="30">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Los dos primeros de cada grupo y los ocho mejores terceros avanzarán a los dieciseisavos de final.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="29">
+    <row r="6" ht="16.5" customHeight="1" s="30">
       <c r="A6" s="1" t="n"/>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="29">
+    <row r="7" ht="16.5" customHeight="1" s="30">
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Los equipos que lleguen a la final del 19 de julio habrán disputado ocho partidos, uno más que en Catar 2022.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="29">
+    <row r="8" ht="16.5" customHeight="1" s="30">
       <c r="A8" s="1" t="n"/>
     </row>
-    <row r="9" ht="33" customHeight="1" s="29">
+    <row r="9" ht="33" customHeight="1" s="30">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>El nuevo esquema establece que los equipos que lleguen a la final, a jugarse el domingo 19 de julio, tendrán que haber atravesado ocho partidos, uno más de los disputados en la última Copa Mundial de la FIFA 2022™, en Catar.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="29">
+    <row r="10" ht="16.5" customHeight="1" s="30">
       <c r="A10" s="1" t="n"/>
     </row>
-    <row r="11" ht="26.25" customHeight="1" s="29">
+    <row r="11" ht="26.25" customHeight="1" s="30">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>CÓMO FUNCIONA:</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="29">
+    <row r="13" ht="16.5" customHeight="1" s="30">
       <c r="A13" s="1" t="inlineStr">
         <is>
           <t>1. Pestaña 'Grupos': Ingresa los resultados. Las tablas se calculan en tiempo real.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="29">
+    <row r="14" ht="16.5" customHeight="1" s="30">
       <c r="A14" s="1" t="inlineStr">
         <is>
           <t>2. Pestaña 'Eliminatorias': Al ir llenando, verás cómo los nombres se auto-completan gracias a la corrección del motor.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="29">
+    <row r="15" ht="16.5" customHeight="1" s="30">
       <c r="A15" s="1" t="inlineStr">
         <is>
           <t>3. Puedes empezar a llenar y los líderes de cada grupo aparecerán de inmediato.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="29">
+    <row r="16" ht="16.5" customHeight="1" s="30">
       <c r="A16" s="27" t="inlineStr">
         <is>
           <t>4. Guarda tu quiniela con tu nombre y apellido. Ejemplo: Quiniela_Cristiano_Ronaldo.xlsx, Quiniela_Lionel_Messi.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="26.25" customHeight="1" s="29">
+    <row r="17" ht="26.25" customHeight="1" s="30">
       <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Sistema de Puntuación</t>
@@ -788,7 +855,7 @@
     <row r="18">
       <c r="A18" s="7" t="n"/>
     </row>
-    <row r="19" ht="15.75" customHeight="1" s="29">
+    <row r="19" ht="15.75" customHeight="1" s="30">
       <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Fase de Grupos:</t>
@@ -812,7 +879,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="29">
+    <row r="24" ht="15.75" customHeight="1" s="30">
       <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Fase Eliminatoria:</t>
@@ -878,7 +945,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1" s="29">
+    <row r="35" ht="15.75" customHeight="1" s="30">
       <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Podio (Predicciones Finales):</t>
@@ -945,50 +1012,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H212"/>
+  <dimension ref="A1:I212"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <cols>
+    <col width="9.5703125" bestFit="1" customWidth="1" style="30" min="1" max="1"/>
+    <col width="28.85546875" bestFit="1" customWidth="1" style="30" min="2" max="2"/>
+    <col width="8.28515625" bestFit="1" customWidth="1" style="30" min="3" max="3"/>
+    <col width="16.140625" bestFit="1" customWidth="1" style="30" min="4" max="4"/>
+    <col width="19.5703125" bestFit="1" customWidth="1" style="30" min="5" max="5"/>
+    <col width="28.140625" bestFit="1" customWidth="1" style="30" min="6" max="6"/>
+    <col width="19.42578125" bestFit="1" customWidth="1" style="30" min="7" max="7"/>
+    <col width="15.7109375" bestFit="1" customWidth="1" style="30" min="8" max="8"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="16.5" customHeight="1" s="30">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Posición</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Selección</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Código</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Puntos Totales</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Puntos Anteriores</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Diferencia de Puntos (+/-)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Cambio de Puesto</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Confederación</t>
         </is>
       </c>
+      <c r="I1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -8175,30 +8253,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T99"/>
+  <dimension ref="A1:U99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="29" min="1" max="1"/>
-    <col width="16" customWidth="1" style="29" min="3" max="3"/>
-    <col width="16" customWidth="1" style="29" min="7" max="7"/>
-    <col width="35" customWidth="1" style="29" min="9" max="9"/>
-    <col width="16" customWidth="1" style="29" min="11" max="11"/>
+    <col width="8" customWidth="1" style="30" min="1" max="1"/>
+    <col width="16" customWidth="1" style="30" min="3" max="3"/>
+    <col width="16" customWidth="1" style="30" min="7" max="7"/>
+    <col width="35" customWidth="1" style="30" min="9" max="9"/>
+    <col width="3" customWidth="1" style="30" min="10" max="10"/>
+    <col width="16" customWidth="1" style="30" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="29">
+    <row r="1" ht="15" customHeight="1" s="30">
       <c r="A1" s="31" t="inlineStr">
         <is>
           <t>PARTIDOS DE GRUPOS</t>
         </is>
       </c>
-      <c r="J1" s="28" t="inlineStr">
+      <c r="I1" s="2" t="n"/>
+      <c r="K1" s="32" t="inlineStr">
         <is>
           <t>TABLAS DE POSICIONES (AUTOMÁTICAS)</t>
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="4" ht="16.5" customHeight="1" s="29">
+    <row r="2" ht="16.5" customHeight="1" s="30">
+      <c r="I2" s="2" t="n"/>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="16.5" customHeight="1" s="30">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ID</t>
@@ -8244,70 +8327,70 @@
           <t>Fecha y Hora</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>PJ</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>PG</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>PE</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>PP</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>GF</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>DIF</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>PTS</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="U4" s="3" t="inlineStr">
         <is>
           <t>SCORE TIEBREAK</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18.75" customHeight="1" s="29">
-      <c r="A5" s="30" t="inlineStr">
+    <row r="5" ht="18.75" customHeight="1" s="30">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>GRUPO A</t>
         </is>
       </c>
-      <c r="I5" s="35" t="n"/>
-      <c r="J5" s="30" t="inlineStr">
+      <c r="I5" s="28" t="n"/>
+      <c r="K5" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO A</t>
         </is>
@@ -8340,49 +8423,49 @@
           <t>Jueves, 11 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>México</t>
         </is>
       </c>
-      <c r="L6">
+      <c r="M6">
         <f>IF(ISNUMBER(D6),1,0)+IF(ISNUMBER(D8),1,0)+IF(ISNUMBER(F10),1,0)</f>
         <v/>
       </c>
-      <c r="M6">
+      <c r="N6">
         <f>IF(AND(ISNUMBER(D6),ISNUMBER(F6),D6&gt;F6),1,0)+IF(AND(ISNUMBER(D8),ISNUMBER(F8),D8&gt;F8),1,0)+IF(AND(ISNUMBER(F10),ISNUMBER(D10),F10&gt;D10),1,0)</f>
         <v/>
       </c>
-      <c r="N6">
+      <c r="O6">
         <f>IF(AND(ISNUMBER(D6),ISNUMBER(F6),D6=F6),1,0)+IF(AND(ISNUMBER(D8),ISNUMBER(F8),D8=F8),1,0)+IF(AND(ISNUMBER(F10),ISNUMBER(D10),F10=D10),1,0)</f>
         <v/>
       </c>
-      <c r="O6">
+      <c r="P6">
         <f>IF(AND(ISNUMBER(D6),ISNUMBER(F6),D6&lt;F6),1,0)+IF(AND(ISNUMBER(D8),ISNUMBER(F8),D8&lt;F8),1,0)+IF(AND(ISNUMBER(F10),ISNUMBER(D10),F10&lt;D10),1,0)</f>
         <v/>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <f>IF(ISNUMBER(D6),D6,0)+IF(ISNUMBER(D8),D8,0)+IF(ISNUMBER(F10),F10,0)</f>
         <v/>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <f>IF(ISNUMBER(F6),F6,0)+IF(ISNUMBER(F8),F8,0)+IF(ISNUMBER(D10),D10,0)</f>
         <v/>
       </c>
-      <c r="R6">
+      <c r="S6">
         <f>P6-Q6</f>
         <v/>
       </c>
-      <c r="S6">
+      <c r="T6">
         <f>M6*3+N6</f>
         <v/>
       </c>
-      <c r="T6">
+      <c r="U6">
         <f>S6*100000000 + (R6+100)*100000 + P6*1000 + IFERROR(VLOOKUP(K6, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -8414,49 +8497,49 @@
           <t>Jueves, 11 de junio 2026 - 20:00</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Sudáfrica</t>
         </is>
       </c>
-      <c r="L7">
+      <c r="M7">
         <f>IF(ISNUMBER(F6),1,0)+IF(ISNUMBER(D9),1,0)+IF(ISNUMBER(D11),1,0)</f>
         <v/>
       </c>
-      <c r="M7">
+      <c r="N7">
         <f>IF(AND(ISNUMBER(F6),ISNUMBER(D6),F6&gt;D6),1,0)+IF(AND(ISNUMBER(D9),ISNUMBER(F9),D9&gt;F9),1,0)+IF(AND(ISNUMBER(D11),ISNUMBER(F11),D11&gt;F11),1,0)</f>
         <v/>
       </c>
-      <c r="N7">
+      <c r="O7">
         <f>IF(AND(ISNUMBER(F6),ISNUMBER(D6),F6=D6),1,0)+IF(AND(ISNUMBER(D9),ISNUMBER(F9),D9=F9),1,0)+IF(AND(ISNUMBER(D11),ISNUMBER(F11),D11=F11),1,0)</f>
         <v/>
       </c>
-      <c r="O7">
+      <c r="P7">
         <f>IF(AND(ISNUMBER(F6),ISNUMBER(D6),F6&lt;D6),1,0)+IF(AND(ISNUMBER(D9),ISNUMBER(F9),D9&lt;F9),1,0)+IF(AND(ISNUMBER(D11),ISNUMBER(F11),D11&lt;F11),1,0)</f>
         <v/>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <f>IF(ISNUMBER(F6),F6,0)+IF(ISNUMBER(D9),D9,0)+IF(ISNUMBER(D11),D11,0)</f>
         <v/>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <f>IF(ISNUMBER(D6),D6,0)+IF(ISNUMBER(F9),F9,0)+IF(ISNUMBER(F11),F11,0)</f>
         <v/>
       </c>
-      <c r="R7">
+      <c r="S7">
         <f>P7-Q7</f>
         <v/>
       </c>
-      <c r="S7">
+      <c r="T7">
         <f>M7*3+N7</f>
         <v/>
       </c>
-      <c r="T7">
+      <c r="U7">
         <f>S7*100000000 + (R7+100)*100000 + P7*1000 + IFERROR(VLOOKUP(K7, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -8488,49 +8571,49 @@
           <t>Jueves, 18 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Corea del Sur</t>
         </is>
       </c>
-      <c r="L8">
+      <c r="M8">
         <f>IF(ISNUMBER(D7),1,0)+IF(ISNUMBER(F8),1,0)+IF(ISNUMBER(F11),1,0)</f>
         <v/>
       </c>
-      <c r="M8">
+      <c r="N8">
         <f>IF(AND(ISNUMBER(D7),ISNUMBER(F7),D7&gt;F7),1,0)+IF(AND(ISNUMBER(F8),ISNUMBER(D8),F8&gt;D8),1,0)+IF(AND(ISNUMBER(F11),ISNUMBER(D11),F11&gt;D11),1,0)</f>
         <v/>
       </c>
-      <c r="N8">
+      <c r="O8">
         <f>IF(AND(ISNUMBER(D7),ISNUMBER(F7),D7=F7),1,0)+IF(AND(ISNUMBER(F8),ISNUMBER(D8),F8=D8),1,0)+IF(AND(ISNUMBER(F11),ISNUMBER(D11),F11=D11),1,0)</f>
         <v/>
       </c>
-      <c r="O8">
+      <c r="P8">
         <f>IF(AND(ISNUMBER(D7),ISNUMBER(F7),D7&lt;F7),1,0)+IF(AND(ISNUMBER(F8),ISNUMBER(D8),F8&lt;D8),1,0)+IF(AND(ISNUMBER(F11),ISNUMBER(D11),F11&lt;D11),1,0)</f>
         <v/>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <f>IF(ISNUMBER(D7),D7,0)+IF(ISNUMBER(F8),F8,0)+IF(ISNUMBER(F11),F11,0)</f>
         <v/>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <f>IF(ISNUMBER(F7),F7,0)+IF(ISNUMBER(D8),D8,0)+IF(ISNUMBER(D11),D11,0)</f>
         <v/>
       </c>
-      <c r="R8">
+      <c r="S8">
         <f>P8-Q8</f>
         <v/>
       </c>
-      <c r="S8">
+      <c r="T8">
         <f>M8*3+N8</f>
         <v/>
       </c>
-      <c r="T8">
+      <c r="U8">
         <f>S8*100000000 + (R8+100)*100000 + P8*1000 + IFERROR(VLOOKUP(K8, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -8562,49 +8645,49 @@
           <t>Jueves, 18 de junio 2026 - 10:00</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Chequia</t>
         </is>
       </c>
-      <c r="L9">
+      <c r="M9">
         <f>IF(ISNUMBER(F7),1,0)+IF(ISNUMBER(F9),1,0)+IF(ISNUMBER(D10),1,0)</f>
         <v/>
       </c>
-      <c r="M9">
+      <c r="N9">
         <f>IF(AND(ISNUMBER(F7),ISNUMBER(D7),F7&gt;D7),1,0)+IF(AND(ISNUMBER(F9),ISNUMBER(D9),F9&gt;D9),1,0)+IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10&gt;F10),1,0)</f>
         <v/>
       </c>
-      <c r="N9">
+      <c r="O9">
         <f>IF(AND(ISNUMBER(F7),ISNUMBER(D7),F7=D7),1,0)+IF(AND(ISNUMBER(F9),ISNUMBER(D9),F9=D9),1,0)+IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10=F10),1,0)</f>
         <v/>
       </c>
-      <c r="O9">
+      <c r="P9">
         <f>IF(AND(ISNUMBER(F7),ISNUMBER(D7),F7&lt;D7),1,0)+IF(AND(ISNUMBER(F9),ISNUMBER(D9),F9&lt;D9),1,0)+IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10&lt;F10),1,0)</f>
         <v/>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <f>IF(ISNUMBER(F7),F7,0)+IF(ISNUMBER(F9),F9,0)+IF(ISNUMBER(D10),D10,0)</f>
         <v/>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <f>IF(ISNUMBER(D7),D7,0)+IF(ISNUMBER(D9),D9,0)+IF(ISNUMBER(F10),F10,0)</f>
         <v/>
       </c>
-      <c r="R9">
+      <c r="S9">
         <f>P9-Q9</f>
         <v/>
       </c>
-      <c r="S9">
+      <c r="T9">
         <f>M9*3+N9</f>
         <v/>
       </c>
-      <c r="T9">
+      <c r="U9">
         <f>S9*100000000 + (R9+100)*100000 + P9*1000 + IFERROR(VLOOKUP(K9, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -8637,7 +8720,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18.75" customHeight="1" s="29">
+    <row r="11" ht="18.75" customHeight="1" s="30">
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Sudáfrica</t>
@@ -8664,110 +8747,110 @@
           <t>Miércoles, 24 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J11" s="30" t="inlineStr">
+      <c r="K11" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO B</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Canadá</t>
         </is>
       </c>
-      <c r="L12">
+      <c r="M12">
         <f>IF(ISNUMBER(D14),1,0)+IF(ISNUMBER(D16),1,0)+IF(ISNUMBER(F18),1,0)</f>
         <v/>
       </c>
-      <c r="M12">
+      <c r="N12">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(F14),D14&gt;F14),1,0)+IF(AND(ISNUMBER(D16),ISNUMBER(F16),D16&gt;F16),1,0)+IF(AND(ISNUMBER(F18),ISNUMBER(D18),F18&gt;D18),1,0)</f>
         <v/>
       </c>
-      <c r="N12">
+      <c r="O12">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(F14),D14=F14),1,0)+IF(AND(ISNUMBER(D16),ISNUMBER(F16),D16=F16),1,0)+IF(AND(ISNUMBER(F18),ISNUMBER(D18),F18=D18),1,0)</f>
         <v/>
       </c>
-      <c r="O12">
+      <c r="P12">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(F14),D14&lt;F14),1,0)+IF(AND(ISNUMBER(D16),ISNUMBER(F16),D16&lt;F16),1,0)+IF(AND(ISNUMBER(F18),ISNUMBER(D18),F18&lt;D18),1,0)</f>
         <v/>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <f>IF(ISNUMBER(D14),D14,0)+IF(ISNUMBER(D16),D16,0)+IF(ISNUMBER(F18),F18,0)</f>
         <v/>
       </c>
-      <c r="Q12">
+      <c r="R12">
         <f>IF(ISNUMBER(F14),F14,0)+IF(ISNUMBER(F16),F16,0)+IF(ISNUMBER(D18),D18,0)</f>
         <v/>
       </c>
-      <c r="R12">
+      <c r="S12">
         <f>P12-Q12</f>
         <v/>
       </c>
-      <c r="S12">
+      <c r="T12">
         <f>M12*3+N12</f>
         <v/>
       </c>
-      <c r="T12">
+      <c r="U12">
         <f>S12*100000000 + (R12+100)*100000 + P12*1000 + IFERROR(VLOOKUP(K12, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="18.75" customHeight="1" s="29">
-      <c r="A13" s="30" t="inlineStr">
+    <row r="13" ht="18.75" customHeight="1" s="30">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>GRUPO B</t>
         </is>
       </c>
-      <c r="I13" s="35" t="n"/>
-      <c r="J13" t="inlineStr">
+      <c r="I13" s="28" t="n"/>
+      <c r="K13" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Bosnia y Herze.</t>
         </is>
       </c>
-      <c r="L13">
+      <c r="M13">
         <f>IF(ISNUMBER(F14),1,0)+IF(ISNUMBER(D17),1,0)+IF(ISNUMBER(D19),1,0)</f>
         <v/>
       </c>
-      <c r="M13">
+      <c r="N13">
         <f>IF(AND(ISNUMBER(F14),ISNUMBER(D14),F14&gt;D14),1,0)+IF(AND(ISNUMBER(D17),ISNUMBER(F17),D17&gt;F17),1,0)+IF(AND(ISNUMBER(D19),ISNUMBER(F19),D19&gt;F19),1,0)</f>
         <v/>
       </c>
-      <c r="N13">
+      <c r="O13">
         <f>IF(AND(ISNUMBER(F14),ISNUMBER(D14),F14=D14),1,0)+IF(AND(ISNUMBER(D17),ISNUMBER(F17),D17=F17),1,0)+IF(AND(ISNUMBER(D19),ISNUMBER(F19),D19=F19),1,0)</f>
         <v/>
       </c>
-      <c r="O13">
+      <c r="P13">
         <f>IF(AND(ISNUMBER(F14),ISNUMBER(D14),F14&lt;D14),1,0)+IF(AND(ISNUMBER(D17),ISNUMBER(F17),D17&lt;F17),1,0)+IF(AND(ISNUMBER(D19),ISNUMBER(F19),D19&lt;F19),1,0)</f>
         <v/>
       </c>
-      <c r="P13">
+      <c r="Q13">
         <f>IF(ISNUMBER(F14),F14,0)+IF(ISNUMBER(D17),D17,0)+IF(ISNUMBER(D19),D19,0)</f>
         <v/>
       </c>
-      <c r="Q13">
+      <c r="R13">
         <f>IF(ISNUMBER(D14),D14,0)+IF(ISNUMBER(F17),F17,0)+IF(ISNUMBER(F19),F19,0)</f>
         <v/>
       </c>
-      <c r="R13">
+      <c r="S13">
         <f>P13-Q13</f>
         <v/>
       </c>
-      <c r="S13">
+      <c r="T13">
         <f>M13*3+N13</f>
         <v/>
       </c>
-      <c r="T13">
+      <c r="U13">
         <f>S13*100000000 + (R13+100)*100000 + P13*1000 + IFERROR(VLOOKUP(K13, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -8799,49 +8882,49 @@
           <t>Viernes, 12 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Qatar</t>
         </is>
       </c>
-      <c r="L14">
+      <c r="M14">
         <f>IF(ISNUMBER(D15),1,0)+IF(ISNUMBER(F16),1,0)+IF(ISNUMBER(F19),1,0)</f>
         <v/>
       </c>
-      <c r="M14">
+      <c r="N14">
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(F15),D15&gt;F15),1,0)+IF(AND(ISNUMBER(F16),ISNUMBER(D16),F16&gt;D16),1,0)+IF(AND(ISNUMBER(F19),ISNUMBER(D19),F19&gt;D19),1,0)</f>
         <v/>
       </c>
-      <c r="N14">
+      <c r="O14">
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(F15),D15=F15),1,0)+IF(AND(ISNUMBER(F16),ISNUMBER(D16),F16=D16),1,0)+IF(AND(ISNUMBER(F19),ISNUMBER(D19),F19=D19),1,0)</f>
         <v/>
       </c>
-      <c r="O14">
+      <c r="P14">
         <f>IF(AND(ISNUMBER(D15),ISNUMBER(F15),D15&lt;F15),1,0)+IF(AND(ISNUMBER(F16),ISNUMBER(D16),F16&lt;D16),1,0)+IF(AND(ISNUMBER(F19),ISNUMBER(D19),F19&lt;D19),1,0)</f>
         <v/>
       </c>
-      <c r="P14">
+      <c r="Q14">
         <f>IF(ISNUMBER(D15),D15,0)+IF(ISNUMBER(F16),F16,0)+IF(ISNUMBER(F19),F19,0)</f>
         <v/>
       </c>
-      <c r="Q14">
+      <c r="R14">
         <f>IF(ISNUMBER(F15),F15,0)+IF(ISNUMBER(D16),D16,0)+IF(ISNUMBER(D19),D19,0)</f>
         <v/>
       </c>
-      <c r="R14">
+      <c r="S14">
         <f>P14-Q14</f>
         <v/>
       </c>
-      <c r="S14">
+      <c r="T14">
         <f>M14*3+N14</f>
         <v/>
       </c>
-      <c r="T14">
+      <c r="U14">
         <f>S14*100000000 + (R14+100)*100000 + P14*1000 + IFERROR(VLOOKUP(K14, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -8873,49 +8956,49 @@
           <t>Sábado, 13 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Suiza</t>
         </is>
       </c>
-      <c r="L15">
+      <c r="M15">
         <f>IF(ISNUMBER(F15),1,0)+IF(ISNUMBER(F17),1,0)+IF(ISNUMBER(D18),1,0)</f>
         <v/>
       </c>
-      <c r="M15">
+      <c r="N15">
         <f>IF(AND(ISNUMBER(F15),ISNUMBER(D15),F15&gt;D15),1,0)+IF(AND(ISNUMBER(F17),ISNUMBER(D17),F17&gt;D17),1,0)+IF(AND(ISNUMBER(D18),ISNUMBER(F18),D18&gt;F18),1,0)</f>
         <v/>
       </c>
-      <c r="N15">
+      <c r="O15">
         <f>IF(AND(ISNUMBER(F15),ISNUMBER(D15),F15=D15),1,0)+IF(AND(ISNUMBER(F17),ISNUMBER(D17),F17=D17),1,0)+IF(AND(ISNUMBER(D18),ISNUMBER(F18),D18=F18),1,0)</f>
         <v/>
       </c>
-      <c r="O15">
+      <c r="P15">
         <f>IF(AND(ISNUMBER(F15),ISNUMBER(D15),F15&lt;D15),1,0)+IF(AND(ISNUMBER(F17),ISNUMBER(D17),F17&lt;D17),1,0)+IF(AND(ISNUMBER(D18),ISNUMBER(F18),D18&lt;F18),1,0)</f>
         <v/>
       </c>
-      <c r="P15">
+      <c r="Q15">
         <f>IF(ISNUMBER(F15),F15,0)+IF(ISNUMBER(F17),F17,0)+IF(ISNUMBER(D18),D18,0)</f>
         <v/>
       </c>
-      <c r="Q15">
+      <c r="R15">
         <f>IF(ISNUMBER(D15),D15,0)+IF(ISNUMBER(D17),D17,0)+IF(ISNUMBER(F18),F18,0)</f>
         <v/>
       </c>
-      <c r="R15">
+      <c r="S15">
         <f>P15-Q15</f>
         <v/>
       </c>
-      <c r="S15">
+      <c r="T15">
         <f>M15*3+N15</f>
         <v/>
       </c>
-      <c r="T15">
+      <c r="U15">
         <f>S15*100000000 + (R15+100)*100000 + P15*1000 + IFERROR(VLOOKUP(K15, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -8948,7 +9031,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="18.75" customHeight="1" s="29">
+    <row r="17" ht="18.75" customHeight="1" s="30">
       <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Bosnia y Herze.</t>
@@ -8975,7 +9058,7 @@
           <t>Jueves, 18 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J17" s="30" t="inlineStr">
+      <c r="K17" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO C</t>
         </is>
@@ -9008,49 +9091,49 @@
           <t>Miércoles, 24 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Brasil</t>
         </is>
       </c>
-      <c r="L18">
+      <c r="M18">
         <f>IF(ISNUMBER(D22),1,0)+IF(ISNUMBER(D24),1,0)+IF(ISNUMBER(F26),1,0)</f>
         <v/>
       </c>
-      <c r="M18">
+      <c r="N18">
         <f>IF(AND(ISNUMBER(D22),ISNUMBER(F22),D22&gt;F22),1,0)+IF(AND(ISNUMBER(D24),ISNUMBER(F24),D24&gt;F24),1,0)+IF(AND(ISNUMBER(F26),ISNUMBER(D26),F26&gt;D26),1,0)</f>
         <v/>
       </c>
-      <c r="N18">
+      <c r="O18">
         <f>IF(AND(ISNUMBER(D22),ISNUMBER(F22),D22=F22),1,0)+IF(AND(ISNUMBER(D24),ISNUMBER(F24),D24=F24),1,0)+IF(AND(ISNUMBER(F26),ISNUMBER(D26),F26=D26),1,0)</f>
         <v/>
       </c>
-      <c r="O18">
+      <c r="P18">
         <f>IF(AND(ISNUMBER(D22),ISNUMBER(F22),D22&lt;F22),1,0)+IF(AND(ISNUMBER(D24),ISNUMBER(F24),D24&lt;F24),1,0)+IF(AND(ISNUMBER(F26),ISNUMBER(D26),F26&lt;D26),1,0)</f>
         <v/>
       </c>
-      <c r="P18">
+      <c r="Q18">
         <f>IF(ISNUMBER(D22),D22,0)+IF(ISNUMBER(D24),D24,0)+IF(ISNUMBER(F26),F26,0)</f>
         <v/>
       </c>
-      <c r="Q18">
+      <c r="R18">
         <f>IF(ISNUMBER(F22),F22,0)+IF(ISNUMBER(F24),F24,0)+IF(ISNUMBER(D26),D26,0)</f>
         <v/>
       </c>
-      <c r="R18">
+      <c r="S18">
         <f>P18-Q18</f>
         <v/>
       </c>
-      <c r="S18">
+      <c r="T18">
         <f>M18*3+N18</f>
         <v/>
       </c>
-      <c r="T18">
+      <c r="U18">
         <f>S18*100000000 + (R18+100)*100000 + P18*1000 + IFERROR(VLOOKUP(K18, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9082,151 +9165,151 @@
           <t>Miércoles, 24 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Marruecos</t>
         </is>
       </c>
-      <c r="L19">
+      <c r="M19">
         <f>IF(ISNUMBER(F22),1,0)+IF(ISNUMBER(D25),1,0)+IF(ISNUMBER(D27),1,0)</f>
         <v/>
       </c>
-      <c r="M19">
+      <c r="N19">
         <f>IF(AND(ISNUMBER(F22),ISNUMBER(D22),F22&gt;D22),1,0)+IF(AND(ISNUMBER(D25),ISNUMBER(F25),D25&gt;F25),1,0)+IF(AND(ISNUMBER(D27),ISNUMBER(F27),D27&gt;F27),1,0)</f>
         <v/>
       </c>
-      <c r="N19">
+      <c r="O19">
         <f>IF(AND(ISNUMBER(F22),ISNUMBER(D22),F22=D22),1,0)+IF(AND(ISNUMBER(D25),ISNUMBER(F25),D25=F25),1,0)+IF(AND(ISNUMBER(D27),ISNUMBER(F27),D27=F27),1,0)</f>
         <v/>
       </c>
-      <c r="O19">
+      <c r="P19">
         <f>IF(AND(ISNUMBER(F22),ISNUMBER(D22),F22&lt;D22),1,0)+IF(AND(ISNUMBER(D25),ISNUMBER(F25),D25&lt;F25),1,0)+IF(AND(ISNUMBER(D27),ISNUMBER(F27),D27&lt;F27),1,0)</f>
         <v/>
       </c>
-      <c r="P19">
+      <c r="Q19">
         <f>IF(ISNUMBER(F22),F22,0)+IF(ISNUMBER(D25),D25,0)+IF(ISNUMBER(D27),D27,0)</f>
         <v/>
       </c>
-      <c r="Q19">
+      <c r="R19">
         <f>IF(ISNUMBER(D22),D22,0)+IF(ISNUMBER(F25),F25,0)+IF(ISNUMBER(F27),F27,0)</f>
         <v/>
       </c>
-      <c r="R19">
+      <c r="S19">
         <f>P19-Q19</f>
         <v/>
       </c>
-      <c r="S19">
+      <c r="T19">
         <f>M19*3+N19</f>
         <v/>
       </c>
-      <c r="T19">
+      <c r="U19">
         <f>S19*100000000 + (R19+100)*100000 + P19*1000 + IFERROR(VLOOKUP(K19, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>Haití</t>
         </is>
       </c>
-      <c r="L20">
+      <c r="M20">
         <f>IF(ISNUMBER(D23),1,0)+IF(ISNUMBER(F24),1,0)+IF(ISNUMBER(F27),1,0)</f>
         <v/>
       </c>
-      <c r="M20">
+      <c r="N20">
         <f>IF(AND(ISNUMBER(D23),ISNUMBER(F23),D23&gt;F23),1,0)+IF(AND(ISNUMBER(F24),ISNUMBER(D24),F24&gt;D24),1,0)+IF(AND(ISNUMBER(F27),ISNUMBER(D27),F27&gt;D27),1,0)</f>
         <v/>
       </c>
-      <c r="N20">
+      <c r="O20">
         <f>IF(AND(ISNUMBER(D23),ISNUMBER(F23),D23=F23),1,0)+IF(AND(ISNUMBER(F24),ISNUMBER(D24),F24=D24),1,0)+IF(AND(ISNUMBER(F27),ISNUMBER(D27),F27=D27),1,0)</f>
         <v/>
       </c>
-      <c r="O20">
+      <c r="P20">
         <f>IF(AND(ISNUMBER(D23),ISNUMBER(F23),D23&lt;F23),1,0)+IF(AND(ISNUMBER(F24),ISNUMBER(D24),F24&lt;D24),1,0)+IF(AND(ISNUMBER(F27),ISNUMBER(D27),F27&lt;D27),1,0)</f>
         <v/>
       </c>
-      <c r="P20">
+      <c r="Q20">
         <f>IF(ISNUMBER(D23),D23,0)+IF(ISNUMBER(F24),F24,0)+IF(ISNUMBER(F27),F27,0)</f>
         <v/>
       </c>
-      <c r="Q20">
+      <c r="R20">
         <f>IF(ISNUMBER(F23),F23,0)+IF(ISNUMBER(D24),D24,0)+IF(ISNUMBER(D27),D27,0)</f>
         <v/>
       </c>
-      <c r="R20">
+      <c r="S20">
         <f>P20-Q20</f>
         <v/>
       </c>
-      <c r="S20">
+      <c r="T20">
         <f>M20*3+N20</f>
         <v/>
       </c>
-      <c r="T20">
+      <c r="U20">
         <f>S20*100000000 + (R20+100)*100000 + P20*1000 + IFERROR(VLOOKUP(K20, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="18.75" customHeight="1" s="29">
-      <c r="A21" s="30" t="inlineStr">
+    <row r="21" ht="18.75" customHeight="1" s="30">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>GRUPO C</t>
         </is>
       </c>
-      <c r="I21" s="35" t="n"/>
-      <c r="J21" t="inlineStr">
+      <c r="I21" s="28" t="n"/>
+      <c r="K21" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>Escocia</t>
         </is>
       </c>
-      <c r="L21">
+      <c r="M21">
         <f>IF(ISNUMBER(F23),1,0)+IF(ISNUMBER(F25),1,0)+IF(ISNUMBER(D26),1,0)</f>
         <v/>
       </c>
-      <c r="M21">
+      <c r="N21">
         <f>IF(AND(ISNUMBER(F23),ISNUMBER(D23),F23&gt;D23),1,0)+IF(AND(ISNUMBER(F25),ISNUMBER(D25),F25&gt;D25),1,0)+IF(AND(ISNUMBER(D26),ISNUMBER(F26),D26&gt;F26),1,0)</f>
         <v/>
       </c>
-      <c r="N21">
+      <c r="O21">
         <f>IF(AND(ISNUMBER(F23),ISNUMBER(D23),F23=D23),1,0)+IF(AND(ISNUMBER(F25),ISNUMBER(D25),F25=D25),1,0)+IF(AND(ISNUMBER(D26),ISNUMBER(F26),D26=F26),1,0)</f>
         <v/>
       </c>
-      <c r="O21">
+      <c r="P21">
         <f>IF(AND(ISNUMBER(F23),ISNUMBER(D23),F23&lt;D23),1,0)+IF(AND(ISNUMBER(F25),ISNUMBER(D25),F25&lt;D25),1,0)+IF(AND(ISNUMBER(D26),ISNUMBER(F26),D26&lt;F26),1,0)</f>
         <v/>
       </c>
-      <c r="P21">
+      <c r="Q21">
         <f>IF(ISNUMBER(F23),F23,0)+IF(ISNUMBER(F25),F25,0)+IF(ISNUMBER(D26),D26,0)</f>
         <v/>
       </c>
-      <c r="Q21">
+      <c r="R21">
         <f>IF(ISNUMBER(D23),D23,0)+IF(ISNUMBER(D25),D25,0)+IF(ISNUMBER(F26),F26,0)</f>
         <v/>
       </c>
-      <c r="R21">
+      <c r="S21">
         <f>P21-Q21</f>
         <v/>
       </c>
-      <c r="S21">
+      <c r="T21">
         <f>M21*3+N21</f>
         <v/>
       </c>
-      <c r="T21">
+      <c r="U21">
         <f>S21*100000000 + (R21+100)*100000 + P21*1000 + IFERROR(VLOOKUP(K21, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9259,7 +9342,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="18.75" customHeight="1" s="29">
+    <row r="23" ht="18.75" customHeight="1" s="30">
       <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Haití</t>
@@ -9286,7 +9369,7 @@
           <t>Sábado, 13 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J23" s="30" t="inlineStr">
+      <c r="K23" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO D</t>
         </is>
@@ -9319,49 +9402,49 @@
           <t>Viernes, 19 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>Estados Unidos</t>
         </is>
       </c>
-      <c r="L24">
+      <c r="M24">
         <f>IF(ISNUMBER(D30),1,0)+IF(ISNUMBER(D32),1,0)+IF(ISNUMBER(F34),1,0)</f>
         <v/>
       </c>
-      <c r="M24">
+      <c r="N24">
         <f>IF(AND(ISNUMBER(D30),ISNUMBER(F30),D30&gt;F30),1,0)+IF(AND(ISNUMBER(D32),ISNUMBER(F32),D32&gt;F32),1,0)+IF(AND(ISNUMBER(F34),ISNUMBER(D34),F34&gt;D34),1,0)</f>
         <v/>
       </c>
-      <c r="N24">
+      <c r="O24">
         <f>IF(AND(ISNUMBER(D30),ISNUMBER(F30),D30=F30),1,0)+IF(AND(ISNUMBER(D32),ISNUMBER(F32),D32=F32),1,0)+IF(AND(ISNUMBER(F34),ISNUMBER(D34),F34=D34),1,0)</f>
         <v/>
       </c>
-      <c r="O24">
+      <c r="P24">
         <f>IF(AND(ISNUMBER(D30),ISNUMBER(F30),D30&lt;F30),1,0)+IF(AND(ISNUMBER(D32),ISNUMBER(F32),D32&lt;F32),1,0)+IF(AND(ISNUMBER(F34),ISNUMBER(D34),F34&lt;D34),1,0)</f>
         <v/>
       </c>
-      <c r="P24">
+      <c r="Q24">
         <f>IF(ISNUMBER(D30),D30,0)+IF(ISNUMBER(D32),D32,0)+IF(ISNUMBER(F34),F34,0)</f>
         <v/>
       </c>
-      <c r="Q24">
+      <c r="R24">
         <f>IF(ISNUMBER(F30),F30,0)+IF(ISNUMBER(F32),F32,0)+IF(ISNUMBER(D34),D34,0)</f>
         <v/>
       </c>
-      <c r="R24">
+      <c r="S24">
         <f>P24-Q24</f>
         <v/>
       </c>
-      <c r="S24">
+      <c r="T24">
         <f>M24*3+N24</f>
         <v/>
       </c>
-      <c r="T24">
+      <c r="U24">
         <f>S24*100000000 + (R24+100)*100000 + P24*1000 + IFERROR(VLOOKUP(K24, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9393,49 +9476,49 @@
           <t>Viernes, 19 de junio 2026 - 16:00</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="L25">
+      <c r="M25">
         <f>IF(ISNUMBER(F30),1,0)+IF(ISNUMBER(D33),1,0)+IF(ISNUMBER(D35),1,0)</f>
         <v/>
       </c>
-      <c r="M25">
+      <c r="N25">
         <f>IF(AND(ISNUMBER(F30),ISNUMBER(D30),F30&gt;D30),1,0)+IF(AND(ISNUMBER(D33),ISNUMBER(F33),D33&gt;F33),1,0)+IF(AND(ISNUMBER(D35),ISNUMBER(F35),D35&gt;F35),1,0)</f>
         <v/>
       </c>
-      <c r="N25">
+      <c r="O25">
         <f>IF(AND(ISNUMBER(F30),ISNUMBER(D30),F30=D30),1,0)+IF(AND(ISNUMBER(D33),ISNUMBER(F33),D33=F33),1,0)+IF(AND(ISNUMBER(D35),ISNUMBER(F35),D35=F35),1,0)</f>
         <v/>
       </c>
-      <c r="O25">
+      <c r="P25">
         <f>IF(AND(ISNUMBER(F30),ISNUMBER(D30),F30&lt;D30),1,0)+IF(AND(ISNUMBER(D33),ISNUMBER(F33),D33&lt;F33),1,0)+IF(AND(ISNUMBER(D35),ISNUMBER(F35),D35&lt;F35),1,0)</f>
         <v/>
       </c>
-      <c r="P25">
+      <c r="Q25">
         <f>IF(ISNUMBER(F30),F30,0)+IF(ISNUMBER(D33),D33,0)+IF(ISNUMBER(D35),D35,0)</f>
         <v/>
       </c>
-      <c r="Q25">
+      <c r="R25">
         <f>IF(ISNUMBER(D30),D30,0)+IF(ISNUMBER(F33),F33,0)+IF(ISNUMBER(F35),F35,0)</f>
         <v/>
       </c>
-      <c r="R25">
+      <c r="S25">
         <f>P25-Q25</f>
         <v/>
       </c>
-      <c r="S25">
+      <c r="T25">
         <f>M25*3+N25</f>
         <v/>
       </c>
-      <c r="T25">
+      <c r="U25">
         <f>S25*100000000 + (R25+100)*100000 + P25*1000 + IFERROR(VLOOKUP(K25, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9467,49 +9550,49 @@
           <t>Miércoles, 24 de junio 2026 - 16:00</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="L26">
+      <c r="M26">
         <f>IF(ISNUMBER(D31),1,0)+IF(ISNUMBER(F32),1,0)+IF(ISNUMBER(F35),1,0)</f>
         <v/>
       </c>
-      <c r="M26">
+      <c r="N26">
         <f>IF(AND(ISNUMBER(D31),ISNUMBER(F31),D31&gt;F31),1,0)+IF(AND(ISNUMBER(F32),ISNUMBER(D32),F32&gt;D32),1,0)+IF(AND(ISNUMBER(F35),ISNUMBER(D35),F35&gt;D35),1,0)</f>
         <v/>
       </c>
-      <c r="N26">
+      <c r="O26">
         <f>IF(AND(ISNUMBER(D31),ISNUMBER(F31),D31=F31),1,0)+IF(AND(ISNUMBER(F32),ISNUMBER(D32),F32=D32),1,0)+IF(AND(ISNUMBER(F35),ISNUMBER(D35),F35=D35),1,0)</f>
         <v/>
       </c>
-      <c r="O26">
+      <c r="P26">
         <f>IF(AND(ISNUMBER(D31),ISNUMBER(F31),D31&lt;F31),1,0)+IF(AND(ISNUMBER(F32),ISNUMBER(D32),F32&lt;D32),1,0)+IF(AND(ISNUMBER(F35),ISNUMBER(D35),F35&lt;D35),1,0)</f>
         <v/>
       </c>
-      <c r="P26">
+      <c r="Q26">
         <f>IF(ISNUMBER(D31),D31,0)+IF(ISNUMBER(F32),F32,0)+IF(ISNUMBER(F35),F35,0)</f>
         <v/>
       </c>
-      <c r="Q26">
+      <c r="R26">
         <f>IF(ISNUMBER(F31),F31,0)+IF(ISNUMBER(D32),D32,0)+IF(ISNUMBER(D35),D35,0)</f>
         <v/>
       </c>
-      <c r="R26">
+      <c r="S26">
         <f>P26-Q26</f>
         <v/>
       </c>
-      <c r="S26">
+      <c r="T26">
         <f>M26*3+N26</f>
         <v/>
       </c>
-      <c r="T26">
+      <c r="U26">
         <f>S26*100000000 + (R26+100)*100000 + P26*1000 + IFERROR(VLOOKUP(K26, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9541,61 +9624,62 @@
           <t>Miércoles, 24 de junio 2026 - 16:00</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>Turquía</t>
         </is>
       </c>
-      <c r="L27">
+      <c r="M27">
         <f>IF(ISNUMBER(F31),1,0)+IF(ISNUMBER(F33),1,0)+IF(ISNUMBER(D34),1,0)</f>
         <v/>
       </c>
-      <c r="M27">
+      <c r="N27">
         <f>IF(AND(ISNUMBER(F31),ISNUMBER(D31),F31&gt;D31),1,0)+IF(AND(ISNUMBER(F33),ISNUMBER(D33),F33&gt;D33),1,0)+IF(AND(ISNUMBER(D34),ISNUMBER(F34),D34&gt;F34),1,0)</f>
         <v/>
       </c>
-      <c r="N27">
+      <c r="O27">
         <f>IF(AND(ISNUMBER(F31),ISNUMBER(D31),F31=D31),1,0)+IF(AND(ISNUMBER(F33),ISNUMBER(D33),F33=D33),1,0)+IF(AND(ISNUMBER(D34),ISNUMBER(F34),D34=F34),1,0)</f>
         <v/>
       </c>
-      <c r="O27">
+      <c r="P27">
         <f>IF(AND(ISNUMBER(F31),ISNUMBER(D31),F31&lt;D31),1,0)+IF(AND(ISNUMBER(F33),ISNUMBER(D33),F33&lt;D33),1,0)+IF(AND(ISNUMBER(D34),ISNUMBER(F34),D34&lt;F34),1,0)</f>
         <v/>
       </c>
-      <c r="P27">
+      <c r="Q27">
         <f>IF(ISNUMBER(F31),F31,0)+IF(ISNUMBER(F33),F33,0)+IF(ISNUMBER(D34),D34,0)</f>
         <v/>
       </c>
-      <c r="Q27">
+      <c r="R27">
         <f>IF(ISNUMBER(D31),D31,0)+IF(ISNUMBER(D33),D33,0)+IF(ISNUMBER(F34),F34,0)</f>
         <v/>
       </c>
-      <c r="R27">
+      <c r="S27">
         <f>P27-Q27</f>
         <v/>
       </c>
-      <c r="S27">
+      <c r="T27">
         <f>M27*3+N27</f>
         <v/>
       </c>
-      <c r="T27">
+      <c r="U27">
         <f>S27*100000000 + (R27+100)*100000 + P27*1000 + IFERROR(VLOOKUP(K27, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="29" ht="18.75" customHeight="1" s="29">
-      <c r="A29" s="30" t="inlineStr">
+    <row r="28"/>
+    <row r="29" ht="18.75" customHeight="1" s="30">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>GRUPO D</t>
         </is>
       </c>
-      <c r="I29" s="35" t="n"/>
-      <c r="J29" s="30" t="inlineStr">
+      <c r="I29" s="28" t="n"/>
+      <c r="K29" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO E</t>
         </is>
@@ -9628,49 +9712,49 @@
           <t>Viernes, 12 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>Alemania</t>
         </is>
       </c>
-      <c r="L30">
+      <c r="M30">
         <f>IF(ISNUMBER(D38),1,0)+IF(ISNUMBER(D40),1,0)+IF(ISNUMBER(F42),1,0)</f>
         <v/>
       </c>
-      <c r="M30">
+      <c r="N30">
         <f>IF(AND(ISNUMBER(D38),ISNUMBER(F38),D38&gt;F38),1,0)+IF(AND(ISNUMBER(D40),ISNUMBER(F40),D40&gt;F40),1,0)+IF(AND(ISNUMBER(F42),ISNUMBER(D42),F42&gt;D42),1,0)</f>
         <v/>
       </c>
-      <c r="N30">
+      <c r="O30">
         <f>IF(AND(ISNUMBER(D38),ISNUMBER(F38),D38=F38),1,0)+IF(AND(ISNUMBER(D40),ISNUMBER(F40),D40=F40),1,0)+IF(AND(ISNUMBER(F42),ISNUMBER(D42),F42=D42),1,0)</f>
         <v/>
       </c>
-      <c r="O30">
+      <c r="P30">
         <f>IF(AND(ISNUMBER(D38),ISNUMBER(F38),D38&lt;F38),1,0)+IF(AND(ISNUMBER(D40),ISNUMBER(F40),D40&lt;F40),1,0)+IF(AND(ISNUMBER(F42),ISNUMBER(D42),F42&lt;D42),1,0)</f>
         <v/>
       </c>
-      <c r="P30">
+      <c r="Q30">
         <f>IF(ISNUMBER(D38),D38,0)+IF(ISNUMBER(D40),D40,0)+IF(ISNUMBER(F42),F42,0)</f>
         <v/>
       </c>
-      <c r="Q30">
+      <c r="R30">
         <f>IF(ISNUMBER(F38),F38,0)+IF(ISNUMBER(F40),F40,0)+IF(ISNUMBER(D42),D42,0)</f>
         <v/>
       </c>
-      <c r="R30">
+      <c r="S30">
         <f>P30-Q30</f>
         <v/>
       </c>
-      <c r="S30">
+      <c r="T30">
         <f>M30*3+N30</f>
         <v/>
       </c>
-      <c r="T30">
+      <c r="U30">
         <f>S30*100000000 + (R30+100)*100000 + P30*1000 + IFERROR(VLOOKUP(K30, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9702,49 +9786,49 @@
           <t>Sábado, 13 de junio 2026 - 22:00</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="L31">
+      <c r="M31">
         <f>IF(ISNUMBER(F38),1,0)+IF(ISNUMBER(D41),1,0)+IF(ISNUMBER(D43),1,0)</f>
         <v/>
       </c>
-      <c r="M31">
+      <c r="N31">
         <f>IF(AND(ISNUMBER(F38),ISNUMBER(D38),F38&gt;D38),1,0)+IF(AND(ISNUMBER(D41),ISNUMBER(F41),D41&gt;F41),1,0)+IF(AND(ISNUMBER(D43),ISNUMBER(F43),D43&gt;F43),1,0)</f>
         <v/>
       </c>
-      <c r="N31">
+      <c r="O31">
         <f>IF(AND(ISNUMBER(F38),ISNUMBER(D38),F38=D38),1,0)+IF(AND(ISNUMBER(D41),ISNUMBER(F41),D41=F41),1,0)+IF(AND(ISNUMBER(D43),ISNUMBER(F43),D43=F43),1,0)</f>
         <v/>
       </c>
-      <c r="O31">
+      <c r="P31">
         <f>IF(AND(ISNUMBER(F38),ISNUMBER(D38),F38&lt;D38),1,0)+IF(AND(ISNUMBER(D41),ISNUMBER(F41),D41&lt;F41),1,0)+IF(AND(ISNUMBER(D43),ISNUMBER(F43),D43&lt;F43),1,0)</f>
         <v/>
       </c>
-      <c r="P31">
+      <c r="Q31">
         <f>IF(ISNUMBER(F38),F38,0)+IF(ISNUMBER(D41),D41,0)+IF(ISNUMBER(D43),D43,0)</f>
         <v/>
       </c>
-      <c r="Q31">
+      <c r="R31">
         <f>IF(ISNUMBER(D38),D38,0)+IF(ISNUMBER(F41),F41,0)+IF(ISNUMBER(F43),F43,0)</f>
         <v/>
       </c>
-      <c r="R31">
+      <c r="S31">
         <f>P31-Q31</f>
         <v/>
       </c>
-      <c r="S31">
+      <c r="T31">
         <f>M31*3+N31</f>
         <v/>
       </c>
-      <c r="T31">
+      <c r="U31">
         <f>S31*100000000 + (R31+100)*100000 + P31*1000 + IFERROR(VLOOKUP(K31, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9776,49 +9860,49 @@
           <t>Viernes, 19 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>Costa de Marfil</t>
         </is>
       </c>
-      <c r="L32">
+      <c r="M32">
         <f>IF(ISNUMBER(D39),1,0)+IF(ISNUMBER(F40),1,0)+IF(ISNUMBER(F43),1,0)</f>
         <v/>
       </c>
-      <c r="M32">
+      <c r="N32">
         <f>IF(AND(ISNUMBER(D39),ISNUMBER(F39),D39&gt;F39),1,0)+IF(AND(ISNUMBER(F40),ISNUMBER(D40),F40&gt;D40),1,0)+IF(AND(ISNUMBER(F43),ISNUMBER(D43),F43&gt;D43),1,0)</f>
         <v/>
       </c>
-      <c r="N32">
+      <c r="O32">
         <f>IF(AND(ISNUMBER(D39),ISNUMBER(F39),D39=F39),1,0)+IF(AND(ISNUMBER(F40),ISNUMBER(D40),F40=D40),1,0)+IF(AND(ISNUMBER(F43),ISNUMBER(D43),F43=D43),1,0)</f>
         <v/>
       </c>
-      <c r="O32">
+      <c r="P32">
         <f>IF(AND(ISNUMBER(D39),ISNUMBER(F39),D39&lt;F39),1,0)+IF(AND(ISNUMBER(F40),ISNUMBER(D40),F40&lt;D40),1,0)+IF(AND(ISNUMBER(F43),ISNUMBER(D43),F43&lt;D43),1,0)</f>
         <v/>
       </c>
-      <c r="P32">
+      <c r="Q32">
         <f>IF(ISNUMBER(D39),D39,0)+IF(ISNUMBER(F40),F40,0)+IF(ISNUMBER(F43),F43,0)</f>
         <v/>
       </c>
-      <c r="Q32">
+      <c r="R32">
         <f>IF(ISNUMBER(F39),F39,0)+IF(ISNUMBER(D40),D40,0)+IF(ISNUMBER(D43),D43,0)</f>
         <v/>
       </c>
-      <c r="R32">
+      <c r="S32">
         <f>P32-Q32</f>
         <v/>
       </c>
-      <c r="S32">
+      <c r="T32">
         <f>M32*3+N32</f>
         <v/>
       </c>
-      <c r="T32">
+      <c r="U32">
         <f>S32*100000000 + (R32+100)*100000 + P32*1000 + IFERROR(VLOOKUP(K32, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9850,49 +9934,49 @@
           <t>Viernes, 19 de junio 2026 - 22:00</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="L33">
+      <c r="M33">
         <f>IF(ISNUMBER(F39),1,0)+IF(ISNUMBER(F41),1,0)+IF(ISNUMBER(D42),1,0)</f>
         <v/>
       </c>
-      <c r="M33">
+      <c r="N33">
         <f>IF(AND(ISNUMBER(F39),ISNUMBER(D39),F39&gt;D39),1,0)+IF(AND(ISNUMBER(F41),ISNUMBER(D41),F41&gt;D41),1,0)+IF(AND(ISNUMBER(D42),ISNUMBER(F42),D42&gt;F42),1,0)</f>
         <v/>
       </c>
-      <c r="N33">
+      <c r="O33">
         <f>IF(AND(ISNUMBER(F39),ISNUMBER(D39),F39=D39),1,0)+IF(AND(ISNUMBER(F41),ISNUMBER(D41),F41=D41),1,0)+IF(AND(ISNUMBER(D42),ISNUMBER(F42),D42=F42),1,0)</f>
         <v/>
       </c>
-      <c r="O33">
+      <c r="P33">
         <f>IF(AND(ISNUMBER(F39),ISNUMBER(D39),F39&lt;D39),1,0)+IF(AND(ISNUMBER(F41),ISNUMBER(D41),F41&lt;D41),1,0)+IF(AND(ISNUMBER(D42),ISNUMBER(F42),D42&lt;F42),1,0)</f>
         <v/>
       </c>
-      <c r="P33">
+      <c r="Q33">
         <f>IF(ISNUMBER(F39),F39,0)+IF(ISNUMBER(F41),F41,0)+IF(ISNUMBER(D42),D42,0)</f>
         <v/>
       </c>
-      <c r="Q33">
+      <c r="R33">
         <f>IF(ISNUMBER(D39),D39,0)+IF(ISNUMBER(D41),D41,0)+IF(ISNUMBER(F42),F42,0)</f>
         <v/>
       </c>
-      <c r="R33">
+      <c r="S33">
         <f>P33-Q33</f>
         <v/>
       </c>
-      <c r="S33">
+      <c r="T33">
         <f>M33*3+N33</f>
         <v/>
       </c>
-      <c r="T33">
+      <c r="U33">
         <f>S33*100000000 + (R33+100)*100000 + P33*1000 + IFERROR(VLOOKUP(K33, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -9925,7 +10009,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="18.75" customHeight="1" s="29">
+    <row r="35" ht="18.75" customHeight="1" s="30">
       <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Paraguay</t>
@@ -9952,110 +10036,110 @@
           <t>Jueves, 25 de junio 2026 - 20:00</t>
         </is>
       </c>
-      <c r="J35" s="30" t="inlineStr">
+      <c r="K35" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO F</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>Países Bajos</t>
         </is>
       </c>
-      <c r="L36">
+      <c r="M36">
         <f>IF(ISNUMBER(D46),1,0)+IF(ISNUMBER(D48),1,0)+IF(ISNUMBER(F50),1,0)</f>
         <v/>
       </c>
-      <c r="M36">
+      <c r="N36">
         <f>IF(AND(ISNUMBER(D46),ISNUMBER(F46),D46&gt;F46),1,0)+IF(AND(ISNUMBER(D48),ISNUMBER(F48),D48&gt;F48),1,0)+IF(AND(ISNUMBER(F50),ISNUMBER(D50),F50&gt;D50),1,0)</f>
         <v/>
       </c>
-      <c r="N36">
+      <c r="O36">
         <f>IF(AND(ISNUMBER(D46),ISNUMBER(F46),D46=F46),1,0)+IF(AND(ISNUMBER(D48),ISNUMBER(F48),D48=F48),1,0)+IF(AND(ISNUMBER(F50),ISNUMBER(D50),F50=D50),1,0)</f>
         <v/>
       </c>
-      <c r="O36">
+      <c r="P36">
         <f>IF(AND(ISNUMBER(D46),ISNUMBER(F46),D46&lt;F46),1,0)+IF(AND(ISNUMBER(D48),ISNUMBER(F48),D48&lt;F48),1,0)+IF(AND(ISNUMBER(F50),ISNUMBER(D50),F50&lt;D50),1,0)</f>
         <v/>
       </c>
-      <c r="P36">
+      <c r="Q36">
         <f>IF(ISNUMBER(D46),D46,0)+IF(ISNUMBER(D48),D48,0)+IF(ISNUMBER(F50),F50,0)</f>
         <v/>
       </c>
-      <c r="Q36">
+      <c r="R36">
         <f>IF(ISNUMBER(F46),F46,0)+IF(ISNUMBER(F48),F48,0)+IF(ISNUMBER(D50),D50,0)</f>
         <v/>
       </c>
-      <c r="R36">
+      <c r="S36">
         <f>P36-Q36</f>
         <v/>
       </c>
-      <c r="S36">
+      <c r="T36">
         <f>M36*3+N36</f>
         <v/>
       </c>
-      <c r="T36">
+      <c r="U36">
         <f>S36*100000000 + (R36+100)*100000 + P36*1000 + IFERROR(VLOOKUP(K36, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="37" ht="18.75" customHeight="1" s="29">
-      <c r="A37" s="30" t="inlineStr">
+    <row r="37" ht="18.75" customHeight="1" s="30">
+      <c r="A37" s="29" t="inlineStr">
         <is>
           <t>GRUPO E</t>
         </is>
       </c>
-      <c r="I37" s="35" t="n"/>
-      <c r="J37" t="inlineStr">
+      <c r="I37" s="28" t="n"/>
+      <c r="K37" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>Japón</t>
         </is>
       </c>
-      <c r="L37">
+      <c r="M37">
         <f>IF(ISNUMBER(F46),1,0)+IF(ISNUMBER(D49),1,0)+IF(ISNUMBER(D51),1,0)</f>
         <v/>
       </c>
-      <c r="M37">
+      <c r="N37">
         <f>IF(AND(ISNUMBER(F46),ISNUMBER(D46),F46&gt;D46),1,0)+IF(AND(ISNUMBER(D49),ISNUMBER(F49),D49&gt;F49),1,0)+IF(AND(ISNUMBER(D51),ISNUMBER(F51),D51&gt;F51),1,0)</f>
         <v/>
       </c>
-      <c r="N37">
+      <c r="O37">
         <f>IF(AND(ISNUMBER(F46),ISNUMBER(D46),F46=D46),1,0)+IF(AND(ISNUMBER(D49),ISNUMBER(F49),D49=F49),1,0)+IF(AND(ISNUMBER(D51),ISNUMBER(F51),D51=F51),1,0)</f>
         <v/>
       </c>
-      <c r="O37">
+      <c r="P37">
         <f>IF(AND(ISNUMBER(F46),ISNUMBER(D46),F46&lt;D46),1,0)+IF(AND(ISNUMBER(D49),ISNUMBER(F49),D49&lt;F49),1,0)+IF(AND(ISNUMBER(D51),ISNUMBER(F51),D51&lt;F51),1,0)</f>
         <v/>
       </c>
-      <c r="P37">
+      <c r="Q37">
         <f>IF(ISNUMBER(F46),F46,0)+IF(ISNUMBER(D49),D49,0)+IF(ISNUMBER(D51),D51,0)</f>
         <v/>
       </c>
-      <c r="Q37">
+      <c r="R37">
         <f>IF(ISNUMBER(D46),D46,0)+IF(ISNUMBER(F49),F49,0)+IF(ISNUMBER(F51),F51,0)</f>
         <v/>
       </c>
-      <c r="R37">
+      <c r="S37">
         <f>P37-Q37</f>
         <v/>
       </c>
-      <c r="S37">
+      <c r="T37">
         <f>M37*3+N37</f>
         <v/>
       </c>
-      <c r="T37">
+      <c r="U37">
         <f>S37*100000000 + (R37+100)*100000 + P37*1000 + IFERROR(VLOOKUP(K37, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10087,49 +10171,49 @@
           <t>Domingo, 14 de junio 2026 - 11:00</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>Suecia</t>
         </is>
       </c>
-      <c r="L38">
+      <c r="M38">
         <f>IF(ISNUMBER(D47),1,0)+IF(ISNUMBER(F48),1,0)+IF(ISNUMBER(F51),1,0)</f>
         <v/>
       </c>
-      <c r="M38">
+      <c r="N38">
         <f>IF(AND(ISNUMBER(D47),ISNUMBER(F47),D47&gt;F47),1,0)+IF(AND(ISNUMBER(F48),ISNUMBER(D48),F48&gt;D48),1,0)+IF(AND(ISNUMBER(F51),ISNUMBER(D51),F51&gt;D51),1,0)</f>
         <v/>
       </c>
-      <c r="N38">
+      <c r="O38">
         <f>IF(AND(ISNUMBER(D47),ISNUMBER(F47),D47=F47),1,0)+IF(AND(ISNUMBER(F48),ISNUMBER(D48),F48=D48),1,0)+IF(AND(ISNUMBER(F51),ISNUMBER(D51),F51=D51),1,0)</f>
         <v/>
       </c>
-      <c r="O38">
+      <c r="P38">
         <f>IF(AND(ISNUMBER(D47),ISNUMBER(F47),D47&lt;F47),1,0)+IF(AND(ISNUMBER(F48),ISNUMBER(D48),F48&lt;D48),1,0)+IF(AND(ISNUMBER(F51),ISNUMBER(D51),F51&lt;D51),1,0)</f>
         <v/>
       </c>
-      <c r="P38">
+      <c r="Q38">
         <f>IF(ISNUMBER(D47),D47,0)+IF(ISNUMBER(F48),F48,0)+IF(ISNUMBER(F51),F51,0)</f>
         <v/>
       </c>
-      <c r="Q38">
+      <c r="R38">
         <f>IF(ISNUMBER(F47),F47,0)+IF(ISNUMBER(D48),D48,0)+IF(ISNUMBER(D51),D51,0)</f>
         <v/>
       </c>
-      <c r="R38">
+      <c r="S38">
         <f>P38-Q38</f>
         <v/>
       </c>
-      <c r="S38">
+      <c r="T38">
         <f>M38*3+N38</f>
         <v/>
       </c>
-      <c r="T38">
+      <c r="U38">
         <f>S38*100000000 + (R38+100)*100000 + P38*1000 + IFERROR(VLOOKUP(K38, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10161,49 +10245,49 @@
           <t>Domingo, 14 de junio 2026 - 17:00</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>Túnez</t>
         </is>
       </c>
-      <c r="L39">
+      <c r="M39">
         <f>IF(ISNUMBER(F47),1,0)+IF(ISNUMBER(F49),1,0)+IF(ISNUMBER(D50),1,0)</f>
         <v/>
       </c>
-      <c r="M39">
+      <c r="N39">
         <f>IF(AND(ISNUMBER(F47),ISNUMBER(D47),F47&gt;D47),1,0)+IF(AND(ISNUMBER(F49),ISNUMBER(D49),F49&gt;D49),1,0)+IF(AND(ISNUMBER(D50),ISNUMBER(F50),D50&gt;F50),1,0)</f>
         <v/>
       </c>
-      <c r="N39">
+      <c r="O39">
         <f>IF(AND(ISNUMBER(F47),ISNUMBER(D47),F47=D47),1,0)+IF(AND(ISNUMBER(F49),ISNUMBER(D49),F49=D49),1,0)+IF(AND(ISNUMBER(D50),ISNUMBER(F50),D50=F50),1,0)</f>
         <v/>
       </c>
-      <c r="O39">
+      <c r="P39">
         <f>IF(AND(ISNUMBER(F47),ISNUMBER(D47),F47&lt;D47),1,0)+IF(AND(ISNUMBER(F49),ISNUMBER(D49),F49&lt;D49),1,0)+IF(AND(ISNUMBER(D50),ISNUMBER(F50),D50&lt;F50),1,0)</f>
         <v/>
       </c>
-      <c r="P39">
+      <c r="Q39">
         <f>IF(ISNUMBER(F47),F47,0)+IF(ISNUMBER(F49),F49,0)+IF(ISNUMBER(D50),D50,0)</f>
         <v/>
       </c>
-      <c r="Q39">
+      <c r="R39">
         <f>IF(ISNUMBER(D47),D47,0)+IF(ISNUMBER(D49),D49,0)+IF(ISNUMBER(F50),F50,0)</f>
         <v/>
       </c>
-      <c r="R39">
+      <c r="S39">
         <f>P39-Q39</f>
         <v/>
       </c>
-      <c r="S39">
+      <c r="T39">
         <f>M39*3+N39</f>
         <v/>
       </c>
-      <c r="T39">
+      <c r="U39">
         <f>S39*100000000 + (R39+100)*100000 + P39*1000 + IFERROR(VLOOKUP(K39, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10236,7 +10320,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="18.75" customHeight="1" s="29">
+    <row r="41" ht="18.75" customHeight="1" s="30">
       <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Curaçao</t>
@@ -10263,7 +10347,7 @@
           <t>Viernes, 19 de junio 2026 - 14:00</t>
         </is>
       </c>
-      <c r="J41" s="30" t="inlineStr">
+      <c r="K41" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO G</t>
         </is>
@@ -10296,49 +10380,49 @@
           <t>Jueves, 25 de junio 2026 - 14:00</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>Bélgica</t>
         </is>
       </c>
-      <c r="L42">
+      <c r="M42">
         <f>IF(ISNUMBER(D54),1,0)+IF(ISNUMBER(D56),1,0)+IF(ISNUMBER(F58),1,0)</f>
         <v/>
       </c>
-      <c r="M42">
+      <c r="N42">
         <f>IF(AND(ISNUMBER(D54),ISNUMBER(F54),D54&gt;F54),1,0)+IF(AND(ISNUMBER(D56),ISNUMBER(F56),D56&gt;F56),1,0)+IF(AND(ISNUMBER(F58),ISNUMBER(D58),F58&gt;D58),1,0)</f>
         <v/>
       </c>
-      <c r="N42">
+      <c r="O42">
         <f>IF(AND(ISNUMBER(D54),ISNUMBER(F54),D54=F54),1,0)+IF(AND(ISNUMBER(D56),ISNUMBER(F56),D56=F56),1,0)+IF(AND(ISNUMBER(F58),ISNUMBER(D58),F58=D58),1,0)</f>
         <v/>
       </c>
-      <c r="O42">
+      <c r="P42">
         <f>IF(AND(ISNUMBER(D54),ISNUMBER(F54),D54&lt;F54),1,0)+IF(AND(ISNUMBER(D56),ISNUMBER(F56),D56&lt;F56),1,0)+IF(AND(ISNUMBER(F58),ISNUMBER(D58),F58&lt;D58),1,0)</f>
         <v/>
       </c>
-      <c r="P42">
+      <c r="Q42">
         <f>IF(ISNUMBER(D54),D54,0)+IF(ISNUMBER(D56),D56,0)+IF(ISNUMBER(F58),F58,0)</f>
         <v/>
       </c>
-      <c r="Q42">
+      <c r="R42">
         <f>IF(ISNUMBER(F54),F54,0)+IF(ISNUMBER(F56),F56,0)+IF(ISNUMBER(D58),D58,0)</f>
         <v/>
       </c>
-      <c r="R42">
+      <c r="S42">
         <f>P42-Q42</f>
         <v/>
       </c>
-      <c r="S42">
+      <c r="T42">
         <f>M42*3+N42</f>
         <v/>
       </c>
-      <c r="T42">
+      <c r="U42">
         <f>S42*100000000 + (R42+100)*100000 + P42*1000 + IFERROR(VLOOKUP(K42, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10370,151 +10454,151 @@
           <t>Miércoles, 24 de junio 2026 - 14:00</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>Egipto</t>
         </is>
       </c>
-      <c r="L43">
+      <c r="M43">
         <f>IF(ISNUMBER(F54),1,0)+IF(ISNUMBER(D57),1,0)+IF(ISNUMBER(D59),1,0)</f>
         <v/>
       </c>
-      <c r="M43">
+      <c r="N43">
         <f>IF(AND(ISNUMBER(F54),ISNUMBER(D54),F54&gt;D54),1,0)+IF(AND(ISNUMBER(D57),ISNUMBER(F57),D57&gt;F57),1,0)+IF(AND(ISNUMBER(D59),ISNUMBER(F59),D59&gt;F59),1,0)</f>
         <v/>
       </c>
-      <c r="N43">
+      <c r="O43">
         <f>IF(AND(ISNUMBER(F54),ISNUMBER(D54),F54=D54),1,0)+IF(AND(ISNUMBER(D57),ISNUMBER(F57),D57=F57),1,0)+IF(AND(ISNUMBER(D59),ISNUMBER(F59),D59=F59),1,0)</f>
         <v/>
       </c>
-      <c r="O43">
+      <c r="P43">
         <f>IF(AND(ISNUMBER(F54),ISNUMBER(D54),F54&lt;D54),1,0)+IF(AND(ISNUMBER(D57),ISNUMBER(F57),D57&lt;F57),1,0)+IF(AND(ISNUMBER(D59),ISNUMBER(F59),D59&lt;F59),1,0)</f>
         <v/>
       </c>
-      <c r="P43">
+      <c r="Q43">
         <f>IF(ISNUMBER(F54),F54,0)+IF(ISNUMBER(D57),D57,0)+IF(ISNUMBER(D59),D59,0)</f>
         <v/>
       </c>
-      <c r="Q43">
+      <c r="R43">
         <f>IF(ISNUMBER(D54),D54,0)+IF(ISNUMBER(F57),F57,0)+IF(ISNUMBER(F59),F59,0)</f>
         <v/>
       </c>
-      <c r="R43">
+      <c r="S43">
         <f>P43-Q43</f>
         <v/>
       </c>
-      <c r="S43">
+      <c r="T43">
         <f>M43*3+N43</f>
         <v/>
       </c>
-      <c r="T43">
+      <c r="U43">
         <f>S43*100000000 + (R43+100)*100000 + P43*1000 + IFERROR(VLOOKUP(K43, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>Irán</t>
         </is>
       </c>
-      <c r="L44">
+      <c r="M44">
         <f>IF(ISNUMBER(D55),1,0)+IF(ISNUMBER(F56),1,0)+IF(ISNUMBER(F59),1,0)</f>
         <v/>
       </c>
-      <c r="M44">
+      <c r="N44">
         <f>IF(AND(ISNUMBER(D55),ISNUMBER(F55),D55&gt;F55),1,0)+IF(AND(ISNUMBER(F56),ISNUMBER(D56),F56&gt;D56),1,0)+IF(AND(ISNUMBER(F59),ISNUMBER(D59),F59&gt;D59),1,0)</f>
         <v/>
       </c>
-      <c r="N44">
+      <c r="O44">
         <f>IF(AND(ISNUMBER(D55),ISNUMBER(F55),D55=F55),1,0)+IF(AND(ISNUMBER(F56),ISNUMBER(D56),F56=D56),1,0)+IF(AND(ISNUMBER(F59),ISNUMBER(D59),F59=D59),1,0)</f>
         <v/>
       </c>
-      <c r="O44">
+      <c r="P44">
         <f>IF(AND(ISNUMBER(D55),ISNUMBER(F55),D55&lt;F55),1,0)+IF(AND(ISNUMBER(F56),ISNUMBER(D56),F56&lt;D56),1,0)+IF(AND(ISNUMBER(F59),ISNUMBER(D59),F59&lt;D59),1,0)</f>
         <v/>
       </c>
-      <c r="P44">
+      <c r="Q44">
         <f>IF(ISNUMBER(D55),D55,0)+IF(ISNUMBER(F56),F56,0)+IF(ISNUMBER(F59),F59,0)</f>
         <v/>
       </c>
-      <c r="Q44">
+      <c r="R44">
         <f>IF(ISNUMBER(F55),F55,0)+IF(ISNUMBER(D56),D56,0)+IF(ISNUMBER(D59),D59,0)</f>
         <v/>
       </c>
-      <c r="R44">
+      <c r="S44">
         <f>P44-Q44</f>
         <v/>
       </c>
-      <c r="S44">
+      <c r="T44">
         <f>M44*3+N44</f>
         <v/>
       </c>
-      <c r="T44">
+      <c r="U44">
         <f>S44*100000000 + (R44+100)*100000 + P44*1000 + IFERROR(VLOOKUP(K44, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="45" ht="18.75" customHeight="1" s="29">
-      <c r="A45" s="30" t="inlineStr">
+    <row r="45" ht="18.75" customHeight="1" s="30">
+      <c r="A45" s="29" t="inlineStr">
         <is>
           <t>GRUPO F</t>
         </is>
       </c>
-      <c r="I45" s="35" t="n"/>
-      <c r="J45" t="inlineStr">
+      <c r="I45" s="28" t="n"/>
+      <c r="K45" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>Nueva Zelanda</t>
         </is>
       </c>
-      <c r="L45">
+      <c r="M45">
         <f>IF(ISNUMBER(F55),1,0)+IF(ISNUMBER(F57),1,0)+IF(ISNUMBER(D58),1,0)</f>
         <v/>
       </c>
-      <c r="M45">
+      <c r="N45">
         <f>IF(AND(ISNUMBER(F55),ISNUMBER(D55),F55&gt;D55),1,0)+IF(AND(ISNUMBER(F57),ISNUMBER(D57),F57&gt;D57),1,0)+IF(AND(ISNUMBER(D58),ISNUMBER(F58),D58&gt;F58),1,0)</f>
         <v/>
       </c>
-      <c r="N45">
+      <c r="O45">
         <f>IF(AND(ISNUMBER(F55),ISNUMBER(D55),F55=D55),1,0)+IF(AND(ISNUMBER(F57),ISNUMBER(D57),F57=D57),1,0)+IF(AND(ISNUMBER(D58),ISNUMBER(F58),D58=F58),1,0)</f>
         <v/>
       </c>
-      <c r="O45">
+      <c r="P45">
         <f>IF(AND(ISNUMBER(F55),ISNUMBER(D55),F55&lt;D55),1,0)+IF(AND(ISNUMBER(F57),ISNUMBER(D57),F57&lt;D57),1,0)+IF(AND(ISNUMBER(D58),ISNUMBER(F58),D58&lt;F58),1,0)</f>
         <v/>
       </c>
-      <c r="P45">
+      <c r="Q45">
         <f>IF(ISNUMBER(F55),F55,0)+IF(ISNUMBER(F57),F57,0)+IF(ISNUMBER(D58),D58,0)</f>
         <v/>
       </c>
-      <c r="Q45">
+      <c r="R45">
         <f>IF(ISNUMBER(D55),D55,0)+IF(ISNUMBER(D57),D57,0)+IF(ISNUMBER(F58),F58,0)</f>
         <v/>
       </c>
-      <c r="R45">
+      <c r="S45">
         <f>P45-Q45</f>
         <v/>
       </c>
-      <c r="S45">
+      <c r="T45">
         <f>M45*3+N45</f>
         <v/>
       </c>
-      <c r="T45">
+      <c r="U45">
         <f>S45*100000000 + (R45+100)*100000 + P45*1000 + IFERROR(VLOOKUP(K45, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10547,7 +10631,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="18.75" customHeight="1" s="29">
+    <row r="47" ht="18.75" customHeight="1" s="30">
       <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Suecia</t>
@@ -10574,7 +10658,7 @@
           <t>Domingo, 14 de junio 2026 - 20:00</t>
         </is>
       </c>
-      <c r="J47" s="30" t="inlineStr">
+      <c r="K47" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO H</t>
         </is>
@@ -10607,49 +10691,49 @@
           <t>Sábado, 20 de junio 2026 - 11:00</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>España</t>
         </is>
       </c>
-      <c r="L48">
+      <c r="M48">
         <f>IF(ISNUMBER(D62),1,0)+IF(ISNUMBER(D64),1,0)+IF(ISNUMBER(F66),1,0)</f>
         <v/>
       </c>
-      <c r="M48">
+      <c r="N48">
         <f>IF(AND(ISNUMBER(D62),ISNUMBER(F62),D62&gt;F62),1,0)+IF(AND(ISNUMBER(D64),ISNUMBER(F64),D64&gt;F64),1,0)+IF(AND(ISNUMBER(F66),ISNUMBER(D66),F66&gt;D66),1,0)</f>
         <v/>
       </c>
-      <c r="N48">
+      <c r="O48">
         <f>IF(AND(ISNUMBER(D62),ISNUMBER(F62),D62=F62),1,0)+IF(AND(ISNUMBER(D64),ISNUMBER(F64),D64=F64),1,0)+IF(AND(ISNUMBER(F66),ISNUMBER(D66),F66=D66),1,0)</f>
         <v/>
       </c>
-      <c r="O48">
+      <c r="P48">
         <f>IF(AND(ISNUMBER(D62),ISNUMBER(F62),D62&lt;F62),1,0)+IF(AND(ISNUMBER(D64),ISNUMBER(F64),D64&lt;F64),1,0)+IF(AND(ISNUMBER(F66),ISNUMBER(D66),F66&lt;D66),1,0)</f>
         <v/>
       </c>
-      <c r="P48">
+      <c r="Q48">
         <f>IF(ISNUMBER(D62),D62,0)+IF(ISNUMBER(D64),D64,0)+IF(ISNUMBER(F66),F66,0)</f>
         <v/>
       </c>
-      <c r="Q48">
+      <c r="R48">
         <f>IF(ISNUMBER(F62),F62,0)+IF(ISNUMBER(F64),F64,0)+IF(ISNUMBER(D66),D66,0)</f>
         <v/>
       </c>
-      <c r="R48">
+      <c r="S48">
         <f>P48-Q48</f>
         <v/>
       </c>
-      <c r="S48">
+      <c r="T48">
         <f>M48*3+N48</f>
         <v/>
       </c>
-      <c r="T48">
+      <c r="U48">
         <f>S48*100000000 + (R48+100)*100000 + P48*1000 + IFERROR(VLOOKUP(K48, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10681,49 +10765,49 @@
           <t>Sábado, 20 de junio 2026 - 22:00</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>Cabo Verde</t>
         </is>
       </c>
-      <c r="L49">
+      <c r="M49">
         <f>IF(ISNUMBER(F62),1,0)+IF(ISNUMBER(D65),1,0)+IF(ISNUMBER(D67),1,0)</f>
         <v/>
       </c>
-      <c r="M49">
+      <c r="N49">
         <f>IF(AND(ISNUMBER(F62),ISNUMBER(D62),F62&gt;D62),1,0)+IF(AND(ISNUMBER(D65),ISNUMBER(F65),D65&gt;F65),1,0)+IF(AND(ISNUMBER(D67),ISNUMBER(F67),D67&gt;F67),1,0)</f>
         <v/>
       </c>
-      <c r="N49">
+      <c r="O49">
         <f>IF(AND(ISNUMBER(F62),ISNUMBER(D62),F62=D62),1,0)+IF(AND(ISNUMBER(D65),ISNUMBER(F65),D65=F65),1,0)+IF(AND(ISNUMBER(D67),ISNUMBER(F67),D67=F67),1,0)</f>
         <v/>
       </c>
-      <c r="O49">
+      <c r="P49">
         <f>IF(AND(ISNUMBER(F62),ISNUMBER(D62),F62&lt;D62),1,0)+IF(AND(ISNUMBER(D65),ISNUMBER(F65),D65&lt;F65),1,0)+IF(AND(ISNUMBER(D67),ISNUMBER(F67),D67&lt;F67),1,0)</f>
         <v/>
       </c>
-      <c r="P49">
+      <c r="Q49">
         <f>IF(ISNUMBER(F62),F62,0)+IF(ISNUMBER(D65),D65,0)+IF(ISNUMBER(D67),D67,0)</f>
         <v/>
       </c>
-      <c r="Q49">
+      <c r="R49">
         <f>IF(ISNUMBER(D62),D62,0)+IF(ISNUMBER(F65),F65,0)+IF(ISNUMBER(F67),F67,0)</f>
         <v/>
       </c>
-      <c r="R49">
+      <c r="S49">
         <f>P49-Q49</f>
         <v/>
       </c>
-      <c r="S49">
+      <c r="T49">
         <f>M49*3+N49</f>
         <v/>
       </c>
-      <c r="T49">
+      <c r="U49">
         <f>S49*100000000 + (R49+100)*100000 + P49*1000 + IFERROR(VLOOKUP(K49, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10755,49 +10839,49 @@
           <t>Jueves, 25 de junio 2026 - 17:00</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>Arabia Saud.</t>
         </is>
       </c>
-      <c r="L50">
+      <c r="M50">
         <f>IF(ISNUMBER(D63),1,0)+IF(ISNUMBER(F64),1,0)+IF(ISNUMBER(F67),1,0)</f>
         <v/>
       </c>
-      <c r="M50">
+      <c r="N50">
         <f>IF(AND(ISNUMBER(D63),ISNUMBER(F63),D63&gt;F63),1,0)+IF(AND(ISNUMBER(F64),ISNUMBER(D64),F64&gt;D64),1,0)+IF(AND(ISNUMBER(F67),ISNUMBER(D67),F67&gt;D67),1,0)</f>
         <v/>
       </c>
-      <c r="N50">
+      <c r="O50">
         <f>IF(AND(ISNUMBER(D63),ISNUMBER(F63),D63=F63),1,0)+IF(AND(ISNUMBER(F64),ISNUMBER(D64),F64=D64),1,0)+IF(AND(ISNUMBER(F67),ISNUMBER(D67),F67=D67),1,0)</f>
         <v/>
       </c>
-      <c r="O50">
+      <c r="P50">
         <f>IF(AND(ISNUMBER(D63),ISNUMBER(F63),D63&lt;F63),1,0)+IF(AND(ISNUMBER(F64),ISNUMBER(D64),F64&lt;D64),1,0)+IF(AND(ISNUMBER(F67),ISNUMBER(D67),F67&lt;D67),1,0)</f>
         <v/>
       </c>
-      <c r="P50">
+      <c r="Q50">
         <f>IF(ISNUMBER(D63),D63,0)+IF(ISNUMBER(F64),F64,0)+IF(ISNUMBER(F67),F67,0)</f>
         <v/>
       </c>
-      <c r="Q50">
+      <c r="R50">
         <f>IF(ISNUMBER(F63),F63,0)+IF(ISNUMBER(D64),D64,0)+IF(ISNUMBER(D67),D67,0)</f>
         <v/>
       </c>
-      <c r="R50">
+      <c r="S50">
         <f>P50-Q50</f>
         <v/>
       </c>
-      <c r="S50">
+      <c r="T50">
         <f>M50*3+N50</f>
         <v/>
       </c>
-      <c r="T50">
+      <c r="U50">
         <f>S50*100000000 + (R50+100)*100000 + P50*1000 + IFERROR(VLOOKUP(K50, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10829,61 +10913,62 @@
           <t>Jueves, 25 de junio 2026 - 17:00</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="L51" t="inlineStr">
         <is>
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="L51">
+      <c r="M51">
         <f>IF(ISNUMBER(F63),1,0)+IF(ISNUMBER(F65),1,0)+IF(ISNUMBER(D66),1,0)</f>
         <v/>
       </c>
-      <c r="M51">
+      <c r="N51">
         <f>IF(AND(ISNUMBER(F63),ISNUMBER(D63),F63&gt;D63),1,0)+IF(AND(ISNUMBER(F65),ISNUMBER(D65),F65&gt;D65),1,0)+IF(AND(ISNUMBER(D66),ISNUMBER(F66),D66&gt;F66),1,0)</f>
         <v/>
       </c>
-      <c r="N51">
+      <c r="O51">
         <f>IF(AND(ISNUMBER(F63),ISNUMBER(D63),F63=D63),1,0)+IF(AND(ISNUMBER(F65),ISNUMBER(D65),F65=D65),1,0)+IF(AND(ISNUMBER(D66),ISNUMBER(F66),D66=F66),1,0)</f>
         <v/>
       </c>
-      <c r="O51">
+      <c r="P51">
         <f>IF(AND(ISNUMBER(F63),ISNUMBER(D63),F63&lt;D63),1,0)+IF(AND(ISNUMBER(F65),ISNUMBER(D65),F65&lt;D65),1,0)+IF(AND(ISNUMBER(D66),ISNUMBER(F66),D66&lt;F66),1,0)</f>
         <v/>
       </c>
-      <c r="P51">
+      <c r="Q51">
         <f>IF(ISNUMBER(F63),F63,0)+IF(ISNUMBER(F65),F65,0)+IF(ISNUMBER(D66),D66,0)</f>
         <v/>
       </c>
-      <c r="Q51">
+      <c r="R51">
         <f>IF(ISNUMBER(D63),D63,0)+IF(ISNUMBER(D65),D65,0)+IF(ISNUMBER(F66),F66,0)</f>
         <v/>
       </c>
-      <c r="R51">
+      <c r="S51">
         <f>P51-Q51</f>
         <v/>
       </c>
-      <c r="S51">
+      <c r="T51">
         <f>M51*3+N51</f>
         <v/>
       </c>
-      <c r="T51">
+      <c r="U51">
         <f>S51*100000000 + (R51+100)*100000 + P51*1000 + IFERROR(VLOOKUP(K51, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="53" ht="18.75" customHeight="1" s="29">
-      <c r="A53" s="30" t="inlineStr">
+    <row r="52"/>
+    <row r="53" ht="18.75" customHeight="1" s="30">
+      <c r="A53" s="29" t="inlineStr">
         <is>
           <t>GRUPO G</t>
         </is>
       </c>
-      <c r="I53" s="35" t="n"/>
-      <c r="J53" s="30" t="inlineStr">
+      <c r="I53" s="28" t="n"/>
+      <c r="K53" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO I</t>
         </is>
@@ -10916,49 +11001,49 @@
           <t>Lunes, 15 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>Francia</t>
         </is>
       </c>
-      <c r="L54">
+      <c r="M54">
         <f>IF(ISNUMBER(D70),1,0)+IF(ISNUMBER(D72),1,0)+IF(ISNUMBER(F74),1,0)</f>
         <v/>
       </c>
-      <c r="M54">
+      <c r="N54">
         <f>IF(AND(ISNUMBER(D70),ISNUMBER(F70),D70&gt;F70),1,0)+IF(AND(ISNUMBER(D72),ISNUMBER(F72),D72&gt;F72),1,0)+IF(AND(ISNUMBER(F74),ISNUMBER(D74),F74&gt;D74),1,0)</f>
         <v/>
       </c>
-      <c r="N54">
+      <c r="O54">
         <f>IF(AND(ISNUMBER(D70),ISNUMBER(F70),D70=F70),1,0)+IF(AND(ISNUMBER(D72),ISNUMBER(F72),D72=F72),1,0)+IF(AND(ISNUMBER(F74),ISNUMBER(D74),F74=D74),1,0)</f>
         <v/>
       </c>
-      <c r="O54">
+      <c r="P54">
         <f>IF(AND(ISNUMBER(D70),ISNUMBER(F70),D70&lt;F70),1,0)+IF(AND(ISNUMBER(D72),ISNUMBER(F72),D72&lt;F72),1,0)+IF(AND(ISNUMBER(F74),ISNUMBER(D74),F74&lt;D74),1,0)</f>
         <v/>
       </c>
-      <c r="P54">
+      <c r="Q54">
         <f>IF(ISNUMBER(D70),D70,0)+IF(ISNUMBER(D72),D72,0)+IF(ISNUMBER(F74),F74,0)</f>
         <v/>
       </c>
-      <c r="Q54">
+      <c r="R54">
         <f>IF(ISNUMBER(F70),F70,0)+IF(ISNUMBER(F72),F72,0)+IF(ISNUMBER(D74),D74,0)</f>
         <v/>
       </c>
-      <c r="R54">
+      <c r="S54">
         <f>P54-Q54</f>
         <v/>
       </c>
-      <c r="S54">
+      <c r="T54">
         <f>M54*3+N54</f>
         <v/>
       </c>
-      <c r="T54">
+      <c r="U54">
         <f>S54*100000000 + (R54+100)*100000 + P54*1000 + IFERROR(VLOOKUP(K54, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -10990,49 +11075,49 @@
           <t>Lunes, 15 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="L55" t="inlineStr">
         <is>
           <t>Senegal</t>
         </is>
       </c>
-      <c r="L55">
+      <c r="M55">
         <f>IF(ISNUMBER(F70),1,0)+IF(ISNUMBER(D73),1,0)+IF(ISNUMBER(D75),1,0)</f>
         <v/>
       </c>
-      <c r="M55">
+      <c r="N55">
         <f>IF(AND(ISNUMBER(F70),ISNUMBER(D70),F70&gt;D70),1,0)+IF(AND(ISNUMBER(D73),ISNUMBER(F73),D73&gt;F73),1,0)+IF(AND(ISNUMBER(D75),ISNUMBER(F75),D75&gt;F75),1,0)</f>
         <v/>
       </c>
-      <c r="N55">
+      <c r="O55">
         <f>IF(AND(ISNUMBER(F70),ISNUMBER(D70),F70=D70),1,0)+IF(AND(ISNUMBER(D73),ISNUMBER(F73),D73=F73),1,0)+IF(AND(ISNUMBER(D75),ISNUMBER(F75),D75=F75),1,0)</f>
         <v/>
       </c>
-      <c r="O55">
+      <c r="P55">
         <f>IF(AND(ISNUMBER(F70),ISNUMBER(D70),F70&lt;D70),1,0)+IF(AND(ISNUMBER(D73),ISNUMBER(F73),D73&lt;F73),1,0)+IF(AND(ISNUMBER(D75),ISNUMBER(F75),D75&lt;F75),1,0)</f>
         <v/>
       </c>
-      <c r="P55">
+      <c r="Q55">
         <f>IF(ISNUMBER(F70),F70,0)+IF(ISNUMBER(D73),D73,0)+IF(ISNUMBER(D75),D75,0)</f>
         <v/>
       </c>
-      <c r="Q55">
+      <c r="R55">
         <f>IF(ISNUMBER(D70),D70,0)+IF(ISNUMBER(F73),F73,0)+IF(ISNUMBER(F75),F75,0)</f>
         <v/>
       </c>
-      <c r="R55">
+      <c r="S55">
         <f>P55-Q55</f>
         <v/>
       </c>
-      <c r="S55">
+      <c r="T55">
         <f>M55*3+N55</f>
         <v/>
       </c>
-      <c r="T55">
+      <c r="U55">
         <f>S55*100000000 + (R55+100)*100000 + P55*1000 + IFERROR(VLOOKUP(K55, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11064,49 +11149,49 @@
           <t>Domingo, 21 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="L56" t="inlineStr">
         <is>
           <t>Irak</t>
         </is>
       </c>
-      <c r="L56">
+      <c r="M56">
         <f>IF(ISNUMBER(D71),1,0)+IF(ISNUMBER(F72),1,0)+IF(ISNUMBER(F75),1,0)</f>
         <v/>
       </c>
-      <c r="M56">
+      <c r="N56">
         <f>IF(AND(ISNUMBER(D71),ISNUMBER(F71),D71&gt;F71),1,0)+IF(AND(ISNUMBER(F72),ISNUMBER(D72),F72&gt;D72),1,0)+IF(AND(ISNUMBER(F75),ISNUMBER(D75),F75&gt;D75),1,0)</f>
         <v/>
       </c>
-      <c r="N56">
+      <c r="O56">
         <f>IF(AND(ISNUMBER(D71),ISNUMBER(F71),D71=F71),1,0)+IF(AND(ISNUMBER(F72),ISNUMBER(D72),F72=D72),1,0)+IF(AND(ISNUMBER(F75),ISNUMBER(D75),F75=D75),1,0)</f>
         <v/>
       </c>
-      <c r="O56">
+      <c r="P56">
         <f>IF(AND(ISNUMBER(D71),ISNUMBER(F71),D71&lt;F71),1,0)+IF(AND(ISNUMBER(F72),ISNUMBER(D72),F72&lt;D72),1,0)+IF(AND(ISNUMBER(F75),ISNUMBER(D75),F75&lt;D75),1,0)</f>
         <v/>
       </c>
-      <c r="P56">
+      <c r="Q56">
         <f>IF(ISNUMBER(D71),D71,0)+IF(ISNUMBER(F72),F72,0)+IF(ISNUMBER(F75),F75,0)</f>
         <v/>
       </c>
-      <c r="Q56">
+      <c r="R56">
         <f>IF(ISNUMBER(F71),F71,0)+IF(ISNUMBER(D72),D72,0)+IF(ISNUMBER(D75),D75,0)</f>
         <v/>
       </c>
-      <c r="R56">
+      <c r="S56">
         <f>P56-Q56</f>
         <v/>
       </c>
-      <c r="S56">
+      <c r="T56">
         <f>M56*3+N56</f>
         <v/>
       </c>
-      <c r="T56">
+      <c r="U56">
         <f>S56*100000000 + (R56+100)*100000 + P56*1000 + IFERROR(VLOOKUP(K56, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11138,49 +11223,49 @@
           <t>Domingo, 21 de junio 2026 - 19:00</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="L57" t="inlineStr">
         <is>
           <t>Noruega</t>
         </is>
       </c>
-      <c r="L57">
+      <c r="M57">
         <f>IF(ISNUMBER(F71),1,0)+IF(ISNUMBER(F73),1,0)+IF(ISNUMBER(D74),1,0)</f>
         <v/>
       </c>
-      <c r="M57">
+      <c r="N57">
         <f>IF(AND(ISNUMBER(F71),ISNUMBER(D71),F71&gt;D71),1,0)+IF(AND(ISNUMBER(F73),ISNUMBER(D73),F73&gt;D73),1,0)+IF(AND(ISNUMBER(D74),ISNUMBER(F74),D74&gt;F74),1,0)</f>
         <v/>
       </c>
-      <c r="N57">
+      <c r="O57">
         <f>IF(AND(ISNUMBER(F71),ISNUMBER(D71),F71=D71),1,0)+IF(AND(ISNUMBER(F73),ISNUMBER(D73),F73=D73),1,0)+IF(AND(ISNUMBER(D74),ISNUMBER(F74),D74=F74),1,0)</f>
         <v/>
       </c>
-      <c r="O57">
+      <c r="P57">
         <f>IF(AND(ISNUMBER(F71),ISNUMBER(D71),F71&lt;D71),1,0)+IF(AND(ISNUMBER(F73),ISNUMBER(D73),F73&lt;D73),1,0)+IF(AND(ISNUMBER(D74),ISNUMBER(F74),D74&lt;F74),1,0)</f>
         <v/>
       </c>
-      <c r="P57">
+      <c r="Q57">
         <f>IF(ISNUMBER(F71),F71,0)+IF(ISNUMBER(F73),F73,0)+IF(ISNUMBER(D74),D74,0)</f>
         <v/>
       </c>
-      <c r="Q57">
+      <c r="R57">
         <f>IF(ISNUMBER(D71),D71,0)+IF(ISNUMBER(D73),D73,0)+IF(ISNUMBER(F74),F74,0)</f>
         <v/>
       </c>
-      <c r="R57">
+      <c r="S57">
         <f>P57-Q57</f>
         <v/>
       </c>
-      <c r="S57">
+      <c r="T57">
         <f>M57*3+N57</f>
         <v/>
       </c>
-      <c r="T57">
+      <c r="U57">
         <f>S57*100000000 + (R57+100)*100000 + P57*1000 + IFERROR(VLOOKUP(K57, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11213,7 +11298,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="18.75" customHeight="1" s="29">
+    <row r="59" ht="18.75" customHeight="1" s="30">
       <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Egipto</t>
@@ -11240,110 +11325,110 @@
           <t>Viernes, 26 de junio 2026 - 21:00</t>
         </is>
       </c>
-      <c r="J59" s="30" t="inlineStr">
+      <c r="K59" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO J</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="J60" t="inlineStr">
+      <c r="K60" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="L60" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="L60">
+      <c r="M60">
         <f>IF(ISNUMBER(D78),1,0)+IF(ISNUMBER(D80),1,0)+IF(ISNUMBER(F82),1,0)</f>
         <v/>
       </c>
-      <c r="M60">
+      <c r="N60">
         <f>IF(AND(ISNUMBER(D78),ISNUMBER(F78),D78&gt;F78),1,0)+IF(AND(ISNUMBER(D80),ISNUMBER(F80),D80&gt;F80),1,0)+IF(AND(ISNUMBER(F82),ISNUMBER(D82),F82&gt;D82),1,0)</f>
         <v/>
       </c>
-      <c r="N60">
+      <c r="O60">
         <f>IF(AND(ISNUMBER(D78),ISNUMBER(F78),D78=F78),1,0)+IF(AND(ISNUMBER(D80),ISNUMBER(F80),D80=F80),1,0)+IF(AND(ISNUMBER(F82),ISNUMBER(D82),F82=D82),1,0)</f>
         <v/>
       </c>
-      <c r="O60">
+      <c r="P60">
         <f>IF(AND(ISNUMBER(D78),ISNUMBER(F78),D78&lt;F78),1,0)+IF(AND(ISNUMBER(D80),ISNUMBER(F80),D80&lt;F80),1,0)+IF(AND(ISNUMBER(F82),ISNUMBER(D82),F82&lt;D82),1,0)</f>
         <v/>
       </c>
-      <c r="P60">
+      <c r="Q60">
         <f>IF(ISNUMBER(D78),D78,0)+IF(ISNUMBER(D80),D80,0)+IF(ISNUMBER(F82),F82,0)</f>
         <v/>
       </c>
-      <c r="Q60">
+      <c r="R60">
         <f>IF(ISNUMBER(F78),F78,0)+IF(ISNUMBER(F80),F80,0)+IF(ISNUMBER(D82),D82,0)</f>
         <v/>
       </c>
-      <c r="R60">
+      <c r="S60">
         <f>P60-Q60</f>
         <v/>
       </c>
-      <c r="S60">
+      <c r="T60">
         <f>M60*3+N60</f>
         <v/>
       </c>
-      <c r="T60">
+      <c r="U60">
         <f>S60*100000000 + (R60+100)*100000 + P60*1000 + IFERROR(VLOOKUP(K60, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="61" ht="18.75" customHeight="1" s="29">
-      <c r="A61" s="30" t="inlineStr">
+    <row r="61" ht="18.75" customHeight="1" s="30">
+      <c r="A61" s="29" t="inlineStr">
         <is>
           <t>GRUPO H</t>
         </is>
       </c>
-      <c r="I61" s="35" t="n"/>
-      <c r="J61" t="inlineStr">
+      <c r="I61" s="28" t="n"/>
+      <c r="K61" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="L61" t="inlineStr">
         <is>
           <t>Argelia</t>
         </is>
       </c>
-      <c r="L61">
+      <c r="M61">
         <f>IF(ISNUMBER(F78),1,0)+IF(ISNUMBER(D81),1,0)+IF(ISNUMBER(D83),1,0)</f>
         <v/>
       </c>
-      <c r="M61">
+      <c r="N61">
         <f>IF(AND(ISNUMBER(F78),ISNUMBER(D78),F78&gt;D78),1,0)+IF(AND(ISNUMBER(D81),ISNUMBER(F81),D81&gt;F81),1,0)+IF(AND(ISNUMBER(D83),ISNUMBER(F83),D83&gt;F83),1,0)</f>
         <v/>
       </c>
-      <c r="N61">
+      <c r="O61">
         <f>IF(AND(ISNUMBER(F78),ISNUMBER(D78),F78=D78),1,0)+IF(AND(ISNUMBER(D81),ISNUMBER(F81),D81=F81),1,0)+IF(AND(ISNUMBER(D83),ISNUMBER(F83),D83=F83),1,0)</f>
         <v/>
       </c>
-      <c r="O61">
+      <c r="P61">
         <f>IF(AND(ISNUMBER(F78),ISNUMBER(D78),F78&lt;D78),1,0)+IF(AND(ISNUMBER(D81),ISNUMBER(F81),D81&lt;F81),1,0)+IF(AND(ISNUMBER(D83),ISNUMBER(F83),D83&lt;F83),1,0)</f>
         <v/>
       </c>
-      <c r="P61">
+      <c r="Q61">
         <f>IF(ISNUMBER(F78),F78,0)+IF(ISNUMBER(D81),D81,0)+IF(ISNUMBER(D83),D83,0)</f>
         <v/>
       </c>
-      <c r="Q61">
+      <c r="R61">
         <f>IF(ISNUMBER(D78),D78,0)+IF(ISNUMBER(F81),F81,0)+IF(ISNUMBER(F83),F83,0)</f>
         <v/>
       </c>
-      <c r="R61">
+      <c r="S61">
         <f>P61-Q61</f>
         <v/>
       </c>
-      <c r="S61">
+      <c r="T61">
         <f>M61*3+N61</f>
         <v/>
       </c>
-      <c r="T61">
+      <c r="U61">
         <f>S61*100000000 + (R61+100)*100000 + P61*1000 + IFERROR(VLOOKUP(K61, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11375,49 +11460,49 @@
           <t>Lunes, 15 de junio 2026 - 10:00</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="L62" t="inlineStr">
         <is>
           <t>Austria</t>
         </is>
       </c>
-      <c r="L62">
+      <c r="M62">
         <f>IF(ISNUMBER(D79),1,0)+IF(ISNUMBER(F80),1,0)+IF(ISNUMBER(F83),1,0)</f>
         <v/>
       </c>
-      <c r="M62">
+      <c r="N62">
         <f>IF(AND(ISNUMBER(D79),ISNUMBER(F79),D79&gt;F79),1,0)+IF(AND(ISNUMBER(F80),ISNUMBER(D80),F80&gt;D80),1,0)+IF(AND(ISNUMBER(F83),ISNUMBER(D83),F83&gt;D83),1,0)</f>
         <v/>
       </c>
-      <c r="N62">
+      <c r="O62">
         <f>IF(AND(ISNUMBER(D79),ISNUMBER(F79),D79=F79),1,0)+IF(AND(ISNUMBER(F80),ISNUMBER(D80),F80=D80),1,0)+IF(AND(ISNUMBER(F83),ISNUMBER(D83),F83=D83),1,0)</f>
         <v/>
       </c>
-      <c r="O62">
+      <c r="P62">
         <f>IF(AND(ISNUMBER(D79),ISNUMBER(F79),D79&lt;F79),1,0)+IF(AND(ISNUMBER(F80),ISNUMBER(D80),F80&lt;D80),1,0)+IF(AND(ISNUMBER(F83),ISNUMBER(D83),F83&lt;D83),1,0)</f>
         <v/>
       </c>
-      <c r="P62">
+      <c r="Q62">
         <f>IF(ISNUMBER(D79),D79,0)+IF(ISNUMBER(F80),F80,0)+IF(ISNUMBER(F83),F83,0)</f>
         <v/>
       </c>
-      <c r="Q62">
+      <c r="R62">
         <f>IF(ISNUMBER(F79),F79,0)+IF(ISNUMBER(D80),D80,0)+IF(ISNUMBER(D83),D83,0)</f>
         <v/>
       </c>
-      <c r="R62">
+      <c r="S62">
         <f>P62-Q62</f>
         <v/>
       </c>
-      <c r="S62">
+      <c r="T62">
         <f>M62*3+N62</f>
         <v/>
       </c>
-      <c r="T62">
+      <c r="U62">
         <f>S62*100000000 + (R62+100)*100000 + P62*1000 + IFERROR(VLOOKUP(K62, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11449,49 +11534,49 @@
           <t>Lunes, 15 de junio 2026 - 16:00</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>Jordania</t>
         </is>
       </c>
-      <c r="L63">
+      <c r="M63">
         <f>IF(ISNUMBER(F79),1,0)+IF(ISNUMBER(F81),1,0)+IF(ISNUMBER(D82),1,0)</f>
         <v/>
       </c>
-      <c r="M63">
+      <c r="N63">
         <f>IF(AND(ISNUMBER(F79),ISNUMBER(D79),F79&gt;D79),1,0)+IF(AND(ISNUMBER(F81),ISNUMBER(D81),F81&gt;D81),1,0)+IF(AND(ISNUMBER(D82),ISNUMBER(F82),D82&gt;F82),1,0)</f>
         <v/>
       </c>
-      <c r="N63">
+      <c r="O63">
         <f>IF(AND(ISNUMBER(F79),ISNUMBER(D79),F79=D79),1,0)+IF(AND(ISNUMBER(F81),ISNUMBER(D81),F81=D81),1,0)+IF(AND(ISNUMBER(D82),ISNUMBER(F82),D82=F82),1,0)</f>
         <v/>
       </c>
-      <c r="O63">
+      <c r="P63">
         <f>IF(AND(ISNUMBER(F79),ISNUMBER(D79),F79&lt;D79),1,0)+IF(AND(ISNUMBER(F81),ISNUMBER(D81),F81&lt;D81),1,0)+IF(AND(ISNUMBER(D82),ISNUMBER(F82),D82&lt;F82),1,0)</f>
         <v/>
       </c>
-      <c r="P63">
+      <c r="Q63">
         <f>IF(ISNUMBER(F79),F79,0)+IF(ISNUMBER(F81),F81,0)+IF(ISNUMBER(D82),D82,0)</f>
         <v/>
       </c>
-      <c r="Q63">
+      <c r="R63">
         <f>IF(ISNUMBER(D79),D79,0)+IF(ISNUMBER(D81),D81,0)+IF(ISNUMBER(F82),F82,0)</f>
         <v/>
       </c>
-      <c r="R63">
+      <c r="S63">
         <f>P63-Q63</f>
         <v/>
       </c>
-      <c r="S63">
+      <c r="T63">
         <f>M63*3+N63</f>
         <v/>
       </c>
-      <c r="T63">
+      <c r="U63">
         <f>S63*100000000 + (R63+100)*100000 + P63*1000 + IFERROR(VLOOKUP(K63, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11524,7 +11609,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="18.75" customHeight="1" s="29">
+    <row r="65" ht="18.75" customHeight="1" s="30">
       <c r="C65" s="4" t="inlineStr">
         <is>
           <t>Cabo Verde</t>
@@ -11551,7 +11636,7 @@
           <t>Domingo, 21 de junio 2026 - 16:00</t>
         </is>
       </c>
-      <c r="J65" s="30" t="inlineStr">
+      <c r="K65" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO K</t>
         </is>
@@ -11584,49 +11669,49 @@
           <t>Viernes, 26 de junio 2026 - 18:00</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="K66" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr">
+      <c r="L66" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="L66">
+      <c r="M66">
         <f>IF(ISNUMBER(D86),1,0)+IF(ISNUMBER(D88),1,0)+IF(ISNUMBER(F90),1,0)</f>
         <v/>
       </c>
-      <c r="M66">
+      <c r="N66">
         <f>IF(AND(ISNUMBER(D86),ISNUMBER(F86),D86&gt;F86),1,0)+IF(AND(ISNUMBER(D88),ISNUMBER(F88),D88&gt;F88),1,0)+IF(AND(ISNUMBER(F90),ISNUMBER(D90),F90&gt;D90),1,0)</f>
         <v/>
       </c>
-      <c r="N66">
+      <c r="O66">
         <f>IF(AND(ISNUMBER(D86),ISNUMBER(F86),D86=F86),1,0)+IF(AND(ISNUMBER(D88),ISNUMBER(F88),D88=F88),1,0)+IF(AND(ISNUMBER(F90),ISNUMBER(D90),F90=D90),1,0)</f>
         <v/>
       </c>
-      <c r="O66">
+      <c r="P66">
         <f>IF(AND(ISNUMBER(D86),ISNUMBER(F86),D86&lt;F86),1,0)+IF(AND(ISNUMBER(D88),ISNUMBER(F88),D88&lt;F88),1,0)+IF(AND(ISNUMBER(F90),ISNUMBER(D90),F90&lt;D90),1,0)</f>
         <v/>
       </c>
-      <c r="P66">
+      <c r="Q66">
         <f>IF(ISNUMBER(D86),D86,0)+IF(ISNUMBER(D88),D88,0)+IF(ISNUMBER(F90),F90,0)</f>
         <v/>
       </c>
-      <c r="Q66">
+      <c r="R66">
         <f>IF(ISNUMBER(F86),F86,0)+IF(ISNUMBER(F88),F88,0)+IF(ISNUMBER(D90),D90,0)</f>
         <v/>
       </c>
-      <c r="R66">
+      <c r="S66">
         <f>P66-Q66</f>
         <v/>
       </c>
-      <c r="S66">
+      <c r="T66">
         <f>M66*3+N66</f>
         <v/>
       </c>
-      <c r="T66">
+      <c r="U66">
         <f>S66*100000000 + (R66+100)*100000 + P66*1000 + IFERROR(VLOOKUP(K66, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11658,151 +11743,151 @@
           <t>Viernes, 26 de junio 2026 - 18:00</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="K67" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
+      <c r="L67" t="inlineStr">
         <is>
           <t>RD Congo</t>
         </is>
       </c>
-      <c r="L67">
+      <c r="M67">
         <f>IF(ISNUMBER(F86),1,0)+IF(ISNUMBER(D89),1,0)+IF(ISNUMBER(D91),1,0)</f>
         <v/>
       </c>
-      <c r="M67">
+      <c r="N67">
         <f>IF(AND(ISNUMBER(F86),ISNUMBER(D86),F86&gt;D86),1,0)+IF(AND(ISNUMBER(D89),ISNUMBER(F89),D89&gt;F89),1,0)+IF(AND(ISNUMBER(D91),ISNUMBER(F91),D91&gt;F91),1,0)</f>
         <v/>
       </c>
-      <c r="N67">
+      <c r="O67">
         <f>IF(AND(ISNUMBER(F86),ISNUMBER(D86),F86=D86),1,0)+IF(AND(ISNUMBER(D89),ISNUMBER(F89),D89=F89),1,0)+IF(AND(ISNUMBER(D91),ISNUMBER(F91),D91=F91),1,0)</f>
         <v/>
       </c>
-      <c r="O67">
+      <c r="P67">
         <f>IF(AND(ISNUMBER(F86),ISNUMBER(D86),F86&lt;D86),1,0)+IF(AND(ISNUMBER(D89),ISNUMBER(F89),D89&lt;F89),1,0)+IF(AND(ISNUMBER(D91),ISNUMBER(F91),D91&lt;F91),1,0)</f>
         <v/>
       </c>
-      <c r="P67">
+      <c r="Q67">
         <f>IF(ISNUMBER(F86),F86,0)+IF(ISNUMBER(D89),D89,0)+IF(ISNUMBER(D91),D91,0)</f>
         <v/>
       </c>
-      <c r="Q67">
+      <c r="R67">
         <f>IF(ISNUMBER(D86),D86,0)+IF(ISNUMBER(F89),F89,0)+IF(ISNUMBER(F91),F91,0)</f>
         <v/>
       </c>
-      <c r="R67">
+      <c r="S67">
         <f>P67-Q67</f>
         <v/>
       </c>
-      <c r="S67">
+      <c r="T67">
         <f>M67*3+N67</f>
         <v/>
       </c>
-      <c r="T67">
+      <c r="U67">
         <f>S67*100000000 + (R67+100)*100000 + P67*1000 + IFERROR(VLOOKUP(K67, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="J68" t="inlineStr">
+      <c r="K68" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr">
+      <c r="L68" t="inlineStr">
         <is>
           <t>Uzbekistán</t>
         </is>
       </c>
-      <c r="L68">
+      <c r="M68">
         <f>IF(ISNUMBER(D87),1,0)+IF(ISNUMBER(F88),1,0)+IF(ISNUMBER(F91),1,0)</f>
         <v/>
       </c>
-      <c r="M68">
+      <c r="N68">
         <f>IF(AND(ISNUMBER(D87),ISNUMBER(F87),D87&gt;F87),1,0)+IF(AND(ISNUMBER(F88),ISNUMBER(D88),F88&gt;D88),1,0)+IF(AND(ISNUMBER(F91),ISNUMBER(D91),F91&gt;D91),1,0)</f>
         <v/>
       </c>
-      <c r="N68">
+      <c r="O68">
         <f>IF(AND(ISNUMBER(D87),ISNUMBER(F87),D87=F87),1,0)+IF(AND(ISNUMBER(F88),ISNUMBER(D88),F88=D88),1,0)+IF(AND(ISNUMBER(F91),ISNUMBER(D91),F91=D91),1,0)</f>
         <v/>
       </c>
-      <c r="O68">
+      <c r="P68">
         <f>IF(AND(ISNUMBER(D87),ISNUMBER(F87),D87&lt;F87),1,0)+IF(AND(ISNUMBER(F88),ISNUMBER(D88),F88&lt;D88),1,0)+IF(AND(ISNUMBER(F91),ISNUMBER(D91),F91&lt;D91),1,0)</f>
         <v/>
       </c>
-      <c r="P68">
+      <c r="Q68">
         <f>IF(ISNUMBER(D87),D87,0)+IF(ISNUMBER(F88),F88,0)+IF(ISNUMBER(F91),F91,0)</f>
         <v/>
       </c>
-      <c r="Q68">
+      <c r="R68">
         <f>IF(ISNUMBER(F87),F87,0)+IF(ISNUMBER(D88),D88,0)+IF(ISNUMBER(D91),D91,0)</f>
         <v/>
       </c>
-      <c r="R68">
+      <c r="S68">
         <f>P68-Q68</f>
         <v/>
       </c>
-      <c r="S68">
+      <c r="T68">
         <f>M68*3+N68</f>
         <v/>
       </c>
-      <c r="T68">
+      <c r="U68">
         <f>S68*100000000 + (R68+100)*100000 + P68*1000 + IFERROR(VLOOKUP(K68, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="69" ht="18.75" customHeight="1" s="29">
-      <c r="A69" s="30" t="inlineStr">
+    <row r="69" ht="18.75" customHeight="1" s="30">
+      <c r="A69" s="29" t="inlineStr">
         <is>
           <t>GRUPO I</t>
         </is>
       </c>
-      <c r="I69" s="35" t="n"/>
-      <c r="J69" t="inlineStr">
+      <c r="I69" s="28" t="n"/>
+      <c r="K69" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="L69" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="L69">
+      <c r="M69">
         <f>IF(ISNUMBER(F87),1,0)+IF(ISNUMBER(F89),1,0)+IF(ISNUMBER(D90),1,0)</f>
         <v/>
       </c>
-      <c r="M69">
+      <c r="N69">
         <f>IF(AND(ISNUMBER(F87),ISNUMBER(D87),F87&gt;D87),1,0)+IF(AND(ISNUMBER(F89),ISNUMBER(D89),F89&gt;D89),1,0)+IF(AND(ISNUMBER(D90),ISNUMBER(F90),D90&gt;F90),1,0)</f>
         <v/>
       </c>
-      <c r="N69">
+      <c r="O69">
         <f>IF(AND(ISNUMBER(F87),ISNUMBER(D87),F87=D87),1,0)+IF(AND(ISNUMBER(F89),ISNUMBER(D89),F89=D89),1,0)+IF(AND(ISNUMBER(D90),ISNUMBER(F90),D90=F90),1,0)</f>
         <v/>
       </c>
-      <c r="O69">
+      <c r="P69">
         <f>IF(AND(ISNUMBER(F87),ISNUMBER(D87),F87&lt;D87),1,0)+IF(AND(ISNUMBER(F89),ISNUMBER(D89),F89&lt;D89),1,0)+IF(AND(ISNUMBER(D90),ISNUMBER(F90),D90&lt;F90),1,0)</f>
         <v/>
       </c>
-      <c r="P69">
+      <c r="Q69">
         <f>IF(ISNUMBER(F87),F87,0)+IF(ISNUMBER(F89),F89,0)+IF(ISNUMBER(D90),D90,0)</f>
         <v/>
       </c>
-      <c r="Q69">
+      <c r="R69">
         <f>IF(ISNUMBER(D87),D87,0)+IF(ISNUMBER(D89),D89,0)+IF(ISNUMBER(F90),F90,0)</f>
         <v/>
       </c>
-      <c r="R69">
+      <c r="S69">
         <f>P69-Q69</f>
         <v/>
       </c>
-      <c r="S69">
+      <c r="T69">
         <f>M69*3+N69</f>
         <v/>
       </c>
-      <c r="T69">
+      <c r="U69">
         <f>S69*100000000 + (R69+100)*100000 + P69*1000 + IFERROR(VLOOKUP(K69, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11835,7 +11920,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="18.75" customHeight="1" s="29">
+    <row r="71" ht="18.75" customHeight="1" s="30">
       <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Irak</t>
@@ -11862,7 +11947,7 @@
           <t>Martes, 16 de junio 2026 - 16:00</t>
         </is>
       </c>
-      <c r="J71" s="30" t="inlineStr">
+      <c r="K71" s="29" t="inlineStr">
         <is>
           <t>CLASIFICACIÓN GRUPO L</t>
         </is>
@@ -11895,49 +11980,49 @@
           <t>Lunes, 22 de junio 2026 - 15:00</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="K72" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
+      <c r="L72" t="inlineStr">
         <is>
           <t>Inglaterra</t>
         </is>
       </c>
-      <c r="L72">
+      <c r="M72">
         <f>IF(ISNUMBER(D94),1,0)+IF(ISNUMBER(D96),1,0)+IF(ISNUMBER(F98),1,0)</f>
         <v/>
       </c>
-      <c r="M72">
+      <c r="N72">
         <f>IF(AND(ISNUMBER(D94),ISNUMBER(F94),D94&gt;F94),1,0)+IF(AND(ISNUMBER(D96),ISNUMBER(F96),D96&gt;F96),1,0)+IF(AND(ISNUMBER(F98),ISNUMBER(D98),F98&gt;D98),1,0)</f>
         <v/>
       </c>
-      <c r="N72">
+      <c r="O72">
         <f>IF(AND(ISNUMBER(D94),ISNUMBER(F94),D94=F94),1,0)+IF(AND(ISNUMBER(D96),ISNUMBER(F96),D96=F96),1,0)+IF(AND(ISNUMBER(F98),ISNUMBER(D98),F98=D98),1,0)</f>
         <v/>
       </c>
-      <c r="O72">
+      <c r="P72">
         <f>IF(AND(ISNUMBER(D94),ISNUMBER(F94),D94&lt;F94),1,0)+IF(AND(ISNUMBER(D96),ISNUMBER(F96),D96&lt;F96),1,0)+IF(AND(ISNUMBER(F98),ISNUMBER(D98),F98&lt;D98),1,0)</f>
         <v/>
       </c>
-      <c r="P72">
+      <c r="Q72">
         <f>IF(ISNUMBER(D94),D94,0)+IF(ISNUMBER(D96),D96,0)+IF(ISNUMBER(F98),F98,0)</f>
         <v/>
       </c>
-      <c r="Q72">
+      <c r="R72">
         <f>IF(ISNUMBER(F94),F94,0)+IF(ISNUMBER(F96),F96,0)+IF(ISNUMBER(D98),D98,0)</f>
         <v/>
       </c>
-      <c r="R72">
+      <c r="S72">
         <f>P72-Q72</f>
         <v/>
       </c>
-      <c r="S72">
+      <c r="T72">
         <f>M72*3+N72</f>
         <v/>
       </c>
-      <c r="T72">
+      <c r="U72">
         <f>S72*100000000 + (R72+100)*100000 + P72*1000 + IFERROR(VLOOKUP(K72, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -11969,49 +12054,49 @@
           <t>Lunes, 22 de junio 2026 - 18:00</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="K73" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="L73" t="inlineStr">
         <is>
           <t>Croacia</t>
         </is>
       </c>
-      <c r="L73">
+      <c r="M73">
         <f>IF(ISNUMBER(F94),1,0)+IF(ISNUMBER(D97),1,0)+IF(ISNUMBER(D99),1,0)</f>
         <v/>
       </c>
-      <c r="M73">
+      <c r="N73">
         <f>IF(AND(ISNUMBER(F94),ISNUMBER(D94),F94&gt;D94),1,0)+IF(AND(ISNUMBER(D97),ISNUMBER(F97),D97&gt;F97),1,0)+IF(AND(ISNUMBER(D99),ISNUMBER(F99),D99&gt;F99),1,0)</f>
         <v/>
       </c>
-      <c r="N73">
+      <c r="O73">
         <f>IF(AND(ISNUMBER(F94),ISNUMBER(D94),F94=D94),1,0)+IF(AND(ISNUMBER(D97),ISNUMBER(F97),D97=F97),1,0)+IF(AND(ISNUMBER(D99),ISNUMBER(F99),D99=F99),1,0)</f>
         <v/>
       </c>
-      <c r="O73">
+      <c r="P73">
         <f>IF(AND(ISNUMBER(F94),ISNUMBER(D94),F94&lt;D94),1,0)+IF(AND(ISNUMBER(D97),ISNUMBER(F97),D97&lt;F97),1,0)+IF(AND(ISNUMBER(D99),ISNUMBER(F99),D99&lt;F99),1,0)</f>
         <v/>
       </c>
-      <c r="P73">
+      <c r="Q73">
         <f>IF(ISNUMBER(F94),F94,0)+IF(ISNUMBER(D97),D97,0)+IF(ISNUMBER(D99),D99,0)</f>
         <v/>
       </c>
-      <c r="Q73">
+      <c r="R73">
         <f>IF(ISNUMBER(D94),D94,0)+IF(ISNUMBER(F97),F97,0)+IF(ISNUMBER(F99),F99,0)</f>
         <v/>
       </c>
-      <c r="R73">
+      <c r="S73">
         <f>P73-Q73</f>
         <v/>
       </c>
-      <c r="S73">
+      <c r="T73">
         <f>M73*3+N73</f>
         <v/>
       </c>
-      <c r="T73">
+      <c r="U73">
         <f>S73*100000000 + (R73+100)*100000 + P73*1000 + IFERROR(VLOOKUP(K73, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -12043,49 +12128,49 @@
           <t>Viernes, 26 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="K74" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr">
+      <c r="L74" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="L74">
+      <c r="M74">
         <f>IF(ISNUMBER(D95),1,0)+IF(ISNUMBER(F96),1,0)+IF(ISNUMBER(F99),1,0)</f>
         <v/>
       </c>
-      <c r="M74">
+      <c r="N74">
         <f>IF(AND(ISNUMBER(D95),ISNUMBER(F95),D95&gt;F95),1,0)+IF(AND(ISNUMBER(F96),ISNUMBER(D96),F96&gt;D96),1,0)+IF(AND(ISNUMBER(F99),ISNUMBER(D99),F99&gt;D99),1,0)</f>
         <v/>
       </c>
-      <c r="N74">
+      <c r="O74">
         <f>IF(AND(ISNUMBER(D95),ISNUMBER(F95),D95=F95),1,0)+IF(AND(ISNUMBER(F96),ISNUMBER(D96),F96=D96),1,0)+IF(AND(ISNUMBER(F99),ISNUMBER(D99),F99=D99),1,0)</f>
         <v/>
       </c>
-      <c r="O74">
+      <c r="P74">
         <f>IF(AND(ISNUMBER(D95),ISNUMBER(F95),D95&lt;F95),1,0)+IF(AND(ISNUMBER(F96),ISNUMBER(D96),F96&lt;D96),1,0)+IF(AND(ISNUMBER(F99),ISNUMBER(D99),F99&lt;D99),1,0)</f>
         <v/>
       </c>
-      <c r="P74">
+      <c r="Q74">
         <f>IF(ISNUMBER(D95),D95,0)+IF(ISNUMBER(F96),F96,0)+IF(ISNUMBER(F99),F99,0)</f>
         <v/>
       </c>
-      <c r="Q74">
+      <c r="R74">
         <f>IF(ISNUMBER(F95),F95,0)+IF(ISNUMBER(D96),D96,0)+IF(ISNUMBER(D99),D99,0)</f>
         <v/>
       </c>
-      <c r="R74">
+      <c r="S74">
         <f>P74-Q74</f>
         <v/>
       </c>
-      <c r="S74">
+      <c r="T74">
         <f>M74*3+N74</f>
         <v/>
       </c>
-      <c r="T74">
+      <c r="U74">
         <f>S74*100000000 + (R74+100)*100000 + P74*1000 + IFERROR(VLOOKUP(K74, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
@@ -12117,60 +12202,61 @@
           <t>Viernes, 26 de junio 2026 - 13:00</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="K75" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr">
+      <c r="L75" t="inlineStr">
         <is>
           <t>Panamá</t>
         </is>
       </c>
-      <c r="L75">
+      <c r="M75">
         <f>IF(ISNUMBER(F95),1,0)+IF(ISNUMBER(F97),1,0)+IF(ISNUMBER(D98),1,0)</f>
         <v/>
       </c>
-      <c r="M75">
+      <c r="N75">
         <f>IF(AND(ISNUMBER(F95),ISNUMBER(D95),F95&gt;D95),1,0)+IF(AND(ISNUMBER(F97),ISNUMBER(D97),F97&gt;D97),1,0)+IF(AND(ISNUMBER(D98),ISNUMBER(F98),D98&gt;F98),1,0)</f>
         <v/>
       </c>
-      <c r="N75">
+      <c r="O75">
         <f>IF(AND(ISNUMBER(F95),ISNUMBER(D95),F95=D95),1,0)+IF(AND(ISNUMBER(F97),ISNUMBER(D97),F97=D97),1,0)+IF(AND(ISNUMBER(D98),ISNUMBER(F98),D98=F98),1,0)</f>
         <v/>
       </c>
-      <c r="O75">
+      <c r="P75">
         <f>IF(AND(ISNUMBER(F95),ISNUMBER(D95),F95&lt;D95),1,0)+IF(AND(ISNUMBER(F97),ISNUMBER(D97),F97&lt;D97),1,0)+IF(AND(ISNUMBER(D98),ISNUMBER(F98),D98&lt;F98),1,0)</f>
         <v/>
       </c>
-      <c r="P75">
+      <c r="Q75">
         <f>IF(ISNUMBER(F95),F95,0)+IF(ISNUMBER(F97),F97,0)+IF(ISNUMBER(D98),D98,0)</f>
         <v/>
       </c>
-      <c r="Q75">
+      <c r="R75">
         <f>IF(ISNUMBER(D95),D95,0)+IF(ISNUMBER(D97),D97,0)+IF(ISNUMBER(F98),F98,0)</f>
         <v/>
       </c>
-      <c r="R75">
+      <c r="S75">
         <f>P75-Q75</f>
         <v/>
       </c>
-      <c r="S75">
+      <c r="T75">
         <f>M75*3+N75</f>
         <v/>
       </c>
-      <c r="T75">
+      <c r="U75">
         <f>S75*100000000 + (R75+100)*100000 + P75*1000 + IFERROR(VLOOKUP(K75, RankingFIFA!$A$1:$B$48, 2, FALSE), 0)</f>
         <v/>
       </c>
     </row>
-    <row r="77" ht="18.75" customHeight="1" s="29">
-      <c r="A77" s="30" t="inlineStr">
+    <row r="76"/>
+    <row r="77" ht="18.75" customHeight="1" s="30">
+      <c r="A77" s="29" t="inlineStr">
         <is>
           <t>GRUPO J</t>
         </is>
       </c>
-      <c r="I77" s="35" t="n"/>
+      <c r="I77" s="28" t="n"/>
     </row>
     <row r="78">
       <c r="C78" s="4" t="inlineStr">
@@ -12340,13 +12426,14 @@
         </is>
       </c>
     </row>
-    <row r="85" ht="18.75" customHeight="1" s="29">
-      <c r="A85" s="30" t="inlineStr">
+    <row r="84"/>
+    <row r="85" ht="18.75" customHeight="1" s="30">
+      <c r="A85" s="29" t="inlineStr">
         <is>
           <t>GRUPO K</t>
         </is>
       </c>
-      <c r="I85" s="35" t="n"/>
+      <c r="I85" s="28" t="n"/>
     </row>
     <row r="86">
       <c r="C86" s="4" t="inlineStr">
@@ -12516,13 +12603,14 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="18.75" customHeight="1" s="29">
-      <c r="A93" s="30" t="inlineStr">
+    <row r="92"/>
+    <row r="93" ht="18.75" customHeight="1" s="30">
+      <c r="A93" s="29" t="inlineStr">
         <is>
           <t>GRUPO L</t>
         </is>
       </c>
-      <c r="I93" s="35" t="n"/>
+      <c r="I93" s="28" t="n"/>
     </row>
     <row r="94">
       <c r="C94" s="4" t="inlineStr">
@@ -12694,8 +12782,8 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="J17:T17"/>
     <mergeCell ref="J23:T23"/>
-    <mergeCell ref="J17:T17"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="J29:T29"/>
     <mergeCell ref="J5:T5"/>
@@ -12734,22 +12822,22 @@
   <dimension ref="B2:G17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" style="29" min="1" max="1"/>
-    <col width="12" customWidth="1" style="29" min="2" max="3"/>
-    <col width="25" customWidth="1" style="29" min="4" max="4"/>
-    <col width="10" customWidth="1" style="29" min="5" max="6"/>
-    <col width="25" customWidth="1" style="29" min="7" max="7"/>
+    <col width="3" customWidth="1" style="30" min="1" max="1"/>
+    <col width="12" customWidth="1" style="30" min="2" max="3"/>
+    <col width="25" customWidth="1" style="30" min="4" max="4"/>
+    <col width="10" customWidth="1" style="30" min="5" max="6"/>
+    <col width="25" customWidth="1" style="30" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="32" t="inlineStr">
+      <c r="B2" s="33" t="inlineStr">
         <is>
           <t>RANKING DE MEJORES TERCEROS LUGARES</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="5" ht="16.5" customHeight="1" s="29">
+    <row r="5" ht="16.5" customHeight="1" s="30">
       <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Posición</t>
@@ -12781,7 +12869,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="29">
+    <row r="6" ht="16.5" customHeight="1" s="30">
       <c r="B6" s="20" t="n">
         <v>1</v>
       </c>
@@ -12806,7 +12894,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="29">
+    <row r="7" ht="16.5" customHeight="1" s="30">
       <c r="B7" s="23" t="n">
         <v>2</v>
       </c>
@@ -12831,7 +12919,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="29">
+    <row r="8" ht="16.5" customHeight="1" s="30">
       <c r="B8" s="20" t="n">
         <v>3</v>
       </c>
@@ -12856,7 +12944,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="29">
+    <row r="9" ht="16.5" customHeight="1" s="30">
       <c r="B9" s="23" t="n">
         <v>4</v>
       </c>
@@ -12881,7 +12969,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="29">
+    <row r="10" ht="16.5" customHeight="1" s="30">
       <c r="B10" s="20" t="n">
         <v>5</v>
       </c>
@@ -12906,7 +12994,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="29">
+    <row r="11" ht="16.5" customHeight="1" s="30">
       <c r="B11" s="23" t="n">
         <v>6</v>
       </c>
@@ -12931,7 +13019,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="29">
+    <row r="12" ht="16.5" customHeight="1" s="30">
       <c r="B12" s="20" t="n">
         <v>7</v>
       </c>
@@ -12956,7 +13044,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="29">
+    <row r="13" ht="16.5" customHeight="1" s="30">
       <c r="B13" s="23" t="n">
         <v>8</v>
       </c>
@@ -12981,7 +13069,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="29">
+    <row r="14" ht="16.5" customHeight="1" s="30">
       <c r="B14" s="20" t="n">
         <v>9</v>
       </c>
@@ -13006,7 +13094,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="29">
+    <row r="15" ht="16.5" customHeight="1" s="30">
       <c r="B15" s="23" t="n">
         <v>10</v>
       </c>
@@ -13031,7 +13119,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="29">
+    <row r="16" ht="16.5" customHeight="1" s="30">
       <c r="B16" s="20" t="n">
         <v>11</v>
       </c>
@@ -13056,7 +13144,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="29">
+    <row r="17" ht="16.5" customHeight="1" s="30">
       <c r="B17" s="23" t="n">
         <v>12</v>
       </c>
@@ -13635,12 +13723,12 @@
   <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="29" min="2" max="2"/>
-    <col width="6" customWidth="1" style="29" min="3" max="4"/>
-    <col width="3" customWidth="1" style="29" min="5" max="5"/>
-    <col width="6" customWidth="1" style="29" min="6" max="7"/>
-    <col width="18" customWidth="1" style="29" min="8" max="9"/>
-    <col width="45" customWidth="1" style="29" min="10" max="10"/>
+    <col width="20" customWidth="1" style="30" min="2" max="2"/>
+    <col width="6" customWidth="1" style="30" min="3" max="4"/>
+    <col width="3" customWidth="1" style="30" min="5" max="5"/>
+    <col width="6" customWidth="1" style="30" min="6" max="7"/>
+    <col width="18" customWidth="1" style="30" min="8" max="9"/>
+    <col width="56.5703125" customWidth="1" style="30" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13651,64 +13739,62 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3">
-      <c r="J3" t="inlineStr">
+    <row r="4" ht="18.75" customHeight="1" s="30">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>DIECISEISAVOS DE FINAL (Ronda de 32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="30">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Partido</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Equipo A</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Goles</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Pen.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Pen.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Goles</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Equipo B</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Clasifica</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Fecha y Estadio</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18.75" customHeight="1" s="29">
-      <c r="A4" s="30" t="inlineStr">
-        <is>
-          <t>DIECISEISAVOS DE FINAL (Ronda de 32)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16.5" customHeight="1" s="29">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Partido</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Equipo A</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Goles</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Pen.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>vs</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Pen.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Goles</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Equipo B</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Clasifica</t>
         </is>
       </c>
     </row>
@@ -14240,12 +14326,13 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="18.75" customHeight="1" s="29">
-      <c r="A23" s="30" t="inlineStr">
+    <row r="23" ht="18.75" customHeight="1" s="30">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>OCTAVOS DE FINAL</t>
         </is>
       </c>
+      <c r="J23" s="28" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -14529,14 +14616,15 @@
       <c r="H34" s="8" t="n"/>
       <c r="I34" s="8" t="n"/>
     </row>
-    <row r="35" ht="18.75" customHeight="1" s="29">
-      <c r="A35" s="33" t="inlineStr">
+    <row r="35" ht="18.75" customHeight="1" s="30">
+      <c r="A35" s="34" t="inlineStr">
         <is>
           <t>CUARTOS DE FINAL</t>
         </is>
       </c>
-    </row>
-    <row r="36" ht="16.5" customHeight="1" s="29">
+      <c r="J35" s="28" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="30">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -14570,6 +14658,11 @@
       <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Fecha y Estadio</t>
         </is>
       </c>
     </row>
@@ -14723,14 +14816,15 @@
       <c r="H42" s="8" t="n"/>
       <c r="I42" s="8" t="n"/>
     </row>
-    <row r="43" ht="18.75" customHeight="1" s="29">
-      <c r="A43" s="33" t="inlineStr">
+    <row r="43" ht="18.75" customHeight="1" s="30">
+      <c r="A43" s="34" t="inlineStr">
         <is>
           <t>SEMIFINALES</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="16.5" customHeight="1" s="29">
+      <c r="J43" s="28" t="n"/>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="30">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -14764,6 +14858,11 @@
       <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Fecha y Estadio</t>
         </is>
       </c>
     </row>
@@ -14851,14 +14950,15 @@
       <c r="H48" s="8" t="n"/>
       <c r="I48" s="8" t="n"/>
     </row>
-    <row r="49" ht="18.75" customHeight="1" s="29">
-      <c r="A49" s="33" t="inlineStr">
+    <row r="49" ht="18.75" customHeight="1" s="30">
+      <c r="A49" s="34" t="inlineStr">
         <is>
           <t>PARTIDO POR EL TERCER LUGAR</t>
         </is>
       </c>
-    </row>
-    <row r="50" ht="16.5" customHeight="1" s="29">
+      <c r="J49" s="28" t="n"/>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="30">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -14892,6 +14992,11 @@
       <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Fecha y Estadio</t>
         </is>
       </c>
     </row>
@@ -14946,14 +15051,14 @@
       <c r="H53" s="8" t="n"/>
       <c r="I53" s="8" t="n"/>
     </row>
-    <row r="54" ht="18.75" customHeight="1" s="29">
-      <c r="A54" s="33" t="inlineStr">
+    <row r="54" ht="18.75" customHeight="1" s="30">
+      <c r="A54" s="34" t="inlineStr">
         <is>
           <t>GRAN FINAL</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="29">
+    <row r="55" ht="16.5" customHeight="1" s="30">
       <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Partido</t>
@@ -14987,6 +15092,11 @@
       <c r="I55" s="2" t="inlineStr">
         <is>
           <t>Clasifica</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Fecha y Estadio</t>
         </is>
       </c>
     </row>
@@ -15041,16 +15151,16 @@
       <c r="H58" s="8" t="n"/>
       <c r="I58" s="8" t="n"/>
     </row>
-    <row r="59" ht="18.75" customHeight="1" s="29">
-      <c r="A59" s="33" t="inlineStr">
+    <row r="59" ht="18.75" customHeight="1" s="30">
+      <c r="A59" s="34" t="inlineStr">
         <is>
           <t>PODIO DE HONOR 🏆</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="29">
+    <row r="60" ht="16.5" customHeight="1" s="30">
       <c r="A60" s="8" t="n"/>
-      <c r="B60" s="34" t="inlineStr">
+      <c r="B60" s="35" t="inlineStr">
         <is>
           <t>CAMPEÓN MUNDIAL 🏆</t>
         </is>
@@ -15061,9 +15171,9 @@
       </c>
       <c r="I60" s="8" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="29">
+    <row r="61" ht="16.5" customHeight="1" s="30">
       <c r="A61" s="8" t="n"/>
-      <c r="B61" s="34" t="inlineStr">
+      <c r="B61" s="35" t="inlineStr">
         <is>
           <t>Subcampeón 🥈</t>
         </is>
@@ -15074,9 +15184,9 @@
       </c>
       <c r="I61" s="8" t="n"/>
     </row>
-    <row r="62" ht="16.5" customHeight="1" s="29">
+    <row r="62" ht="16.5" customHeight="1" s="30">
       <c r="A62" s="8" t="n"/>
-      <c r="B62" s="34" t="inlineStr">
+      <c r="B62" s="35" t="inlineStr">
         <is>
           <t>Tercer Lugar 🥉</t>
         </is>
@@ -15090,15 +15200,15 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A59:I59"/>
-    <mergeCell ref="B62:G62"/>
     <mergeCell ref="A43:I43"/>
     <mergeCell ref="A49:I49"/>
     <mergeCell ref="B60:G60"/>
+    <mergeCell ref="A4:I4"/>
     <mergeCell ref="B61:G61"/>
     <mergeCell ref="A23:I23"/>
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="B62:G62"/>
     <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15111,21 +15221,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B183"/>
+  <dimension ref="B2:B183"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="124.28515625" customWidth="1" style="29" min="2" max="2"/>
+    <col width="124.28515625" customWidth="1" style="30" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="26.25" customHeight="1" s="29">
+    <row r="2" ht="26.25" customHeight="1" s="30">
       <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Fase de grupos: calendario y horarios de la Copa Mundial de la FIFA 2026™</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="18" t="inlineStr">
         <is>
@@ -15154,7 +15262,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
@@ -15176,7 +15283,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
@@ -15212,7 +15318,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
@@ -15248,7 +15353,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
@@ -15284,7 +15388,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
@@ -15320,7 +15423,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
@@ -15356,7 +15458,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
@@ -15392,7 +15493,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
@@ -15428,7 +15528,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
@@ -15464,8 +15563,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
@@ -15501,7 +15598,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
@@ -15537,7 +15633,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
@@ -15573,7 +15668,6 @@
         </is>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
@@ -15623,7 +15717,6 @@
         </is>
       </c>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
@@ -15673,7 +15766,6 @@
         </is>
       </c>
     </row>
-    <row r="95"/>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
@@ -15723,7 +15815,6 @@
         </is>
       </c>
     </row>
-    <row r="103"/>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
@@ -15773,7 +15864,6 @@
         </is>
       </c>
     </row>
-    <row r="111"/>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
@@ -15781,7 +15871,6 @@
         </is>
       </c>
     </row>
-    <row r="113"/>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
@@ -15796,7 +15885,6 @@
         </is>
       </c>
     </row>
-    <row r="116"/>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
@@ -15825,7 +15913,6 @@
         </is>
       </c>
     </row>
-    <row r="121"/>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
@@ -15854,7 +15941,6 @@
         </is>
       </c>
     </row>
-    <row r="126"/>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
@@ -15883,7 +15969,6 @@
         </is>
       </c>
     </row>
-    <row r="131"/>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
@@ -15912,7 +15997,6 @@
         </is>
       </c>
     </row>
-    <row r="136"/>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
@@ -15941,7 +16025,6 @@
         </is>
       </c>
     </row>
-    <row r="141"/>
     <row r="142">
       <c r="B142" t="inlineStr">
         <is>
@@ -15970,7 +16053,6 @@
         </is>
       </c>
     </row>
-    <row r="146"/>
     <row r="147">
       <c r="B147" t="inlineStr">
         <is>
@@ -15992,7 +16074,6 @@
         </is>
       </c>
     </row>
-    <row r="150"/>
     <row r="151">
       <c r="B151" t="inlineStr">
         <is>
@@ -16014,7 +16095,6 @@
         </is>
       </c>
     </row>
-    <row r="154"/>
     <row r="155">
       <c r="B155" t="inlineStr">
         <is>
@@ -16036,7 +16116,6 @@
         </is>
       </c>
     </row>
-    <row r="158"/>
     <row r="159">
       <c r="B159" t="inlineStr">
         <is>
@@ -16058,7 +16137,6 @@
         </is>
       </c>
     </row>
-    <row r="162"/>
     <row r="163">
       <c r="B163" t="inlineStr">
         <is>
@@ -16073,7 +16151,6 @@
         </is>
       </c>
     </row>
-    <row r="165"/>
     <row r="166">
       <c r="B166" t="inlineStr">
         <is>
@@ -16095,7 +16172,6 @@
         </is>
       </c>
     </row>
-    <row r="169"/>
     <row r="170">
       <c r="B170" t="inlineStr">
         <is>
@@ -16117,7 +16193,6 @@
         </is>
       </c>
     </row>
-    <row r="173"/>
     <row r="174">
       <c r="B174" t="inlineStr">
         <is>
@@ -16132,7 +16207,6 @@
         </is>
       </c>
     </row>
-    <row r="176"/>
     <row r="177">
       <c r="B177" t="inlineStr">
         <is>
@@ -16154,7 +16228,6 @@
         </is>
       </c>
     </row>
-    <row r="180"/>
     <row r="181">
       <c r="B181" t="inlineStr">
         <is>
@@ -16190,24 +16263,24 @@
   <dimension ref="B2:B8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="146" customWidth="1" style="29" min="2" max="2"/>
+    <col width="146" customWidth="1" style="30" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="2" ht="26.25" customHeight="1" s="29">
+    <row r="2" ht="26.25" customHeight="1" s="30">
       <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Link para descargar archvivo ICS del  Calendario Mundial 2026 para Outlook o iPhone:</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1" s="29">
+    <row r="3" ht="45" customHeight="1" s="30">
       <c r="B3" s="16" t="inlineStr">
         <is>
           <t>https://calendar.google.com/calendar/ical/611d68120c62daa60625df08296c3333f1416dbeb64241045a3c75dd62f175d8%40group.calendar.google.com/public/basic.ics</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="26.25" customHeight="1" s="29">
+    <row r="6" ht="26.25" customHeight="1" s="30">
       <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Calendario para Google Calendar</t>
@@ -16217,7 +16290,7 @@
     <row r="7">
       <c r="B7" s="17" t="n"/>
     </row>
-    <row r="8" ht="60" customHeight="1" s="29">
+    <row r="8" ht="60" customHeight="1" s="30">
       <c r="B8" s="16" t="inlineStr">
         <is>
           <t>https://calendar.google.com/calendar/u/4?cid=NjExZDY4MTIwYzYyZGFhNjA2MjVkZjA4Mjk2YzMzMzNmMTQxNmRiZWI2NDI0MTA0NWEzYzc1ZGQ2MmYxNzVkOEBncm91cC5jYWxlbmRhci5nb29nbGUuY29t</t>

</xml_diff>